<commit_message>
Audit + outreach: 2026-09-06 10:33 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L298"/>
+  <dimension ref="A1:P298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -439,6 +439,10 @@
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,6 +506,26 @@
           <t>Date Found</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Audit PDF</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Audit Status</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Emailed At</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Email Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -557,6 +581,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>audits/audit_thinkclimatecare.com.pdf</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -617,6 +651,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>audits/audit_heat-pump-installation-springdale.tanddhvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -677,6 +721,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>audits/audit_mclaughlin-air.com.pdf</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -732,6 +786,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>audits/audit_mesquiteheatingandair.com.pdf</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -792,6 +856,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>audits/audit_lovesair.com.pdf</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -852,6 +926,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>audits/audit_lexairconditioning.com.pdf</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -907,6 +991,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>audits/audit_dougsheatingandair.com.pdf</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -962,6 +1056,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>audits/audit_airdoctorx.com.pdf</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1017,6 +1121,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>audits/audit_comfortexpertsinc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1072,6 +1186,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>audits/audit_callmessina.com.pdf</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1127,6 +1251,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>audits/audit_elkhornplumbingid.com.pdf</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1187,6 +1321,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>audits/audit_napervilletitanroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -17759,7 +17903,6 @@
           <t>https://russellplumbingsc.com/plumbing-services/emergency-plumber-greenville-sc/</t>
         </is>
       </c>
-      <c r="E296" t="inlineStr"/>
       <c r="F296" t="inlineStr">
         <is>
           <t>info@russellplumbingsc.com</t>
@@ -17875,7 +18018,6 @@
           <t>https://paynesroofingllc.com/residential/</t>
         </is>
       </c>
-      <c r="E298" t="inlineStr"/>
       <c r="F298" t="inlineStr">
         <is>
           <t>paynesroofing1011@outlook.com</t>

</xml_diff>

<commit_message>
Leads: 2026-09-06 21:37 UTC (cycle 131)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1285"/>
+  <dimension ref="A1:L1288"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -75480,7 +75480,6 @@
           <t>https://www.schneiderheatingeriepa.com/</t>
         </is>
       </c>
-      <c r="E1282" t="inlineStr"/>
       <c r="F1282" t="inlineStr">
         <is>
           <t>info@schneiderheatingeriepa.com</t>
@@ -75536,7 +75535,6 @@
           <t>https://www.kindleheatingandcoolingerie.com/</t>
         </is>
       </c>
-      <c r="E1283" t="inlineStr"/>
       <c r="F1283" t="inlineStr">
         <is>
           <t>kindleheating@verizon.net</t>
@@ -75592,7 +75590,6 @@
           <t>https://www.millfairheatingandcooling.com/</t>
         </is>
       </c>
-      <c r="E1284" t="inlineStr"/>
       <c r="F1284" t="inlineStr">
         <is>
           <t>info@millfairheatingandcooling.com</t>
@@ -75682,6 +75679,182 @@
         </is>
       </c>
       <c r="L1285" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>Progressive Air Systems</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>progressiveairsystems.com</t>
+        </is>
+      </c>
+      <c r="D1286" t="inlineStr">
+        <is>
+          <t>https://progressiveairsystems.com/locations/clearwater-fl-heating-and-cooling/</t>
+        </is>
+      </c>
+      <c r="E1286" t="inlineStr"/>
+      <c r="F1286" t="inlineStr">
+        <is>
+          <t>info@progressiveairsystems.com</t>
+        </is>
+      </c>
+      <c r="G1286" t="inlineStr">
+        <is>
+          <t>727-339-1131</t>
+        </is>
+      </c>
+      <c r="H1286" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I1286" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1286" t="inlineStr">
+        <is>
+          <t>heating and cooling company Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K1286" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1286" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>Plumbing Contractor | John Wayne Plumbing &amp; Drain Services</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>johnwayneplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1287" t="inlineStr">
+        <is>
+          <t>https://www.johnwayneplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E1287" t="inlineStr">
+        <is>
+          <t>Residential Plumbing</t>
+        </is>
+      </c>
+      <c r="F1287" t="inlineStr">
+        <is>
+          <t>office@johnwayneplumbing.com</t>
+        </is>
+      </c>
+      <c r="G1287" t="inlineStr">
+        <is>
+          <t>(205) 343-1770</t>
+        </is>
+      </c>
+      <c r="H1287" t="inlineStr">
+        <is>
+          <t>Tuscaloosa AL</t>
+        </is>
+      </c>
+      <c r="I1287" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1287" t="inlineStr">
+        <is>
+          <t>plumbing company Tuscaloosa AL</t>
+        </is>
+      </c>
+      <c r="K1287" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1287" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>Aaron Plumbing</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>chooseaaronplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1288" t="inlineStr">
+        <is>
+          <t>https://chooseaaronplumbing.com/plumbing-services/water-heaters/</t>
+        </is>
+      </c>
+      <c r="E1288" t="inlineStr">
+        <is>
+          <t>Aaron Plumbing</t>
+        </is>
+      </c>
+      <c r="F1288" t="inlineStr">
+        <is>
+          <t>service@chooseaaronservices.com</t>
+        </is>
+      </c>
+      <c r="G1288" t="inlineStr">
+        <is>
+          <t>(770) 239-6628</t>
+        </is>
+      </c>
+      <c r="H1288" t="inlineStr">
+        <is>
+          <t>Roswell GA</t>
+        </is>
+      </c>
+      <c r="I1288" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1288" t="inlineStr">
+        <is>
+          <t>water heater repair Roswell GA</t>
+        </is>
+      </c>
+      <c r="K1288" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1288" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 21:39 UTC (cycle 132)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1288"/>
+  <dimension ref="A1:L1293"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -75705,7 +75705,6 @@
           <t>https://progressiveairsystems.com/locations/clearwater-fl-heating-and-cooling/</t>
         </is>
       </c>
-      <c r="E1286" t="inlineStr"/>
       <c r="F1286" t="inlineStr">
         <is>
           <t>info@progressiveairsystems.com</t>
@@ -75855,6 +75854,306 @@
         </is>
       </c>
       <c r="L1288" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>Hall and Sons Plumbing</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>hallandsonsplbg.com</t>
+        </is>
+      </c>
+      <c r="D1289" t="inlineStr">
+        <is>
+          <t>https://hallandsonsplbg.com/</t>
+        </is>
+      </c>
+      <c r="E1289" t="inlineStr">
+        <is>
+          <t>Gary Hall</t>
+        </is>
+      </c>
+      <c r="F1289" t="inlineStr">
+        <is>
+          <t>info@hallandsonsplbg.com</t>
+        </is>
+      </c>
+      <c r="G1289" t="inlineStr">
+        <is>
+          <t>904-429-9747</t>
+        </is>
+      </c>
+      <c r="H1289" t="inlineStr">
+        <is>
+          <t>Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="I1289" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1289" t="inlineStr">
+        <is>
+          <t>plumbing company Jacksonville FL</t>
+        </is>
+      </c>
+      <c r="K1289" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1289" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>waterheaterrepairpasadena.com</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>waterheaterrepairpasadena.com</t>
+        </is>
+      </c>
+      <c r="D1290" t="inlineStr">
+        <is>
+          <t>https://waterheaterrepairpasadena.com/</t>
+        </is>
+      </c>
+      <c r="E1290" t="inlineStr">
+        <is>
+          <t>No Matter</t>
+        </is>
+      </c>
+      <c r="F1290" t="inlineStr">
+        <is>
+          <t>service@waterheaterrepairpasadena.com</t>
+        </is>
+      </c>
+      <c r="G1290" t="inlineStr">
+        <is>
+          <t>281-803-9846</t>
+        </is>
+      </c>
+      <c r="H1290" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I1290" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1290" t="inlineStr">
+        <is>
+          <t>water heater repair Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K1290" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1290" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>Water Heater Repair Spring TX</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>waterheaterrepairspringtx.com</t>
+        </is>
+      </c>
+      <c r="D1291" t="inlineStr">
+        <is>
+          <t>https://waterheaterrepairspringtx.com/pasadena-tx.html</t>
+        </is>
+      </c>
+      <c r="E1291" t="inlineStr">
+        <is>
+          <t>Water Heater</t>
+        </is>
+      </c>
+      <c r="F1291" t="inlineStr">
+        <is>
+          <t>service@waterheaterrepairspringtx.com</t>
+        </is>
+      </c>
+      <c r="G1291" t="inlineStr">
+        <is>
+          <t>832-685-8164</t>
+        </is>
+      </c>
+      <c r="H1291" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I1291" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1291" t="inlineStr">
+        <is>
+          <t>water heater repair Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K1291" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1291" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>Texas Quality Plumbing</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>texasqualityplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1292" t="inlineStr">
+        <is>
+          <t>https://texasqualityplumbing.com/water-heater/water-heater-repair-service-pasadena-tx</t>
+        </is>
+      </c>
+      <c r="E1292" t="inlineStr">
+        <is>
+          <t>Why This</t>
+        </is>
+      </c>
+      <c r="F1292" t="inlineStr">
+        <is>
+          <t>info@texasqualityplumbing.com</t>
+        </is>
+      </c>
+      <c r="G1292" t="inlineStr">
+        <is>
+          <t>(346) 636-2418</t>
+        </is>
+      </c>
+      <c r="H1292" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I1292" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1292" t="inlineStr">
+        <is>
+          <t>water heater repair Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K1292" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1292" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>JTR Roofing Inc | Twin Cities Roofing, Siding &amp; Home Exteriors</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>jtrroofinginc.com</t>
+        </is>
+      </c>
+      <c r="D1293" t="inlineStr">
+        <is>
+          <t>https://www.jtrroofinginc.com/roof-repair-bloomington/</t>
+        </is>
+      </c>
+      <c r="E1293" t="inlineStr">
+        <is>
+          <t>Twin Cities</t>
+        </is>
+      </c>
+      <c r="F1293" t="inlineStr">
+        <is>
+          <t>dan@jtrroofinginc.com</t>
+        </is>
+      </c>
+      <c r="G1293" t="inlineStr">
+        <is>
+          <t>(651) 777-7394</t>
+        </is>
+      </c>
+      <c r="H1293" t="inlineStr">
+        <is>
+          <t>Bloomington MN</t>
+        </is>
+      </c>
+      <c r="I1293" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1293" t="inlineStr">
+        <is>
+          <t>roof repair company Bloomington MN</t>
+        </is>
+      </c>
+      <c r="K1293" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1293" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 21:40 UTC (cycle 133)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1293"/>
+  <dimension ref="A1:L1300"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -76159,6 +76159,410 @@
         </is>
       </c>
     </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>Rebel Roofing</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>rebelroofingidaho.com</t>
+        </is>
+      </c>
+      <c r="D1294" t="inlineStr">
+        <is>
+          <t>https://rebelroofingidaho.com/metal-roofing-installation-and-replacement/</t>
+        </is>
+      </c>
+      <c r="E1294" t="inlineStr">
+        <is>
+          <t>At Rebel</t>
+        </is>
+      </c>
+      <c r="F1294" t="inlineStr">
+        <is>
+          <t>rebelroofingidaho@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1294" t="inlineStr">
+        <is>
+          <t>(208) 703-9998</t>
+        </is>
+      </c>
+      <c r="H1294" t="inlineStr">
+        <is>
+          <t>Nampa ID</t>
+        </is>
+      </c>
+      <c r="I1294" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1294" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Nampa ID</t>
+        </is>
+      </c>
+      <c r="K1294" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1294" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>TYCO Plumbing</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>tycoplumbingco.com</t>
+        </is>
+      </c>
+      <c r="D1295" t="inlineStr">
+        <is>
+          <t>https://tycoplumbingco.com/water-heater-repair-replacement-westminster-co/</t>
+        </is>
+      </c>
+      <c r="E1295" t="inlineStr"/>
+      <c r="F1295" t="inlineStr">
+        <is>
+          <t>tycoplumbingco@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1295" t="inlineStr">
+        <is>
+          <t>(720) 826-0800</t>
+        </is>
+      </c>
+      <c r="H1295" t="inlineStr">
+        <is>
+          <t>Westminster CO</t>
+        </is>
+      </c>
+      <c r="I1295" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1295" t="inlineStr">
+        <is>
+          <t>water heater repair Westminster CO</t>
+        </is>
+      </c>
+      <c r="K1295" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1295" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>Pulse Home Services</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>pulsehomeco.com</t>
+        </is>
+      </c>
+      <c r="D1296" t="inlineStr">
+        <is>
+          <t>https://www.pulsehomeco.com/plumbing/water-heater-installation-repair-in-westminster-co/</t>
+        </is>
+      </c>
+      <c r="E1296" t="inlineStr"/>
+      <c r="F1296" t="inlineStr">
+        <is>
+          <t>office@pulsehomeco.com</t>
+        </is>
+      </c>
+      <c r="G1296" t="inlineStr">
+        <is>
+          <t>720-464-5280</t>
+        </is>
+      </c>
+      <c r="H1296" t="inlineStr">
+        <is>
+          <t>Westminster CO</t>
+        </is>
+      </c>
+      <c r="I1296" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1296" t="inlineStr">
+        <is>
+          <t>water heater repair Westminster CO</t>
+        </is>
+      </c>
+      <c r="K1296" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1296" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>Big Apple Plumbing LLC</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>bigappleplumbing.net</t>
+        </is>
+      </c>
+      <c r="D1297" t="inlineStr">
+        <is>
+          <t>https://bigappleplumbing.net/plumbing-services/hot-water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E1297" t="inlineStr">
+        <is>
+          <t>Jason Wilkat</t>
+        </is>
+      </c>
+      <c r="F1297" t="inlineStr">
+        <is>
+          <t>teambigappleplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1297" t="inlineStr">
+        <is>
+          <t>(720) 900-1003</t>
+        </is>
+      </c>
+      <c r="H1297" t="inlineStr">
+        <is>
+          <t>Westminster CO</t>
+        </is>
+      </c>
+      <c r="I1297" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1297" t="inlineStr">
+        <is>
+          <t>water heater repair Westminster CO</t>
+        </is>
+      </c>
+      <c r="K1297" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1297" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>Water Heater Repair Westminster CO | Tankless Installation</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>westminsterplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="D1298" t="inlineStr">
+        <is>
+          <t>https://www.westminsterplumbingllc.com/water-heater</t>
+        </is>
+      </c>
+      <c r="E1298" t="inlineStr"/>
+      <c r="F1298" t="inlineStr">
+        <is>
+          <t>westminsterplumbingllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1298" t="inlineStr">
+        <is>
+          <t>(478) 780-3030</t>
+        </is>
+      </c>
+      <c r="H1298" t="inlineStr">
+        <is>
+          <t>Westminster CO</t>
+        </is>
+      </c>
+      <c r="I1298" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1298" t="inlineStr">
+        <is>
+          <t>water heater repair Westminster CO</t>
+        </is>
+      </c>
+      <c r="K1298" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1298" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>Regional Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>regionalheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D1299" t="inlineStr">
+        <is>
+          <t>https://www.regionalheatingandcooling.com/cranston-hvac</t>
+        </is>
+      </c>
+      <c r="E1299" t="inlineStr">
+        <is>
+          <t>Rhode Island</t>
+        </is>
+      </c>
+      <c r="F1299" t="inlineStr">
+        <is>
+          <t>contact@rhcri.com</t>
+        </is>
+      </c>
+      <c r="G1299" t="inlineStr">
+        <is>
+          <t>(401) 416-2597</t>
+        </is>
+      </c>
+      <c r="H1299" t="inlineStr">
+        <is>
+          <t>Cranston RI</t>
+        </is>
+      </c>
+      <c r="I1299" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1299" t="inlineStr">
+        <is>
+          <t>heating and cooling company Cranston RI</t>
+        </is>
+      </c>
+      <c r="K1299" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1299" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>Water Heater Service, Water Heaters &amp; Water Heater Repair</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>precisionplushvac.com</t>
+        </is>
+      </c>
+      <c r="D1300" t="inlineStr">
+        <is>
+          <t>https://www.precisionplushvac.com/water-heaters/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E1300" t="inlineStr"/>
+      <c r="F1300" t="inlineStr">
+        <is>
+          <t>precisionplusllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1300" t="inlineStr">
+        <is>
+          <t>(304) 598-3105</t>
+        </is>
+      </c>
+      <c r="H1300" t="inlineStr">
+        <is>
+          <t>Morgantown WV</t>
+        </is>
+      </c>
+      <c r="I1300" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1300" t="inlineStr">
+        <is>
+          <t>water heater repair Morgantown WV</t>
+        </is>
+      </c>
+      <c r="K1300" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1300" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 21:42 UTC (cycle 134)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1300"/>
+  <dimension ref="A1:L1303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -76240,7 +76240,6 @@
           <t>https://tycoplumbingco.com/water-heater-repair-replacement-westminster-co/</t>
         </is>
       </c>
-      <c r="E1295" t="inlineStr"/>
       <c r="F1295" t="inlineStr">
         <is>
           <t>tycoplumbingco@gmail.com</t>
@@ -76296,7 +76295,6 @@
           <t>https://www.pulsehomeco.com/plumbing/water-heater-installation-repair-in-westminster-co/</t>
         </is>
       </c>
-      <c r="E1296" t="inlineStr"/>
       <c r="F1296" t="inlineStr">
         <is>
           <t>office@pulsehomeco.com</t>
@@ -76412,7 +76410,6 @@
           <t>https://www.westminsterplumbingllc.com/water-heater</t>
         </is>
       </c>
-      <c r="E1298" t="inlineStr"/>
       <c r="F1298" t="inlineStr">
         <is>
           <t>westminsterplumbingllc@gmail.com</t>
@@ -76528,7 +76525,6 @@
           <t>https://www.precisionplushvac.com/water-heaters/water-heater-repair/</t>
         </is>
       </c>
-      <c r="E1300" t="inlineStr"/>
       <c r="F1300" t="inlineStr">
         <is>
           <t>precisionplusllc@gmail.com</t>
@@ -76558,6 +76554,182 @@
         </is>
       </c>
       <c r="L1300" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>Water Heater Pete</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>waterheaterpete.com</t>
+        </is>
+      </c>
+      <c r="D1301" t="inlineStr">
+        <is>
+          <t>https://waterheaterpete.com/water-heater-replace-repair-service-in-chandler-and-gilbert-az/</t>
+        </is>
+      </c>
+      <c r="E1301" t="inlineStr">
+        <is>
+          <t>Greater Phoenix</t>
+        </is>
+      </c>
+      <c r="F1301" t="inlineStr">
+        <is>
+          <t>pete@waterheaterpete.com</t>
+        </is>
+      </c>
+      <c r="G1301" t="inlineStr">
+        <is>
+          <t>(480) 447-7550</t>
+        </is>
+      </c>
+      <c r="H1301" t="inlineStr">
+        <is>
+          <t>Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="I1301" t="n">
+        <v>92</v>
+      </c>
+      <c r="J1301" t="inlineStr">
+        <is>
+          <t>water heater repair Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="K1301" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1301" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>Bucksworth Home Services</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>getyourbucksworth.com</t>
+        </is>
+      </c>
+      <c r="D1302" t="inlineStr">
+        <is>
+          <t>https://www.getyourbucksworth.com/gilbert-az/plumbing-and-water-heaters/water-heater-repair</t>
+        </is>
+      </c>
+      <c r="E1302" t="inlineStr">
+        <is>
+          <t>One Company</t>
+        </is>
+      </c>
+      <c r="F1302" t="inlineStr">
+        <is>
+          <t>info@getyourbucksworth.com</t>
+        </is>
+      </c>
+      <c r="G1302" t="inlineStr">
+        <is>
+          <t>(480) 422-8388</t>
+        </is>
+      </c>
+      <c r="H1302" t="inlineStr">
+        <is>
+          <t>Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="I1302" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1302" t="inlineStr">
+        <is>
+          <t>water heater repair Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="K1302" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1302" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>AC Installation Carmel IN</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>hoosierdaddyhvac.com</t>
+        </is>
+      </c>
+      <c r="D1303" t="inlineStr">
+        <is>
+          <t>https://www.hoosierdaddyhvac.com/ac-installation-carmel-in/</t>
+        </is>
+      </c>
+      <c r="E1303" t="inlineStr"/>
+      <c r="F1303" t="inlineStr">
+        <is>
+          <t>service@hoosierdaddyhvac.com</t>
+        </is>
+      </c>
+      <c r="G1303" t="inlineStr">
+        <is>
+          <t>(765) 894-0047</t>
+        </is>
+      </c>
+      <c r="H1303" t="inlineStr">
+        <is>
+          <t>Carmel IN</t>
+        </is>
+      </c>
+      <c r="I1303" t="n">
+        <v>84</v>
+      </c>
+      <c r="J1303" t="inlineStr">
+        <is>
+          <t>AC installation Carmel IN</t>
+        </is>
+      </c>
+      <c r="K1303" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1303" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 21:43 UTC (cycle 135)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1303"/>
+  <dimension ref="A1:L1305"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -76700,7 +76700,6 @@
           <t>https://www.hoosierdaddyhvac.com/ac-installation-carmel-in/</t>
         </is>
       </c>
-      <c r="E1303" t="inlineStr"/>
       <c r="F1303" t="inlineStr">
         <is>
           <t>service@hoosierdaddyhvac.com</t>
@@ -76730,6 +76729,126 @@
         </is>
       </c>
       <c r="L1303" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>Capital City Roofing</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>capitalcityroofing.net</t>
+        </is>
+      </c>
+      <c r="D1304" t="inlineStr">
+        <is>
+          <t>https://www.capitalcityroofing.net/roof-repair-roswell-ga</t>
+        </is>
+      </c>
+      <c r="E1304" t="inlineStr">
+        <is>
+          <t>Centers View</t>
+        </is>
+      </c>
+      <c r="F1304" t="inlineStr">
+        <is>
+          <t>info@capitalcityroofing.net</t>
+        </is>
+      </c>
+      <c r="G1304" t="inlineStr">
+        <is>
+          <t>(404) 897-0337</t>
+        </is>
+      </c>
+      <c r="H1304" t="inlineStr">
+        <is>
+          <t>Roswell GA</t>
+        </is>
+      </c>
+      <c r="I1304" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1304" t="inlineStr">
+        <is>
+          <t>roof repair company Roswell GA</t>
+        </is>
+      </c>
+      <c r="K1304" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1304" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>Roof Repair &amp; Replacement Services in Roswell, GA</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>roswell-ga.guyroofingcoinc.com</t>
+        </is>
+      </c>
+      <c r="D1305" t="inlineStr">
+        <is>
+          <t>https://roswell-ga.guyroofingcoinc.com/</t>
+        </is>
+      </c>
+      <c r="E1305" t="inlineStr">
+        <is>
+          <t>Serve We</t>
+        </is>
+      </c>
+      <c r="F1305" t="inlineStr">
+        <is>
+          <t>info@guyroofingcoinc.com</t>
+        </is>
+      </c>
+      <c r="G1305" t="inlineStr">
+        <is>
+          <t>(770) 727-3408</t>
+        </is>
+      </c>
+      <c r="H1305" t="inlineStr">
+        <is>
+          <t>Roswell GA</t>
+        </is>
+      </c>
+      <c r="I1305" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1305" t="inlineStr">
+        <is>
+          <t>roof repair company Roswell GA</t>
+        </is>
+      </c>
+      <c r="K1305" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1305" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 21:45 UTC (cycle 136)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1305"/>
+  <dimension ref="A1:L1310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -76854,6 +76854,294 @@
         </is>
       </c>
     </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>Capitol City Roofing</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>capitolcityroofing.com</t>
+        </is>
+      </c>
+      <c r="D1306" t="inlineStr">
+        <is>
+          <t>https://capitolcityroofing.com/</t>
+        </is>
+      </c>
+      <c r="E1306" t="inlineStr">
+        <is>
+          <t>City Roofing</t>
+        </is>
+      </c>
+      <c r="F1306" t="inlineStr">
+        <is>
+          <t>peltrp2@aol.com</t>
+        </is>
+      </c>
+      <c r="G1306" t="inlineStr">
+        <is>
+          <t>334-277-3311</t>
+        </is>
+      </c>
+      <c r="H1306" t="inlineStr">
+        <is>
+          <t>Montgomery AL</t>
+        </is>
+      </c>
+      <c r="I1306" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1306" t="inlineStr">
+        <is>
+          <t>roof repair company Montgomery AL</t>
+        </is>
+      </c>
+      <c r="K1306" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1306" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>Superior Plumbing</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>superiorplumbingpros.com</t>
+        </is>
+      </c>
+      <c r="D1307" t="inlineStr">
+        <is>
+          <t>https://superiorplumbingpros.com/devenport-ia/</t>
+        </is>
+      </c>
+      <c r="E1307" t="inlineStr"/>
+      <c r="F1307" t="inlineStr">
+        <is>
+          <t>kelly.superiorplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1307" t="inlineStr">
+        <is>
+          <t>(563) 285-2540</t>
+        </is>
+      </c>
+      <c r="H1307" t="inlineStr">
+        <is>
+          <t>Davenport IA</t>
+        </is>
+      </c>
+      <c r="I1307" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1307" t="inlineStr">
+        <is>
+          <t>plumbing company Davenport IA</t>
+        </is>
+      </c>
+      <c r="K1307" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1307" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>Plumbing Contractor | Davenport, IA | C. Ewert Plumbing</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>ewertplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1308" t="inlineStr">
+        <is>
+          <t>https://www.ewertplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E1308" t="inlineStr"/>
+      <c r="F1308" t="inlineStr">
+        <is>
+          <t>office@ewertplumbing.com</t>
+        </is>
+      </c>
+      <c r="G1308" t="inlineStr">
+        <is>
+          <t>563-322-3222</t>
+        </is>
+      </c>
+      <c r="H1308" t="inlineStr">
+        <is>
+          <t>Davenport IA</t>
+        </is>
+      </c>
+      <c r="I1308" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1308" t="inlineStr">
+        <is>
+          <t>plumbing company Davenport IA</t>
+        </is>
+      </c>
+      <c r="K1308" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1308" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>IRoof</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>iroofpros.com</t>
+        </is>
+      </c>
+      <c r="D1309" t="inlineStr">
+        <is>
+          <t>https://iroofpros.com/</t>
+        </is>
+      </c>
+      <c r="E1309" t="inlineStr">
+        <is>
+          <t>Analytics Analytics</t>
+        </is>
+      </c>
+      <c r="F1309" t="inlineStr">
+        <is>
+          <t>info@iroofpros.com</t>
+        </is>
+      </c>
+      <c r="G1309" t="inlineStr">
+        <is>
+          <t>(334) 300-7027</t>
+        </is>
+      </c>
+      <c r="H1309" t="inlineStr">
+        <is>
+          <t>Montgomery AL</t>
+        </is>
+      </c>
+      <c r="I1309" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1309" t="inlineStr">
+        <is>
+          <t>roof repair company Montgomery AL</t>
+        </is>
+      </c>
+      <c r="K1309" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1309" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>Candor Construct &amp; Roofing</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>candorconstructandroofing.com</t>
+        </is>
+      </c>
+      <c r="D1310" t="inlineStr">
+        <is>
+          <t>https://candorconstructandroofing.com/service-areas/midland</t>
+        </is>
+      </c>
+      <c r="E1310" t="inlineStr"/>
+      <c r="F1310" t="inlineStr">
+        <is>
+          <t>contact@candorconstruct.com</t>
+        </is>
+      </c>
+      <c r="G1310" t="inlineStr">
+        <is>
+          <t>(806) 224-2836</t>
+        </is>
+      </c>
+      <c r="H1310" t="inlineStr">
+        <is>
+          <t>Midland TX</t>
+        </is>
+      </c>
+      <c r="I1310" t="n">
+        <v>86</v>
+      </c>
+      <c r="J1310" t="inlineStr">
+        <is>
+          <t>roofing contractor Midland TX</t>
+        </is>
+      </c>
+      <c r="K1310" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1310" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 21:46 UTC (cycle 137)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1310"/>
+  <dimension ref="A1:L1321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -76935,7 +76935,6 @@
           <t>https://superiorplumbingpros.com/devenport-ia/</t>
         </is>
       </c>
-      <c r="E1307" t="inlineStr"/>
       <c r="F1307" t="inlineStr">
         <is>
           <t>kelly.superiorplumbing@gmail.com</t>
@@ -76991,7 +76990,6 @@
           <t>https://www.ewertplumbing.com/</t>
         </is>
       </c>
-      <c r="E1308" t="inlineStr"/>
       <c r="F1308" t="inlineStr">
         <is>
           <t>office@ewertplumbing.com</t>
@@ -77107,7 +77105,6 @@
           <t>https://candorconstructandroofing.com/service-areas/midland</t>
         </is>
       </c>
-      <c r="E1310" t="inlineStr"/>
       <c r="F1310" t="inlineStr">
         <is>
           <t>contact@candorconstruct.com</t>
@@ -77137,6 +77134,654 @@
         </is>
       </c>
       <c r="L1310" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>Red Hawk Roofing</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>redhawkroofing.com</t>
+        </is>
+      </c>
+      <c r="D1311" t="inlineStr">
+        <is>
+          <t>https://redhawkroofing.com/roof-replacement-lakewood-co</t>
+        </is>
+      </c>
+      <c r="E1311" t="inlineStr">
+        <is>
+          <t>Red Hawk</t>
+        </is>
+      </c>
+      <c r="F1311" t="inlineStr">
+        <is>
+          <t>info@redhawkroofing.com</t>
+        </is>
+      </c>
+      <c r="G1311" t="inlineStr">
+        <is>
+          <t>(720) 771-8921</t>
+        </is>
+      </c>
+      <c r="H1311" t="inlineStr">
+        <is>
+          <t>Lakewood CO</t>
+        </is>
+      </c>
+      <c r="I1311" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1311" t="inlineStr">
+        <is>
+          <t>roof replacement Lakewood CO</t>
+        </is>
+      </c>
+      <c r="K1311" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1311" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>Magic Plumbing</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>mymagicplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1312" t="inlineStr">
+        <is>
+          <t>https://mymagicplumbing.com/plumbing-services-in-boise-id/</t>
+        </is>
+      </c>
+      <c r="E1312" t="inlineStr">
+        <is>
+          <t>Plumbing Services</t>
+        </is>
+      </c>
+      <c r="F1312" t="inlineStr">
+        <is>
+          <t>info@mymagicplumbing.com</t>
+        </is>
+      </c>
+      <c r="G1312" t="inlineStr">
+        <is>
+          <t>208-606-7339</t>
+        </is>
+      </c>
+      <c r="H1312" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I1312" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1312" t="inlineStr">
+        <is>
+          <t>plumber Boise ID</t>
+        </is>
+      </c>
+      <c r="K1312" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1312" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>Paul Wright Roofing - Have a problem with your roof? Paul Wright Roofing can hel</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>paulwrightroofing.com</t>
+        </is>
+      </c>
+      <c r="D1313" t="inlineStr">
+        <is>
+          <t>https://paulwrightroofing.com/bethlehem-roofing/</t>
+        </is>
+      </c>
+      <c r="E1313" t="inlineStr">
+        <is>
+          <t>Roof Maintenance</t>
+        </is>
+      </c>
+      <c r="F1313" t="inlineStr">
+        <is>
+          <t>clientservices@paulwrightroofing.net</t>
+        </is>
+      </c>
+      <c r="G1313" t="inlineStr">
+        <is>
+          <t>(610) 770-3979</t>
+        </is>
+      </c>
+      <c r="H1313" t="inlineStr">
+        <is>
+          <t>Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="I1313" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1313" t="inlineStr">
+        <is>
+          <t>roofing contractor Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="K1313" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1313" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>Professional Plumbing</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>proplumbingtucson.com</t>
+        </is>
+      </c>
+      <c r="D1314" t="inlineStr">
+        <is>
+          <t>https://proplumbingtucson.com/</t>
+        </is>
+      </c>
+      <c r="E1314" t="inlineStr"/>
+      <c r="F1314" t="inlineStr">
+        <is>
+          <t>office@proplumbtucson.com</t>
+        </is>
+      </c>
+      <c r="G1314" t="inlineStr">
+        <is>
+          <t>520-749-0777</t>
+        </is>
+      </c>
+      <c r="H1314" t="inlineStr">
+        <is>
+          <t>Tucson AZ</t>
+        </is>
+      </c>
+      <c r="I1314" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1314" t="inlineStr">
+        <is>
+          <t>plumbing company Tucson AZ</t>
+        </is>
+      </c>
+      <c r="K1314" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1314" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>Bachman's Roofing</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>bachmansroofing.com</t>
+        </is>
+      </c>
+      <c r="D1315" t="inlineStr">
+        <is>
+          <t>https://bachmansroofing.com/areas-served/bethlehem/</t>
+        </is>
+      </c>
+      <c r="E1315" t="inlineStr"/>
+      <c r="F1315" t="inlineStr">
+        <is>
+          <t>info@bachmansroofing.com</t>
+        </is>
+      </c>
+      <c r="G1315" t="inlineStr">
+        <is>
+          <t>(888) 775-7384</t>
+        </is>
+      </c>
+      <c r="H1315" t="inlineStr">
+        <is>
+          <t>Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="I1315" t="n">
+        <v>98</v>
+      </c>
+      <c r="J1315" t="inlineStr">
+        <is>
+          <t>roofing contractor Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="K1315" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1315" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>Roof Worx, LLC</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>myroofworx.com</t>
+        </is>
+      </c>
+      <c r="D1316" t="inlineStr">
+        <is>
+          <t>https://myroofworx.com/service-areas/lakewood/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E1316" t="inlineStr">
+        <is>
+          <t>Professional Highlights</t>
+        </is>
+      </c>
+      <c r="F1316" t="inlineStr">
+        <is>
+          <t>sales@myroofworx.com</t>
+        </is>
+      </c>
+      <c r="G1316" t="inlineStr">
+        <is>
+          <t>(303) 353-1825</t>
+        </is>
+      </c>
+      <c r="H1316" t="inlineStr">
+        <is>
+          <t>Lakewood CO</t>
+        </is>
+      </c>
+      <c r="I1316" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1316" t="inlineStr">
+        <is>
+          <t>roof replacement Lakewood CO</t>
+        </is>
+      </c>
+      <c r="K1316" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1316" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>Roofing Company in Lakewood | Free Inspections — PRQ Exteriors</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>prqexteriors.com</t>
+        </is>
+      </c>
+      <c r="D1317" t="inlineStr">
+        <is>
+          <t>https://www.prqexteriors.com/locations/lakewood/</t>
+        </is>
+      </c>
+      <c r="E1317" t="inlineStr">
+        <is>
+          <t>Exteriors Get</t>
+        </is>
+      </c>
+      <c r="F1317" t="inlineStr">
+        <is>
+          <t>sales@prqexteriors.com</t>
+        </is>
+      </c>
+      <c r="G1317" t="inlineStr">
+        <is>
+          <t>(720) 778-9854</t>
+        </is>
+      </c>
+      <c r="H1317" t="inlineStr">
+        <is>
+          <t>Lakewood CO</t>
+        </is>
+      </c>
+      <c r="I1317" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1317" t="inlineStr">
+        <is>
+          <t>roof replacement Lakewood CO</t>
+        </is>
+      </c>
+      <c r="K1317" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1317" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>Blue Peaks Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>bluepeaksroofing.com</t>
+        </is>
+      </c>
+      <c r="D1318" t="inlineStr">
+        <is>
+          <t>https://bluepeaksroofing.com/lakewood-co/</t>
+        </is>
+      </c>
+      <c r="E1318" t="inlineStr">
+        <is>
+          <t>At Blue</t>
+        </is>
+      </c>
+      <c r="F1318" t="inlineStr">
+        <is>
+          <t>primedigitalseo@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1318" t="inlineStr">
+        <is>
+          <t>(303) 808-0687</t>
+        </is>
+      </c>
+      <c r="H1318" t="inlineStr">
+        <is>
+          <t>Lakewood CO</t>
+        </is>
+      </c>
+      <c r="I1318" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1318" t="inlineStr">
+        <is>
+          <t>roof replacement Lakewood CO</t>
+        </is>
+      </c>
+      <c r="K1318" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1318" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr">
+        <is>
+          <t>VM Power Construction</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>vmpowerconstruction.com</t>
+        </is>
+      </c>
+      <c r="D1319" t="inlineStr">
+        <is>
+          <t>https://vmpowerconstruction.com/locations/bethlehem/roofing</t>
+        </is>
+      </c>
+      <c r="E1319" t="inlineStr">
+        <is>
+          <t>Resources Helpful</t>
+        </is>
+      </c>
+      <c r="F1319" t="inlineStr">
+        <is>
+          <t>info@vmpowerconstruction.com</t>
+        </is>
+      </c>
+      <c r="G1319" t="inlineStr">
+        <is>
+          <t>(484) 942-7316</t>
+        </is>
+      </c>
+      <c r="H1319" t="inlineStr">
+        <is>
+          <t>Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="I1319" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1319" t="inlineStr">
+        <is>
+          <t>roofing contractor Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="K1319" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1319" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>Plumber in Boise, ID | Boise Plumbing Pros</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>boiseplumb.com</t>
+        </is>
+      </c>
+      <c r="D1320" t="inlineStr">
+        <is>
+          <t>https://boiseplumb.com/</t>
+        </is>
+      </c>
+      <c r="E1320" t="inlineStr">
+        <is>
+          <t>Treasure Valley</t>
+        </is>
+      </c>
+      <c r="F1320" t="inlineStr">
+        <is>
+          <t>hello@boiseplumb.com</t>
+        </is>
+      </c>
+      <c r="G1320" t="inlineStr">
+        <is>
+          <t>(555) 000-0000</t>
+        </is>
+      </c>
+      <c r="H1320" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I1320" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1320" t="inlineStr">
+        <is>
+          <t>plumber Boise ID</t>
+        </is>
+      </c>
+      <c r="K1320" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1320" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>PA Homeowners Guide</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>pahomeownersguide.com</t>
+        </is>
+      </c>
+      <c r="D1321" t="inlineStr">
+        <is>
+          <t>https://www.pahomeownersguide.com/roofingcontractor/bethlehem</t>
+        </is>
+      </c>
+      <c r="E1321" t="inlineStr">
+        <is>
+          <t>Click Here</t>
+        </is>
+      </c>
+      <c r="F1321" t="inlineStr">
+        <is>
+          <t>sales@mjaybuilders.com</t>
+        </is>
+      </c>
+      <c r="G1321" t="inlineStr"/>
+      <c r="H1321" t="inlineStr">
+        <is>
+          <t>Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="I1321" t="n">
+        <v>66</v>
+      </c>
+      <c r="J1321" t="inlineStr">
+        <is>
+          <t>roofing contractor Bethlehem PA</t>
+        </is>
+      </c>
+      <c r="K1321" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1321" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 21:48 UTC (cycle 138)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1321"/>
+  <dimension ref="A1:L1327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -77340,7 +77340,6 @@
           <t>https://proplumbingtucson.com/</t>
         </is>
       </c>
-      <c r="E1314" t="inlineStr"/>
       <c r="F1314" t="inlineStr">
         <is>
           <t>office@proplumbtucson.com</t>
@@ -77396,7 +77395,6 @@
           <t>https://bachmansroofing.com/areas-served/bethlehem/</t>
         </is>
       </c>
-      <c r="E1315" t="inlineStr"/>
       <c r="F1315" t="inlineStr">
         <is>
           <t>info@bachmansroofing.com</t>
@@ -77762,7 +77760,6 @@
           <t>sales@mjaybuilders.com</t>
         </is>
       </c>
-      <c r="G1321" t="inlineStr"/>
       <c r="H1321" t="inlineStr">
         <is>
           <t>Bethlehem PA</t>
@@ -77782,6 +77779,366 @@
         </is>
       </c>
       <c r="L1321" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>Nevada Pacific Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>nvpacifichvac.com</t>
+        </is>
+      </c>
+      <c r="D1322" t="inlineStr">
+        <is>
+          <t>https://www.nvpacifichvac.com/services/air-conditioning-repair</t>
+        </is>
+      </c>
+      <c r="E1322" t="inlineStr">
+        <is>
+          <t>Nevada Pacific</t>
+        </is>
+      </c>
+      <c r="F1322" t="inlineStr">
+        <is>
+          <t>info@nvpacifichvac.com</t>
+        </is>
+      </c>
+      <c r="G1322" t="inlineStr">
+        <is>
+          <t>775-230-3749</t>
+        </is>
+      </c>
+      <c r="H1322" t="inlineStr">
+        <is>
+          <t>Carson City NV</t>
+        </is>
+      </c>
+      <c r="I1322" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1322" t="inlineStr">
+        <is>
+          <t>air conditioning repair Carson City NV</t>
+        </is>
+      </c>
+      <c r="K1322" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1322" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>Seatown Electric Plumbing Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>seatownservices.com</t>
+        </is>
+      </c>
+      <c r="D1323" t="inlineStr">
+        <is>
+          <t>https://www.seatownservices.com/hvac-services/air-conditioning-installation/</t>
+        </is>
+      </c>
+      <c r="E1323" t="inlineStr">
+        <is>
+          <t>Plumbing Heating</t>
+        </is>
+      </c>
+      <c r="F1323" t="inlineStr">
+        <is>
+          <t>info@seatownservices.com</t>
+        </is>
+      </c>
+      <c r="G1323" t="inlineStr">
+        <is>
+          <t>(360) 549-8262</t>
+        </is>
+      </c>
+      <c r="H1323" t="inlineStr">
+        <is>
+          <t>Seattle WA</t>
+        </is>
+      </c>
+      <c r="I1323" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1323" t="inlineStr">
+        <is>
+          <t>AC installation Seattle WA</t>
+        </is>
+      </c>
+      <c r="K1323" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1323" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>Elite Air of West Texas</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>eliteairofwesttx.com</t>
+        </is>
+      </c>
+      <c r="D1324" t="inlineStr">
+        <is>
+          <t>https://www.eliteairofwesttx.com/midland-heat-pumps/heat-pump-installation/</t>
+        </is>
+      </c>
+      <c r="E1324" t="inlineStr">
+        <is>
+          <t>Pump Installation</t>
+        </is>
+      </c>
+      <c r="F1324" t="inlineStr">
+        <is>
+          <t>jimmy@eliteairofwesttx.com</t>
+        </is>
+      </c>
+      <c r="G1324" t="inlineStr">
+        <is>
+          <t>432-901-0171</t>
+        </is>
+      </c>
+      <c r="H1324" t="inlineStr">
+        <is>
+          <t>Odessa TX</t>
+        </is>
+      </c>
+      <c r="I1324" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1324" t="inlineStr">
+        <is>
+          <t>heat pump installation Odessa TX</t>
+        </is>
+      </c>
+      <c r="K1324" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1324" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>Fuse Service: Heating &amp; Air Conditioning | HVAC Contractor Seattle, WA</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>fusesea.com</t>
+        </is>
+      </c>
+      <c r="D1325" t="inlineStr">
+        <is>
+          <t>https://fusesea.com/air-conditioning-installation/</t>
+        </is>
+      </c>
+      <c r="E1325" t="inlineStr">
+        <is>
+          <t>Fuse Service</t>
+        </is>
+      </c>
+      <c r="F1325" t="inlineStr">
+        <is>
+          <t>support@fusesea.com</t>
+        </is>
+      </c>
+      <c r="G1325" t="inlineStr">
+        <is>
+          <t>(425) 380-4300</t>
+        </is>
+      </c>
+      <c r="H1325" t="inlineStr">
+        <is>
+          <t>Seattle WA</t>
+        </is>
+      </c>
+      <c r="I1325" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1325" t="inlineStr">
+        <is>
+          <t>AC installation Seattle WA</t>
+        </is>
+      </c>
+      <c r="K1325" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1325" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>legacyac.com</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>legacyac.com</t>
+        </is>
+      </c>
+      <c r="D1326" t="inlineStr">
+        <is>
+          <t>https://legacyac.com/service-area/carson-city-nevada-ac-repair/</t>
+        </is>
+      </c>
+      <c r="E1326" t="inlineStr">
+        <is>
+          <t>Forever Innovating</t>
+        </is>
+      </c>
+      <c r="F1326" t="inlineStr">
+        <is>
+          <t>info@legacyac.com</t>
+        </is>
+      </c>
+      <c r="G1326" t="inlineStr">
+        <is>
+          <t>(725) 253-2522</t>
+        </is>
+      </c>
+      <c r="H1326" t="inlineStr">
+        <is>
+          <t>Carson City NV</t>
+        </is>
+      </c>
+      <c r="I1326" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1326" t="inlineStr">
+        <is>
+          <t>air conditioning repair Carson City NV</t>
+        </is>
+      </c>
+      <c r="K1326" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1326" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>My Blog</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>smarthvacsolution.com</t>
+        </is>
+      </c>
+      <c r="D1327" t="inlineStr">
+        <is>
+          <t>https://www.smarthvacsolution.com/</t>
+        </is>
+      </c>
+      <c r="E1327" t="inlineStr">
+        <is>
+          <t>Carson City</t>
+        </is>
+      </c>
+      <c r="F1327" t="inlineStr">
+        <is>
+          <t>inquiry@smarthvacsolution.com</t>
+        </is>
+      </c>
+      <c r="G1327" t="inlineStr">
+        <is>
+          <t>775-490-8107</t>
+        </is>
+      </c>
+      <c r="H1327" t="inlineStr">
+        <is>
+          <t>Carson City NV</t>
+        </is>
+      </c>
+      <c r="I1327" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1327" t="inlineStr">
+        <is>
+          <t>air conditioning repair Carson City NV</t>
+        </is>
+      </c>
+      <c r="K1327" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1327" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 21:49 UTC (cycle 139)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1327"/>
+  <dimension ref="A1:L1330"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -78144,6 +78144,186 @@
         </is>
       </c>
     </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>Metal Roofing in Cheyenne, WY</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>cowboystatemetalroofing.com</t>
+        </is>
+      </c>
+      <c r="D1328" t="inlineStr">
+        <is>
+          <t>https://cowboystatemetalroofing.com/cheyenne/</t>
+        </is>
+      </c>
+      <c r="E1328" t="inlineStr">
+        <is>
+          <t>Cowboy State</t>
+        </is>
+      </c>
+      <c r="F1328" t="inlineStr">
+        <is>
+          <t>compassleadgroup@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1328" t="inlineStr">
+        <is>
+          <t>(307) 298-6829</t>
+        </is>
+      </c>
+      <c r="H1328" t="inlineStr">
+        <is>
+          <t>Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="I1328" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1328" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="K1328" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1328" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr">
+        <is>
+          <t>Petes Builders</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>petesbuilders.com</t>
+        </is>
+      </c>
+      <c r="D1329" t="inlineStr">
+        <is>
+          <t>https://petesbuilders.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E1329" t="inlineStr">
+        <is>
+          <t>Great Team</t>
+        </is>
+      </c>
+      <c r="F1329" t="inlineStr">
+        <is>
+          <t>info@petesbuilders.com</t>
+        </is>
+      </c>
+      <c r="G1329" t="inlineStr">
+        <is>
+          <t>307-314-1005</t>
+        </is>
+      </c>
+      <c r="H1329" t="inlineStr">
+        <is>
+          <t>Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="I1329" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1329" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="K1329" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1329" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>High Plains Custom Metal</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>highplainscustommetal.com</t>
+        </is>
+      </c>
+      <c r="D1330" t="inlineStr">
+        <is>
+          <t>https://highplainscustommetal.com/</t>
+        </is>
+      </c>
+      <c r="E1330" t="inlineStr">
+        <is>
+          <t>Northern Colorado</t>
+        </is>
+      </c>
+      <c r="F1330" t="inlineStr">
+        <is>
+          <t>info@highplainscustommetal.com</t>
+        </is>
+      </c>
+      <c r="G1330" t="inlineStr">
+        <is>
+          <t>307-331-6449</t>
+        </is>
+      </c>
+      <c r="H1330" t="inlineStr">
+        <is>
+          <t>Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="I1330" t="n">
+        <v>94</v>
+      </c>
+      <c r="J1330" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="K1330" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1330" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 21:53 UTC (cycle 142)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1330"/>
+  <dimension ref="A1:L1334"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -78324,6 +78324,234 @@
         </is>
       </c>
     </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr">
+        <is>
+          <t>full AMC site</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>alliedmechanicalcontracting.com</t>
+        </is>
+      </c>
+      <c r="D1331" t="inlineStr">
+        <is>
+          <t>https://alliedmechanicalcontracting.com/</t>
+        </is>
+      </c>
+      <c r="E1331" t="inlineStr"/>
+      <c r="F1331" t="inlineStr">
+        <is>
+          <t>don@alliedmechanicalcontracting.com</t>
+        </is>
+      </c>
+      <c r="G1331" t="inlineStr">
+        <is>
+          <t>1347833589</t>
+        </is>
+      </c>
+      <c r="H1331" t="inlineStr">
+        <is>
+          <t>Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="I1331" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1331" t="inlineStr">
+        <is>
+          <t>HVAC contractor Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="K1331" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1331" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>HVAC Services in Mount Vernon, NY | Manny HVAC</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>mannyhvac.com</t>
+        </is>
+      </c>
+      <c r="D1332" t="inlineStr">
+        <is>
+          <t>https://mannyhvac.com/areas/mount-vernon</t>
+        </is>
+      </c>
+      <c r="E1332" t="inlineStr">
+        <is>
+          <t>Work About</t>
+        </is>
+      </c>
+      <c r="F1332" t="inlineStr">
+        <is>
+          <t>service@mannyhvac.com</t>
+        </is>
+      </c>
+      <c r="G1332" t="inlineStr">
+        <is>
+          <t>(914) 461-7296</t>
+        </is>
+      </c>
+      <c r="H1332" t="inlineStr">
+        <is>
+          <t>Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="I1332" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1332" t="inlineStr">
+        <is>
+          <t>HVAC contractor Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="K1332" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1332" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr">
+        <is>
+          <t>Mount Vernon HVAC Service and Sales</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>mountvernonhvac.com</t>
+        </is>
+      </c>
+      <c r="D1333" t="inlineStr">
+        <is>
+          <t>https://www.mountvernonhvac.com/</t>
+        </is>
+      </c>
+      <c r="E1333" t="inlineStr"/>
+      <c r="F1333" t="inlineStr">
+        <is>
+          <t>admin@mountvernonhvac.com</t>
+        </is>
+      </c>
+      <c r="G1333" t="inlineStr">
+        <is>
+          <t>(914) 344-6550</t>
+        </is>
+      </c>
+      <c r="H1333" t="inlineStr">
+        <is>
+          <t>Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="I1333" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1333" t="inlineStr">
+        <is>
+          <t>HVAC contractor Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="K1333" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1333" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr">
+        <is>
+          <t>HVAC Mechanical Contractor | Mt Vernon, NY | Klairgar Inc.</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>klairgar.com</t>
+        </is>
+      </c>
+      <c r="D1334" t="inlineStr">
+        <is>
+          <t>https://www.klairgar.com/</t>
+        </is>
+      </c>
+      <c r="E1334" t="inlineStr"/>
+      <c r="F1334" t="inlineStr">
+        <is>
+          <t>klairgar@aol.com</t>
+        </is>
+      </c>
+      <c r="G1334" t="inlineStr">
+        <is>
+          <t>(914) 699-1520</t>
+        </is>
+      </c>
+      <c r="H1334" t="inlineStr">
+        <is>
+          <t>Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="I1334" t="n">
+        <v>80</v>
+      </c>
+      <c r="J1334" t="inlineStr">
+        <is>
+          <t>HVAC contractor Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="K1334" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1334" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 21:55 UTC (cycle 143)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1334"/>
+  <dimension ref="A1:L1341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -78345,7 +78345,6 @@
           <t>https://alliedmechanicalcontracting.com/</t>
         </is>
       </c>
-      <c r="E1331" t="inlineStr"/>
       <c r="F1331" t="inlineStr">
         <is>
           <t>don@alliedmechanicalcontracting.com</t>
@@ -78461,7 +78460,6 @@
           <t>https://www.mountvernonhvac.com/</t>
         </is>
       </c>
-      <c r="E1333" t="inlineStr"/>
       <c r="F1333" t="inlineStr">
         <is>
           <t>admin@mountvernonhvac.com</t>
@@ -78517,7 +78515,6 @@
           <t>https://www.klairgar.com/</t>
         </is>
       </c>
-      <c r="E1334" t="inlineStr"/>
       <c r="F1334" t="inlineStr">
         <is>
           <t>klairgar@aol.com</t>
@@ -78547,6 +78544,422 @@
         </is>
       </c>
       <c r="L1334" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>Roper Roofing &amp; Solar</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>roperroofingandsolar.com</t>
+        </is>
+      </c>
+      <c r="D1335" t="inlineStr">
+        <is>
+          <t>https://roperroofingandsolar.com/service-areas/westminster-co/</t>
+        </is>
+      </c>
+      <c r="E1335" t="inlineStr">
+        <is>
+          <t>Services You</t>
+        </is>
+      </c>
+      <c r="F1335" t="inlineStr">
+        <is>
+          <t>info@roperroofing.com</t>
+        </is>
+      </c>
+      <c r="G1335" t="inlineStr">
+        <is>
+          <t>(720) 475-1065</t>
+        </is>
+      </c>
+      <c r="H1335" t="inlineStr">
+        <is>
+          <t>Westminster CO</t>
+        </is>
+      </c>
+      <c r="I1335" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1335" t="inlineStr">
+        <is>
+          <t>residential roofing company Westminster CO</t>
+        </is>
+      </c>
+      <c r="K1335" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1335" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>PUMPED</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>heatpumpla.com</t>
+        </is>
+      </c>
+      <c r="D1336" t="inlineStr">
+        <is>
+          <t>https://heatpumpla.com/</t>
+        </is>
+      </c>
+      <c r="E1336" t="inlineStr"/>
+      <c r="F1336" t="inlineStr">
+        <is>
+          <t>hello@heatpumpla.com</t>
+        </is>
+      </c>
+      <c r="G1336" t="inlineStr">
+        <is>
+          <t>(323) 285-3005</t>
+        </is>
+      </c>
+      <c r="H1336" t="inlineStr">
+        <is>
+          <t>Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="I1336" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1336" t="inlineStr">
+        <is>
+          <t>heat pump installation Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="K1336" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1336" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>LC Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>lahvaclc.com</t>
+        </is>
+      </c>
+      <c r="D1337" t="inlineStr">
+        <is>
+          <t>https://lahvaclc.com/services/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E1337" t="inlineStr">
+        <is>
+          <t>Online Scheduling</t>
+        </is>
+      </c>
+      <c r="F1337" t="inlineStr">
+        <is>
+          <t>support@lahvaclc.com</t>
+        </is>
+      </c>
+      <c r="G1337" t="inlineStr">
+        <is>
+          <t>(323) 970-3113</t>
+        </is>
+      </c>
+      <c r="H1337" t="inlineStr">
+        <is>
+          <t>Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="I1337" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1337" t="inlineStr">
+        <is>
+          <t>heat pump installation Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="K1337" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1337" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>Tornado HVAC</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>tornadohvacca.com</t>
+        </is>
+      </c>
+      <c r="D1338" t="inlineStr">
+        <is>
+          <t>https://tornadohvacca.com/Service/heat-pump-installation-in-los-angeles-ca/</t>
+        </is>
+      </c>
+      <c r="E1338" t="inlineStr">
+        <is>
+          <t>At Tornado</t>
+        </is>
+      </c>
+      <c r="F1338" t="inlineStr">
+        <is>
+          <t>tornadohvac1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1338" t="inlineStr">
+        <is>
+          <t>(818) 740-5813</t>
+        </is>
+      </c>
+      <c r="H1338" t="inlineStr">
+        <is>
+          <t>Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="I1338" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1338" t="inlineStr">
+        <is>
+          <t>heat pump installation Los Angeles CA</t>
+        </is>
+      </c>
+      <c r="K1338" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1338" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr">
+        <is>
+          <t>Mile High Roofing Services</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>milehighroofingservices.com</t>
+        </is>
+      </c>
+      <c r="D1339" t="inlineStr">
+        <is>
+          <t>https://milehighroofingservices.com/residential-roofing/</t>
+        </is>
+      </c>
+      <c r="E1339" t="inlineStr">
+        <is>
+          <t>North Metro</t>
+        </is>
+      </c>
+      <c r="F1339" t="inlineStr">
+        <is>
+          <t>info@mhpsllc.com</t>
+        </is>
+      </c>
+      <c r="G1339" t="inlineStr">
+        <is>
+          <t>(720) 999-8282</t>
+        </is>
+      </c>
+      <c r="H1339" t="inlineStr">
+        <is>
+          <t>Westminster CO</t>
+        </is>
+      </c>
+      <c r="I1339" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1339" t="inlineStr">
+        <is>
+          <t>residential roofing company Westminster CO</t>
+        </is>
+      </c>
+      <c r="K1339" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1339" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="inlineStr">
+        <is>
+          <t>Weddle &amp; Sons Roofing</t>
+        </is>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>weddleandsons.com</t>
+        </is>
+      </c>
+      <c r="D1340" t="inlineStr">
+        <is>
+          <t>https://weddleandsons.com/</t>
+        </is>
+      </c>
+      <c r="E1340" t="inlineStr">
+        <is>
+          <t>Sons Join</t>
+        </is>
+      </c>
+      <c r="F1340" t="inlineStr">
+        <is>
+          <t>info@weddleandsons.com</t>
+        </is>
+      </c>
+      <c r="G1340" t="inlineStr">
+        <is>
+          <t>(844) 974-7663</t>
+        </is>
+      </c>
+      <c r="H1340" t="inlineStr">
+        <is>
+          <t>Westminster CO</t>
+        </is>
+      </c>
+      <c r="I1340" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1340" t="inlineStr">
+        <is>
+          <t>residential roofing company Westminster CO</t>
+        </is>
+      </c>
+      <c r="K1340" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1340" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="inlineStr">
+        <is>
+          <t>Residential &amp; Commercial Roofing in Westminster, CO</t>
+        </is>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>westminster-co.whiteroofingcolorado.com</t>
+        </is>
+      </c>
+      <c r="D1341" t="inlineStr">
+        <is>
+          <t>https://westminster-co.whiteroofingcolorado.com/</t>
+        </is>
+      </c>
+      <c r="E1341" t="inlineStr">
+        <is>
+          <t>White Roofing</t>
+        </is>
+      </c>
+      <c r="F1341" t="inlineStr">
+        <is>
+          <t>info@whiteroofingcolorado.com</t>
+        </is>
+      </c>
+      <c r="G1341" t="inlineStr">
+        <is>
+          <t>(303) 952-2586</t>
+        </is>
+      </c>
+      <c r="H1341" t="inlineStr">
+        <is>
+          <t>Westminster CO</t>
+        </is>
+      </c>
+      <c r="I1341" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1341" t="inlineStr">
+        <is>
+          <t>residential roofing company Westminster CO</t>
+        </is>
+      </c>
+      <c r="K1341" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1341" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 21:56 UTC (cycle 144)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1341"/>
+  <dimension ref="A1:L1347"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -78630,7 +78630,6 @@
           <t>https://heatpumpla.com/</t>
         </is>
       </c>
-      <c r="E1336" t="inlineStr"/>
       <c r="F1336" t="inlineStr">
         <is>
           <t>hello@heatpumpla.com</t>
@@ -78960,6 +78959,354 @@
         </is>
       </c>
       <c r="L1341" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr">
+        <is>
+          <t>Energy Savers of Columbus | Proudly Serving West Georgia &amp; East Alabama for Over</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>energysaversair.com</t>
+        </is>
+      </c>
+      <c r="D1342" t="inlineStr">
+        <is>
+          <t>https://energysaversair.com/columbus-ga/hvac/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E1342" t="inlineStr"/>
+      <c r="F1342" t="inlineStr">
+        <is>
+          <t>customerservice@energysaversair.com</t>
+        </is>
+      </c>
+      <c r="G1342" t="inlineStr">
+        <is>
+          <t>(706) 250-7325</t>
+        </is>
+      </c>
+      <c r="H1342" t="inlineStr">
+        <is>
+          <t>Columbus GA</t>
+        </is>
+      </c>
+      <c r="I1342" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1342" t="inlineStr">
+        <is>
+          <t>furnace repair Columbus GA</t>
+        </is>
+      </c>
+      <c r="K1342" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1342" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr">
+        <is>
+          <t>County Line LLC Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>countylinellcair.com</t>
+        </is>
+      </c>
+      <c r="D1343" t="inlineStr">
+        <is>
+          <t>https://www.countylinellcair.com/columbus-ga-heating-air-conditioning-contractor/</t>
+        </is>
+      </c>
+      <c r="E1343" t="inlineStr">
+        <is>
+          <t>Walker Lee</t>
+        </is>
+      </c>
+      <c r="F1343" t="inlineStr">
+        <is>
+          <t>countylinellc@att.net</t>
+        </is>
+      </c>
+      <c r="G1343" t="inlineStr">
+        <is>
+          <t>706-322-5343</t>
+        </is>
+      </c>
+      <c r="H1343" t="inlineStr">
+        <is>
+          <t>Columbus GA</t>
+        </is>
+      </c>
+      <c r="I1343" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1343" t="inlineStr">
+        <is>
+          <t>furnace repair Columbus GA</t>
+        </is>
+      </c>
+      <c r="K1343" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1343" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr">
+        <is>
+          <t>Livingston Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>livingston-air.com</t>
+        </is>
+      </c>
+      <c r="D1344" t="inlineStr">
+        <is>
+          <t>https://livingston-air.com/hvac-services-in-columbus-georgia/</t>
+        </is>
+      </c>
+      <c r="E1344" t="inlineStr"/>
+      <c r="F1344" t="inlineStr">
+        <is>
+          <t>info@livingston-air.com</t>
+        </is>
+      </c>
+      <c r="G1344" t="inlineStr">
+        <is>
+          <t>334-297-7863</t>
+        </is>
+      </c>
+      <c r="H1344" t="inlineStr">
+        <is>
+          <t>Columbus GA</t>
+        </is>
+      </c>
+      <c r="I1344" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1344" t="inlineStr">
+        <is>
+          <t>furnace repair Columbus GA</t>
+        </is>
+      </c>
+      <c r="K1344" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1344" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="inlineStr">
+        <is>
+          <t>Mr. GoodRoof</t>
+        </is>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>mrgoodroof.com</t>
+        </is>
+      </c>
+      <c r="D1345" t="inlineStr">
+        <is>
+          <t>https://mrgoodroof.com/nashville-tn/</t>
+        </is>
+      </c>
+      <c r="E1345" t="inlineStr">
+        <is>
+          <t>Locally Owned</t>
+        </is>
+      </c>
+      <c r="F1345" t="inlineStr">
+        <is>
+          <t>contactus@mrgoodroof.com</t>
+        </is>
+      </c>
+      <c r="G1345" t="inlineStr">
+        <is>
+          <t>(615) 824-8100</t>
+        </is>
+      </c>
+      <c r="H1345" t="inlineStr">
+        <is>
+          <t>Nashville TN</t>
+        </is>
+      </c>
+      <c r="I1345" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1345" t="inlineStr">
+        <is>
+          <t>roof replacement Nashville TN</t>
+        </is>
+      </c>
+      <c r="K1345" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1345" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="inlineStr">
+        <is>
+          <t>DNA Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>dnahvac.com</t>
+        </is>
+      </c>
+      <c r="D1346" t="inlineStr">
+        <is>
+          <t>https://www.dnahvac.com/locations/columbus-ga/furnace-repair-columbus/</t>
+        </is>
+      </c>
+      <c r="E1346" t="inlineStr"/>
+      <c r="F1346" t="inlineStr">
+        <is>
+          <t>service@dnahvac.com</t>
+        </is>
+      </c>
+      <c r="G1346" t="inlineStr">
+        <is>
+          <t>(706) 349-1414</t>
+        </is>
+      </c>
+      <c r="H1346" t="inlineStr">
+        <is>
+          <t>Columbus GA</t>
+        </is>
+      </c>
+      <c r="I1346" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1346" t="inlineStr">
+        <is>
+          <t>furnace repair Columbus GA</t>
+        </is>
+      </c>
+      <c r="K1346" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1346" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="inlineStr">
+        <is>
+          <t>Nashville Roofing Company</t>
+        </is>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr">
+        <is>
+          <t>nashvilleroofingco.com</t>
+        </is>
+      </c>
+      <c r="D1347" t="inlineStr">
+        <is>
+          <t>https://nashvilleroofingco.com/</t>
+        </is>
+      </c>
+      <c r="E1347" t="inlineStr">
+        <is>
+          <t>Middle Tenn</t>
+        </is>
+      </c>
+      <c r="F1347" t="inlineStr">
+        <is>
+          <t>info@nashvilleroofingco.com</t>
+        </is>
+      </c>
+      <c r="G1347" t="inlineStr">
+        <is>
+          <t>615.800.4355</t>
+        </is>
+      </c>
+      <c r="H1347" t="inlineStr">
+        <is>
+          <t>Nashville TN</t>
+        </is>
+      </c>
+      <c r="I1347" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1347" t="inlineStr">
+        <is>
+          <t>roof replacement Nashville TN</t>
+        </is>
+      </c>
+      <c r="K1347" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1347" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 21:58 UTC (cycle 145)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1347"/>
+  <dimension ref="A1:L1349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -78985,7 +78985,6 @@
           <t>https://energysaversair.com/columbus-ga/hvac/furnace-repair/</t>
         </is>
       </c>
-      <c r="E1342" t="inlineStr"/>
       <c r="F1342" t="inlineStr">
         <is>
           <t>customerservice@energysaversair.com</t>
@@ -79101,7 +79100,6 @@
           <t>https://livingston-air.com/hvac-services-in-columbus-georgia/</t>
         </is>
       </c>
-      <c r="E1344" t="inlineStr"/>
       <c r="F1344" t="inlineStr">
         <is>
           <t>info@livingston-air.com</t>
@@ -79217,7 +79215,6 @@
           <t>https://www.dnahvac.com/locations/columbus-ga/furnace-repair-columbus/</t>
         </is>
       </c>
-      <c r="E1346" t="inlineStr"/>
       <c r="F1346" t="inlineStr">
         <is>
           <t>service@dnahvac.com</t>
@@ -79307,6 +79304,126 @@
         </is>
       </c>
       <c r="L1347" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="inlineStr">
+        <is>
+          <t>Air Conditioning Services in Thornton</t>
+        </is>
+      </c>
+      <c r="B1348" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1348" t="inlineStr">
+        <is>
+          <t>mojoyourhomes.com</t>
+        </is>
+      </c>
+      <c r="D1348" t="inlineStr">
+        <is>
+          <t>https://mojoyourhomes.com/air-conditioning-services/thornton-co</t>
+        </is>
+      </c>
+      <c r="E1348" t="inlineStr">
+        <is>
+          <t>Homeowners Served</t>
+        </is>
+      </c>
+      <c r="F1348" t="inlineStr">
+        <is>
+          <t>support@mojoyourhomes.com</t>
+        </is>
+      </c>
+      <c r="G1348" t="inlineStr">
+        <is>
+          <t>720-807-4050</t>
+        </is>
+      </c>
+      <c r="H1348" t="inlineStr">
+        <is>
+          <t>Thornton CO</t>
+        </is>
+      </c>
+      <c r="I1348" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1348" t="inlineStr">
+        <is>
+          <t>air conditioning repair Thornton CO</t>
+        </is>
+      </c>
+      <c r="K1348" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1348" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="inlineStr">
+        <is>
+          <t>Castillo Roofing Main Site</t>
+        </is>
+      </c>
+      <c r="B1349" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1349" t="inlineStr">
+        <is>
+          <t>castillotx.com</t>
+        </is>
+      </c>
+      <c r="D1349" t="inlineStr">
+        <is>
+          <t>https://castillotx.com/mcallen/</t>
+        </is>
+      </c>
+      <c r="E1349" t="inlineStr">
+        <is>
+          <t>Gold Standard</t>
+        </is>
+      </c>
+      <c r="F1349" t="inlineStr">
+        <is>
+          <t>info@castillotx.com</t>
+        </is>
+      </c>
+      <c r="G1349" t="inlineStr">
+        <is>
+          <t>(956) 264-5251</t>
+        </is>
+      </c>
+      <c r="H1349" t="inlineStr">
+        <is>
+          <t>McAllen TX</t>
+        </is>
+      </c>
+      <c r="I1349" t="n">
+        <v>96</v>
+      </c>
+      <c r="J1349" t="inlineStr">
+        <is>
+          <t>roof replacement McAllen TX</t>
+        </is>
+      </c>
+      <c r="K1349" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1349" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 21:59 UTC (cycle 146)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1349"/>
+  <dimension ref="A1:L1353"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -79429,6 +79429,238 @@
         </is>
       </c>
     </row>
+    <row r="1350">
+      <c r="A1350" t="inlineStr">
+        <is>
+          <t>D&amp;D Home Services</t>
+        </is>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>danddmidland.com</t>
+        </is>
+      </c>
+      <c r="D1350" t="inlineStr">
+        <is>
+          <t>https://danddmidland.com/hvac-services-midland-odessa-tx</t>
+        </is>
+      </c>
+      <c r="E1350" t="inlineStr">
+        <is>
+          <t>Schedule Service</t>
+        </is>
+      </c>
+      <c r="F1350" t="inlineStr">
+        <is>
+          <t>service@danddmidland.com</t>
+        </is>
+      </c>
+      <c r="G1350" t="inlineStr">
+        <is>
+          <t>(432) 687-1011</t>
+        </is>
+      </c>
+      <c r="H1350" t="inlineStr">
+        <is>
+          <t>Odessa TX</t>
+        </is>
+      </c>
+      <c r="I1350" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1350" t="inlineStr">
+        <is>
+          <t>furnace repair Odessa TX</t>
+        </is>
+      </c>
+      <c r="K1350" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1350" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="inlineStr">
+        <is>
+          <t>Redhawk AC</t>
+        </is>
+      </c>
+      <c r="B1351" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1351" t="inlineStr">
+        <is>
+          <t>redhawkac.com</t>
+        </is>
+      </c>
+      <c r="D1351" t="inlineStr">
+        <is>
+          <t>https://www.redhawkac.com/furnaces/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E1351" t="inlineStr"/>
+      <c r="F1351" t="inlineStr">
+        <is>
+          <t>redhawk@pbol.net</t>
+        </is>
+      </c>
+      <c r="G1351" t="inlineStr">
+        <is>
+          <t>432-289-6309</t>
+        </is>
+      </c>
+      <c r="H1351" t="inlineStr">
+        <is>
+          <t>Odessa TX</t>
+        </is>
+      </c>
+      <c r="I1351" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1351" t="inlineStr">
+        <is>
+          <t>furnace repair Odessa TX</t>
+        </is>
+      </c>
+      <c r="K1351" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1351" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="inlineStr">
+        <is>
+          <t>AC Installation &amp; Repair | Tom Torrance Erie PA</t>
+        </is>
+      </c>
+      <c r="B1352" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1352" t="inlineStr">
+        <is>
+          <t>tomtorranceheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="D1352" t="inlineStr">
+        <is>
+          <t>https://www.tomtorranceheatingcooling.com/hvac-services/air-conditioning</t>
+        </is>
+      </c>
+      <c r="E1352" t="inlineStr"/>
+      <c r="F1352" t="inlineStr">
+        <is>
+          <t>info@tomtorranceheatingcooling.com</t>
+        </is>
+      </c>
+      <c r="G1352" t="inlineStr">
+        <is>
+          <t>814-825-7066</t>
+        </is>
+      </c>
+      <c r="H1352" t="inlineStr">
+        <is>
+          <t>Erie PA</t>
+        </is>
+      </c>
+      <c r="I1352" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1352" t="inlineStr">
+        <is>
+          <t>AC installation Erie PA</t>
+        </is>
+      </c>
+      <c r="K1352" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1352" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="inlineStr">
+        <is>
+          <t>Mega Care Solutions</t>
+        </is>
+      </c>
+      <c r="B1353" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1353" t="inlineStr">
+        <is>
+          <t>megacaresolutions.com</t>
+        </is>
+      </c>
+      <c r="D1353" t="inlineStr">
+        <is>
+          <t>https://www.megacaresolutions.com/</t>
+        </is>
+      </c>
+      <c r="E1353" t="inlineStr">
+        <is>
+          <t>Air Conditioning</t>
+        </is>
+      </c>
+      <c r="F1353" t="inlineStr">
+        <is>
+          <t>megaaircond@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1353" t="inlineStr">
+        <is>
+          <t>(432) 580-6342</t>
+        </is>
+      </c>
+      <c r="H1353" t="inlineStr">
+        <is>
+          <t>Odessa TX</t>
+        </is>
+      </c>
+      <c r="I1353" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1353" t="inlineStr">
+        <is>
+          <t>furnace repair Odessa TX</t>
+        </is>
+      </c>
+      <c r="K1353" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1353" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:02 UTC (cycle 148)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1353"/>
+  <dimension ref="A1:L1354"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -79510,7 +79510,6 @@
           <t>https://www.redhawkac.com/furnaces/furnace-repair/</t>
         </is>
       </c>
-      <c r="E1351" t="inlineStr"/>
       <c r="F1351" t="inlineStr">
         <is>
           <t>redhawk@pbol.net</t>
@@ -79566,7 +79565,6 @@
           <t>https://www.tomtorranceheatingcooling.com/hvac-services/air-conditioning</t>
         </is>
       </c>
-      <c r="E1352" t="inlineStr"/>
       <c r="F1352" t="inlineStr">
         <is>
           <t>info@tomtorranceheatingcooling.com</t>
@@ -79656,6 +79654,66 @@
         </is>
       </c>
       <c r="L1353" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="inlineStr">
+        <is>
+          <t>I &amp; M Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B1354" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1354" t="inlineStr">
+        <is>
+          <t>iandmhvac.com</t>
+        </is>
+      </c>
+      <c r="D1354" t="inlineStr">
+        <is>
+          <t>https://www.iandmhvac.com/</t>
+        </is>
+      </c>
+      <c r="E1354" t="inlineStr">
+        <is>
+          <t>Cooling Jeff</t>
+        </is>
+      </c>
+      <c r="F1354" t="inlineStr">
+        <is>
+          <t>info@iandmhvac.com</t>
+        </is>
+      </c>
+      <c r="G1354" t="inlineStr">
+        <is>
+          <t>574 288 3351</t>
+        </is>
+      </c>
+      <c r="H1354" t="inlineStr">
+        <is>
+          <t>South Bend IN</t>
+        </is>
+      </c>
+      <c r="I1354" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1354" t="inlineStr">
+        <is>
+          <t>AC installation South Bend IN</t>
+        </is>
+      </c>
+      <c r="K1354" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1354" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:04 UTC (cycle 149)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1354"/>
+  <dimension ref="A1:L1357"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -79719,6 +79719,186 @@
         </is>
       </c>
     </row>
+    <row r="1355">
+      <c r="A1355" t="inlineStr">
+        <is>
+          <t>Rhino Roofer</t>
+        </is>
+      </c>
+      <c r="B1355" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1355" t="inlineStr">
+        <is>
+          <t>rhinoroofer.com</t>
+        </is>
+      </c>
+      <c r="D1355" t="inlineStr">
+        <is>
+          <t>https://rhinoroofer.com/</t>
+        </is>
+      </c>
+      <c r="E1355" t="inlineStr">
+        <is>
+          <t>Ryan Nelson</t>
+        </is>
+      </c>
+      <c r="F1355" t="inlineStr">
+        <is>
+          <t>sales@rhinoroofer.com</t>
+        </is>
+      </c>
+      <c r="G1355" t="inlineStr">
+        <is>
+          <t>218-724-7663</t>
+        </is>
+      </c>
+      <c r="H1355" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I1355" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1355" t="inlineStr">
+        <is>
+          <t>roofer Duluth MN</t>
+        </is>
+      </c>
+      <c r="K1355" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1355" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" t="inlineStr">
+        <is>
+          <t>Roofers Duluth</t>
+        </is>
+      </c>
+      <c r="B1356" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1356" t="inlineStr">
+        <is>
+          <t>roofersduluth.com</t>
+        </is>
+      </c>
+      <c r="D1356" t="inlineStr">
+        <is>
+          <t>https://roofersduluth.com/</t>
+        </is>
+      </c>
+      <c r="E1356" t="inlineStr">
+        <is>
+          <t>Serving Our</t>
+        </is>
+      </c>
+      <c r="F1356" t="inlineStr">
+        <is>
+          <t>julie@perraultconstruction.com</t>
+        </is>
+      </c>
+      <c r="G1356" t="inlineStr">
+        <is>
+          <t>(218)-522-8993</t>
+        </is>
+      </c>
+      <c r="H1356" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I1356" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1356" t="inlineStr">
+        <is>
+          <t>roofer Duluth MN</t>
+        </is>
+      </c>
+      <c r="K1356" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1356" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" t="inlineStr">
+        <is>
+          <t>Empire Roofing</t>
+        </is>
+      </c>
+      <c r="B1357" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1357" t="inlineStr">
+        <is>
+          <t>empireroofingmn.com</t>
+        </is>
+      </c>
+      <c r="D1357" t="inlineStr">
+        <is>
+          <t>https://empireroofingmn.com/</t>
+        </is>
+      </c>
+      <c r="E1357" t="inlineStr">
+        <is>
+          <t>Star Reviews</t>
+        </is>
+      </c>
+      <c r="F1357" t="inlineStr">
+        <is>
+          <t>info@empireroofingmn.com</t>
+        </is>
+      </c>
+      <c r="G1357" t="inlineStr">
+        <is>
+          <t>218-724-5584</t>
+        </is>
+      </c>
+      <c r="H1357" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I1357" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1357" t="inlineStr">
+        <is>
+          <t>roofer Duluth MN</t>
+        </is>
+      </c>
+      <c r="K1357" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1357" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:05 UTC (cycle 150)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1357"/>
+  <dimension ref="A1:L1361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -79899,6 +79899,238 @@
         </is>
       </c>
     </row>
+    <row r="1358">
+      <c r="A1358" t="inlineStr">
+        <is>
+          <t>Anytime Heating And Cooling</t>
+        </is>
+      </c>
+      <c r="B1358" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1358" t="inlineStr">
+        <is>
+          <t>hvacanytime.com</t>
+        </is>
+      </c>
+      <c r="D1358" t="inlineStr">
+        <is>
+          <t>https://hvacanytime.com/sterling-heights/</t>
+        </is>
+      </c>
+      <c r="E1358" t="inlineStr">
+        <is>
+          <t>Sterling Heights</t>
+        </is>
+      </c>
+      <c r="F1358" t="inlineStr">
+        <is>
+          <t>anytimehvac1@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1358" t="inlineStr">
+        <is>
+          <t>(586) 486-5766</t>
+        </is>
+      </c>
+      <c r="H1358" t="inlineStr">
+        <is>
+          <t>Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="I1358" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1358" t="inlineStr">
+        <is>
+          <t>furnace repair Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="K1358" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1358" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="inlineStr">
+        <is>
+          <t>Jordan Air, Heating, Plumbing, &amp; Electric</t>
+        </is>
+      </c>
+      <c r="B1359" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1359" t="inlineStr">
+        <is>
+          <t>jordanairinc.com</t>
+        </is>
+      </c>
+      <c r="D1359" t="inlineStr">
+        <is>
+          <t>https://jordanairinc.com/hvac-services/ac-installation-and-replacement/</t>
+        </is>
+      </c>
+      <c r="E1359" t="inlineStr"/>
+      <c r="F1359" t="inlineStr">
+        <is>
+          <t>nonemergencybooking@jordanairinc.com</t>
+        </is>
+      </c>
+      <c r="G1359" t="inlineStr">
+        <is>
+          <t>(706) 807-2309</t>
+        </is>
+      </c>
+      <c r="H1359" t="inlineStr">
+        <is>
+          <t>Athens GA</t>
+        </is>
+      </c>
+      <c r="I1359" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1359" t="inlineStr">
+        <is>
+          <t>AC installation Athens GA</t>
+        </is>
+      </c>
+      <c r="K1359" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1359" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" t="inlineStr">
+        <is>
+          <t>Repair - Sterling Heights, MI</t>
+        </is>
+      </c>
+      <c r="B1360" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1360" t="inlineStr">
+        <is>
+          <t>briarwoodheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D1360" t="inlineStr">
+        <is>
+          <t>https://www.briarwoodheatingandcooling.com/furnace-repair-sterling-heights</t>
+        </is>
+      </c>
+      <c r="E1360" t="inlineStr">
+        <is>
+          <t>Sterling Heights</t>
+        </is>
+      </c>
+      <c r="F1360" t="inlineStr">
+        <is>
+          <t>briarwoodheatingcooling@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1360" t="inlineStr">
+        <is>
+          <t>248-299-8126</t>
+        </is>
+      </c>
+      <c r="H1360" t="inlineStr">
+        <is>
+          <t>Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="I1360" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1360" t="inlineStr">
+        <is>
+          <t>furnace repair Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="K1360" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1360" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="inlineStr">
+        <is>
+          <t>Sterling Heights, Mi Furnace Repair, 24 Hour Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B1361" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1361" t="inlineStr">
+        <is>
+          <t>serenecomfort.net</t>
+        </is>
+      </c>
+      <c r="D1361" t="inlineStr">
+        <is>
+          <t>https://serenecomfort.net/Mi_SterlingHeightsHeatingCoolingFurnaceRepair.html</t>
+        </is>
+      </c>
+      <c r="E1361" t="inlineStr"/>
+      <c r="F1361" t="inlineStr">
+        <is>
+          <t>serene.comfort@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G1361" t="inlineStr">
+        <is>
+          <t>(248)765-1714</t>
+        </is>
+      </c>
+      <c r="H1361" t="inlineStr">
+        <is>
+          <t>Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="I1361" t="n">
+        <v>64</v>
+      </c>
+      <c r="J1361" t="inlineStr">
+        <is>
+          <t>furnace repair Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="K1361" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1361" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:07 UTC (cycle 151)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1361"/>
+  <dimension ref="A1:L1364"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -79980,7 +79980,6 @@
           <t>https://jordanairinc.com/hvac-services/ac-installation-and-replacement/</t>
         </is>
       </c>
-      <c r="E1359" t="inlineStr"/>
       <c r="F1359" t="inlineStr">
         <is>
           <t>nonemergencybooking@jordanairinc.com</t>
@@ -80096,7 +80095,6 @@
           <t>https://serenecomfort.net/Mi_SterlingHeightsHeatingCoolingFurnaceRepair.html</t>
         </is>
       </c>
-      <c r="E1361" t="inlineStr"/>
       <c r="F1361" t="inlineStr">
         <is>
           <t>serene.comfort@yahoo.com</t>
@@ -80126,6 +80124,186 @@
         </is>
       </c>
       <c r="L1361" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="inlineStr">
+        <is>
+          <t>Driftwood Builders Roofing - Your Austin Roofing Expert</t>
+        </is>
+      </c>
+      <c r="B1362" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1362" t="inlineStr">
+        <is>
+          <t>driftwoodbuildersroofing.com</t>
+        </is>
+      </c>
+      <c r="D1362" t="inlineStr">
+        <is>
+          <t>https://driftwoodbuildersroofing.com/roofing-company-in-san-marcos-tx/</t>
+        </is>
+      </c>
+      <c r="E1362" t="inlineStr">
+        <is>
+          <t>Trusted Roofing</t>
+        </is>
+      </c>
+      <c r="F1362" t="inlineStr">
+        <is>
+          <t>driftwoodbuilders@driftwoodbuilders.net</t>
+        </is>
+      </c>
+      <c r="G1362" t="inlineStr">
+        <is>
+          <t>512-894-0129</t>
+        </is>
+      </c>
+      <c r="H1362" t="inlineStr">
+        <is>
+          <t>San Marcos TX</t>
+        </is>
+      </c>
+      <c r="I1362" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1362" t="inlineStr">
+        <is>
+          <t>roofer San Marcos TX</t>
+        </is>
+      </c>
+      <c r="K1362" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1362" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" t="inlineStr">
+        <is>
+          <t>Sutton Roofing</t>
+        </is>
+      </c>
+      <c r="B1363" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1363" t="inlineStr">
+        <is>
+          <t>suttonroofinginc.com</t>
+        </is>
+      </c>
+      <c r="D1363" t="inlineStr">
+        <is>
+          <t>https://www.suttonroofinginc.com/service-areas-san-marcos-tx</t>
+        </is>
+      </c>
+      <c r="E1363" t="inlineStr">
+        <is>
+          <t>Accredited Trusted</t>
+        </is>
+      </c>
+      <c r="F1363" t="inlineStr">
+        <is>
+          <t>suttonroofinginc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1363" t="inlineStr">
+        <is>
+          <t>(512) 394-9801</t>
+        </is>
+      </c>
+      <c r="H1363" t="inlineStr">
+        <is>
+          <t>San Marcos TX</t>
+        </is>
+      </c>
+      <c r="I1363" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1363" t="inlineStr">
+        <is>
+          <t>roofer San Marcos TX</t>
+        </is>
+      </c>
+      <c r="K1363" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1363" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="inlineStr">
+        <is>
+          <t>Gotta Go Plumbing</t>
+        </is>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>gottagoplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1364" t="inlineStr">
+        <is>
+          <t>https://gottagoplumbing.com/services/water-heater-service/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E1364" t="inlineStr">
+        <is>
+          <t>Owensboro With</t>
+        </is>
+      </c>
+      <c r="F1364" t="inlineStr">
+        <is>
+          <t>service@gottagoplumbing.com</t>
+        </is>
+      </c>
+      <c r="G1364" t="inlineStr">
+        <is>
+          <t>270-238-5752</t>
+        </is>
+      </c>
+      <c r="H1364" t="inlineStr">
+        <is>
+          <t>Owensboro KY</t>
+        </is>
+      </c>
+      <c r="I1364" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1364" t="inlineStr">
+        <is>
+          <t>water heater repair Owensboro KY</t>
+        </is>
+      </c>
+      <c r="K1364" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1364" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:10 UTC (cycle 153)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1364"/>
+  <dimension ref="A1:L1365"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -80309,6 +80309,66 @@
         </is>
       </c>
     </row>
+    <row r="1365">
+      <c r="A1365" t="inlineStr">
+        <is>
+          <t>Roofers Wilmington DE | Wilmington Roofing Contractor</t>
+        </is>
+      </c>
+      <c r="B1365" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1365" t="inlineStr">
+        <is>
+          <t>roofingwilmingtonde.com</t>
+        </is>
+      </c>
+      <c r="D1365" t="inlineStr">
+        <is>
+          <t>https://roofingwilmingtonde.com/</t>
+        </is>
+      </c>
+      <c r="E1365" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F1365" t="inlineStr">
+        <is>
+          <t>support@roofingwilmingtonde.com</t>
+        </is>
+      </c>
+      <c r="G1365" t="inlineStr">
+        <is>
+          <t>(302) 618-1471</t>
+        </is>
+      </c>
+      <c r="H1365" t="inlineStr">
+        <is>
+          <t>Wilmington DE</t>
+        </is>
+      </c>
+      <c r="I1365" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1365" t="inlineStr">
+        <is>
+          <t>roofing contractor Wilmington DE</t>
+        </is>
+      </c>
+      <c r="K1365" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1365" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:11 UTC (cycle 154)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1365"/>
+  <dimension ref="A1:L1366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -80369,6 +80369,62 @@
         </is>
       </c>
     </row>
+    <row r="1366">
+      <c r="A1366" t="inlineStr">
+        <is>
+          <t>Herman Plumbing Co., Inc.</t>
+        </is>
+      </c>
+      <c r="B1366" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1366" t="inlineStr">
+        <is>
+          <t>hermanplumbing.net</t>
+        </is>
+      </c>
+      <c r="D1366" t="inlineStr">
+        <is>
+          <t>https://hermanplumbing.net/</t>
+        </is>
+      </c>
+      <c r="E1366" t="inlineStr"/>
+      <c r="F1366" t="inlineStr">
+        <is>
+          <t>office@herman-plumbing.com</t>
+        </is>
+      </c>
+      <c r="G1366" t="inlineStr">
+        <is>
+          <t>308-382-3760</t>
+        </is>
+      </c>
+      <c r="H1366" t="inlineStr">
+        <is>
+          <t>Grand Island NE</t>
+        </is>
+      </c>
+      <c r="I1366" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1366" t="inlineStr">
+        <is>
+          <t>plumber Grand Island NE</t>
+        </is>
+      </c>
+      <c r="K1366" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1366" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:14 UTC (cycle 156)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1366"/>
+  <dimension ref="A1:L1374"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -80390,7 +80390,6 @@
           <t>https://hermanplumbing.net/</t>
         </is>
       </c>
-      <c r="E1366" t="inlineStr"/>
       <c r="F1366" t="inlineStr">
         <is>
           <t>office@herman-plumbing.com</t>
@@ -80420,6 +80419,478 @@
         </is>
       </c>
       <c r="L1366" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="inlineStr">
+        <is>
+          <t>Plumbing Company Florida</t>
+        </is>
+      </c>
+      <c r="B1367" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1367" t="inlineStr">
+        <is>
+          <t>clearwater.plumbingcompanyflorida.com</t>
+        </is>
+      </c>
+      <c r="D1367" t="inlineStr">
+        <is>
+          <t>https://clearwater.plumbingcompanyflorida.com/</t>
+        </is>
+      </c>
+      <c r="E1367" t="inlineStr"/>
+      <c r="F1367" t="inlineStr">
+        <is>
+          <t>dispatch@plumbingcompanyflorida.com</t>
+        </is>
+      </c>
+      <c r="G1367" t="inlineStr">
+        <is>
+          <t>407-598-8903</t>
+        </is>
+      </c>
+      <c r="H1367" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I1367" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1367" t="inlineStr">
+        <is>
+          <t>emergency plumber Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K1367" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1367" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="inlineStr">
+        <is>
+          <t>Roofing Company in Bismarck, ND - Serving North Dakota</t>
+        </is>
+      </c>
+      <c r="B1368" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1368" t="inlineStr">
+        <is>
+          <t>highqualitynd.com</t>
+        </is>
+      </c>
+      <c r="D1368" t="inlineStr">
+        <is>
+          <t>https://www.highqualitynd.com/</t>
+        </is>
+      </c>
+      <c r="E1368" t="inlineStr">
+        <is>
+          <t>Services North</t>
+        </is>
+      </c>
+      <c r="F1368" t="inlineStr">
+        <is>
+          <t>hqllc2017@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1368" t="inlineStr">
+        <is>
+          <t>701-299-0462</t>
+        </is>
+      </c>
+      <c r="H1368" t="inlineStr">
+        <is>
+          <t>Bismarck ND</t>
+        </is>
+      </c>
+      <c r="I1368" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1368" t="inlineStr">
+        <is>
+          <t>residential roofing company Bismarck ND</t>
+        </is>
+      </c>
+      <c r="K1368" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1368" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="inlineStr">
+        <is>
+          <t>5 Star Roofing and Contracting</t>
+        </is>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>5starroofingandcontracting.com</t>
+        </is>
+      </c>
+      <c r="D1369" t="inlineStr">
+        <is>
+          <t>https://5starroofingandcontracting.com/roofing/bismarck-nd/</t>
+        </is>
+      </c>
+      <c r="E1369" t="inlineStr">
+        <is>
+          <t>Read Posted</t>
+        </is>
+      </c>
+      <c r="F1369" t="inlineStr">
+        <is>
+          <t>5starroofingandcontracting@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1369" t="inlineStr">
+        <is>
+          <t>(701) 290-2916</t>
+        </is>
+      </c>
+      <c r="H1369" t="inlineStr">
+        <is>
+          <t>Bismarck ND</t>
+        </is>
+      </c>
+      <c r="I1369" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1369" t="inlineStr">
+        <is>
+          <t>residential roofing company Bismarck ND</t>
+        </is>
+      </c>
+      <c r="K1369" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1369" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="inlineStr">
+        <is>
+          <t>Lukas Plumbing &amp; Leak Detection</t>
+        </is>
+      </c>
+      <c r="B1370" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1370" t="inlineStr">
+        <is>
+          <t>lukasleakdetection.com</t>
+        </is>
+      </c>
+      <c r="D1370" t="inlineStr">
+        <is>
+          <t>https://www.lukasleakdetection.com/services/emergency-plumbing/clearwater/</t>
+        </is>
+      </c>
+      <c r="E1370" t="inlineStr">
+        <is>
+          <t>Pinellas County</t>
+        </is>
+      </c>
+      <c r="F1370" t="inlineStr">
+        <is>
+          <t>contact@lukasleakdetection.com</t>
+        </is>
+      </c>
+      <c r="G1370" t="inlineStr">
+        <is>
+          <t>(727) 666-5334</t>
+        </is>
+      </c>
+      <c r="H1370" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I1370" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1370" t="inlineStr">
+        <is>
+          <t>emergency plumber Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K1370" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1370" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="inlineStr">
+        <is>
+          <t>Apex Plumbing</t>
+        </is>
+      </c>
+      <c r="B1371" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1371" t="inlineStr">
+        <is>
+          <t>apexdoyourplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1371" t="inlineStr">
+        <is>
+          <t>https://apexdoyourplumbing.com/emergency-plumber-clearwater-fl/</t>
+        </is>
+      </c>
+      <c r="E1371" t="inlineStr">
+        <is>
+          <t>Drain Cleaning</t>
+        </is>
+      </c>
+      <c r="F1371" t="inlineStr">
+        <is>
+          <t>alex@apex-plumbing.net</t>
+        </is>
+      </c>
+      <c r="G1371" t="inlineStr">
+        <is>
+          <t>(727) 285-8559</t>
+        </is>
+      </c>
+      <c r="H1371" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I1371" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1371" t="inlineStr">
+        <is>
+          <t>emergency plumber Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K1371" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1371" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="inlineStr">
+        <is>
+          <t>JKC Plumbing</t>
+        </is>
+      </c>
+      <c r="B1372" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1372" t="inlineStr">
+        <is>
+          <t>jkcplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1372" t="inlineStr">
+        <is>
+          <t>https://jkcplumbing.com/flint-plumbing/</t>
+        </is>
+      </c>
+      <c r="E1372" t="inlineStr"/>
+      <c r="F1372" t="inlineStr">
+        <is>
+          <t>info@jkcplumbing.com</t>
+        </is>
+      </c>
+      <c r="G1372" t="inlineStr">
+        <is>
+          <t>(517) 458-8097</t>
+        </is>
+      </c>
+      <c r="H1372" t="inlineStr">
+        <is>
+          <t>Flint MI</t>
+        </is>
+      </c>
+      <c r="I1372" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1372" t="inlineStr">
+        <is>
+          <t>emergency plumber Flint MI</t>
+        </is>
+      </c>
+      <c r="K1372" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1372" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="inlineStr">
+        <is>
+          <t>Tampa Bay Plumbing | Best Plumbers in Tampa I Emergency Services</t>
+        </is>
+      </c>
+      <c r="B1373" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1373" t="inlineStr">
+        <is>
+          <t>tampabayplumber.com</t>
+        </is>
+      </c>
+      <c r="D1373" t="inlineStr">
+        <is>
+          <t>https://tampabayplumber.com/</t>
+        </is>
+      </c>
+      <c r="E1373" t="inlineStr">
+        <is>
+          <t>Commercial Plumbing</t>
+        </is>
+      </c>
+      <c r="F1373" t="inlineStr">
+        <is>
+          <t>services@tampabayplumber.com</t>
+        </is>
+      </c>
+      <c r="G1373" t="inlineStr">
+        <is>
+          <t>(727) 223-6400</t>
+        </is>
+      </c>
+      <c r="H1373" t="inlineStr">
+        <is>
+          <t>Clearwater FL</t>
+        </is>
+      </c>
+      <c r="I1373" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1373" t="inlineStr">
+        <is>
+          <t>emergency plumber Clearwater FL</t>
+        </is>
+      </c>
+      <c r="K1373" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1373" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="inlineStr">
+        <is>
+          <t>Emergency Plumber Flint</t>
+        </is>
+      </c>
+      <c r="B1374" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1374" t="inlineStr">
+        <is>
+          <t>canflowplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1374" t="inlineStr">
+        <is>
+          <t>https://canflowplumbing.com/emergency-plumber-flint-mi/</t>
+        </is>
+      </c>
+      <c r="E1374" t="inlineStr">
+        <is>
+          <t>Why Flint</t>
+        </is>
+      </c>
+      <c r="F1374" t="inlineStr">
+        <is>
+          <t>info@canflowplumbing.com</t>
+        </is>
+      </c>
+      <c r="G1374" t="inlineStr">
+        <is>
+          <t>(888) 698-5660</t>
+        </is>
+      </c>
+      <c r="H1374" t="inlineStr">
+        <is>
+          <t>Flint MI</t>
+        </is>
+      </c>
+      <c r="I1374" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1374" t="inlineStr">
+        <is>
+          <t>emergency plumber Flint MI</t>
+        </is>
+      </c>
+      <c r="K1374" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1374" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:17 UTC (cycle 158)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1374"/>
+  <dimension ref="A1:L1375"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -80445,7 +80445,6 @@
           <t>https://clearwater.plumbingcompanyflorida.com/</t>
         </is>
       </c>
-      <c r="E1367" t="inlineStr"/>
       <c r="F1367" t="inlineStr">
         <is>
           <t>dispatch@plumbingcompanyflorida.com</t>
@@ -80741,7 +80740,6 @@
           <t>https://jkcplumbing.com/flint-plumbing/</t>
         </is>
       </c>
-      <c r="E1372" t="inlineStr"/>
       <c r="F1372" t="inlineStr">
         <is>
           <t>info@jkcplumbing.com</t>
@@ -80891,6 +80889,66 @@
         </is>
       </c>
       <c r="L1374" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="inlineStr">
+        <is>
+          <t>East Atlantic Plumbing LLC |</t>
+        </is>
+      </c>
+      <c r="B1375" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1375" t="inlineStr">
+        <is>
+          <t>eastatlanticplumbing.net</t>
+        </is>
+      </c>
+      <c r="D1375" t="inlineStr">
+        <is>
+          <t>https://eastatlanticplumbing.net/residential-plumbing-wilmington-nc/plumbing-repairs/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E1375" t="inlineStr">
+        <is>
+          <t>North Carolina</t>
+        </is>
+      </c>
+      <c r="F1375" t="inlineStr">
+        <is>
+          <t>frantheplumber@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1375" t="inlineStr">
+        <is>
+          <t>(910) 616-3238</t>
+        </is>
+      </c>
+      <c r="H1375" t="inlineStr">
+        <is>
+          <t>Wilmington NC</t>
+        </is>
+      </c>
+      <c r="I1375" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1375" t="inlineStr">
+        <is>
+          <t>water heater repair Wilmington NC</t>
+        </is>
+      </c>
+      <c r="K1375" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1375" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:19 UTC (cycle 159)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1375"/>
+  <dimension ref="A1:L1379"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -80954,6 +80954,246 @@
         </is>
       </c>
     </row>
+    <row r="1376">
+      <c r="A1376" t="inlineStr">
+        <is>
+          <t>All Toasty Heating &amp; AC, LLC</t>
+        </is>
+      </c>
+      <c r="B1376" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1376" t="inlineStr">
+        <is>
+          <t>alltoastyheatingandac.com</t>
+        </is>
+      </c>
+      <c r="D1376" t="inlineStr">
+        <is>
+          <t>https://www.alltoastyheatingandac.com/areas-we-serve/oxnard-ca/</t>
+        </is>
+      </c>
+      <c r="E1376" t="inlineStr">
+        <is>
+          <t>At All</t>
+        </is>
+      </c>
+      <c r="F1376" t="inlineStr">
+        <is>
+          <t>johnsmith@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1376" t="inlineStr">
+        <is>
+          <t>(805) 482-3457</t>
+        </is>
+      </c>
+      <c r="H1376" t="inlineStr">
+        <is>
+          <t>Oxnard CA</t>
+        </is>
+      </c>
+      <c r="I1376" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1376" t="inlineStr">
+        <is>
+          <t>air conditioning repair Oxnard CA</t>
+        </is>
+      </c>
+      <c r="K1376" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1376" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="inlineStr">
+        <is>
+          <t>HVAC Services in Oxnard, CA | Simon Air Conditioning &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B1377" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1377" t="inlineStr">
+        <is>
+          <t>simon-air.com</t>
+        </is>
+      </c>
+      <c r="D1377" t="inlineStr">
+        <is>
+          <t>https://simon-air.com/cities/oxnard.html</t>
+        </is>
+      </c>
+      <c r="E1377" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F1377" t="inlineStr">
+        <is>
+          <t>info@simon-air.com</t>
+        </is>
+      </c>
+      <c r="G1377" t="inlineStr">
+        <is>
+          <t>818-929-0299</t>
+        </is>
+      </c>
+      <c r="H1377" t="inlineStr">
+        <is>
+          <t>Oxnard CA</t>
+        </is>
+      </c>
+      <c r="I1377" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1377" t="inlineStr">
+        <is>
+          <t>air conditioning repair Oxnard CA</t>
+        </is>
+      </c>
+      <c r="K1377" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1377" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="inlineStr">
+        <is>
+          <t>Velocity Mechanical</t>
+        </is>
+      </c>
+      <c r="B1378" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1378" t="inlineStr">
+        <is>
+          <t>velocityheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D1378" t="inlineStr">
+        <is>
+          <t>https://velocityheatingandcooling.com/ac-installation-lancaster-pa/</t>
+        </is>
+      </c>
+      <c r="E1378" t="inlineStr">
+        <is>
+          <t>Lancaster County</t>
+        </is>
+      </c>
+      <c r="F1378" t="inlineStr">
+        <is>
+          <t>info@velocityheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G1378" t="inlineStr">
+        <is>
+          <t>(717) 575-8874</t>
+        </is>
+      </c>
+      <c r="H1378" t="inlineStr">
+        <is>
+          <t>Lancaster PA</t>
+        </is>
+      </c>
+      <c r="I1378" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1378" t="inlineStr">
+        <is>
+          <t>AC installation Lancaster PA</t>
+        </is>
+      </c>
+      <c r="K1378" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1378" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="inlineStr">
+        <is>
+          <t>All County Air Conditioning &amp; Heating, Inc.</t>
+        </is>
+      </c>
+      <c r="B1379" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1379" t="inlineStr">
+        <is>
+          <t>allcountyairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D1379" t="inlineStr">
+        <is>
+          <t>https://allcountyairconditioning.com/ac-repair-in-oxnard-ca/</t>
+        </is>
+      </c>
+      <c r="E1379" t="inlineStr">
+        <is>
+          <t>Heating Inc</t>
+        </is>
+      </c>
+      <c r="F1379" t="inlineStr">
+        <is>
+          <t>info@domainname.com</t>
+        </is>
+      </c>
+      <c r="G1379" t="inlineStr">
+        <is>
+          <t>(805) 433-5292</t>
+        </is>
+      </c>
+      <c r="H1379" t="inlineStr">
+        <is>
+          <t>Oxnard CA</t>
+        </is>
+      </c>
+      <c r="I1379" t="n">
+        <v>86</v>
+      </c>
+      <c r="J1379" t="inlineStr">
+        <is>
+          <t>air conditioning repair Oxnard CA</t>
+        </is>
+      </c>
+      <c r="K1379" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1379" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:20 UTC (cycle 160)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1379"/>
+  <dimension ref="A1:L1384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -81194,6 +81194,306 @@
         </is>
       </c>
     </row>
+    <row r="1380">
+      <c r="A1380" t="inlineStr">
+        <is>
+          <t>United Developers</t>
+        </is>
+      </c>
+      <c r="B1380" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1380" t="inlineStr">
+        <is>
+          <t>udroofing.com</t>
+        </is>
+      </c>
+      <c r="D1380" t="inlineStr">
+        <is>
+          <t>https://udroofing.com/service-area/waldorf/</t>
+        </is>
+      </c>
+      <c r="E1380" t="inlineStr">
+        <is>
+          <t>Waldorf Full</t>
+        </is>
+      </c>
+      <c r="F1380" t="inlineStr">
+        <is>
+          <t>office@udroofing.com</t>
+        </is>
+      </c>
+      <c r="G1380" t="inlineStr">
+        <is>
+          <t>(240) 880-2108</t>
+        </is>
+      </c>
+      <c r="H1380" t="inlineStr">
+        <is>
+          <t>Waldorf MD</t>
+        </is>
+      </c>
+      <c r="I1380" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1380" t="inlineStr">
+        <is>
+          <t>roof replacement Waldorf MD</t>
+        </is>
+      </c>
+      <c r="K1380" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1380" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="inlineStr">
+        <is>
+          <t>Roofing Contractor &amp; Roofer in Great Falls, MT | Stay Dry Roofing</t>
+        </is>
+      </c>
+      <c r="B1381" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1381" t="inlineStr">
+        <is>
+          <t>staydryroofingmt.com</t>
+        </is>
+      </c>
+      <c r="D1381" t="inlineStr">
+        <is>
+          <t>https://staydryroofingmt.com/</t>
+        </is>
+      </c>
+      <c r="E1381" t="inlineStr">
+        <is>
+          <t>Stay Dry</t>
+        </is>
+      </c>
+      <c r="F1381" t="inlineStr">
+        <is>
+          <t>douglas@staydryroofingmt.com</t>
+        </is>
+      </c>
+      <c r="G1381" t="inlineStr">
+        <is>
+          <t>406-781-2277</t>
+        </is>
+      </c>
+      <c r="H1381" t="inlineStr">
+        <is>
+          <t>Great Falls MT</t>
+        </is>
+      </c>
+      <c r="I1381" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1381" t="inlineStr">
+        <is>
+          <t>roof repair company Great Falls MT</t>
+        </is>
+      </c>
+      <c r="K1381" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1381" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1382">
+      <c r="A1382" t="inlineStr">
+        <is>
+          <t>Roof Replacement Waldorf, MD</t>
+        </is>
+      </c>
+      <c r="B1382" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1382" t="inlineStr">
+        <is>
+          <t>providenceroofingandrepair.com</t>
+        </is>
+      </c>
+      <c r="D1382" t="inlineStr">
+        <is>
+          <t>https://www.providenceroofingandrepair.com/roof-replacement-waldorf-md/</t>
+        </is>
+      </c>
+      <c r="E1382" t="inlineStr">
+        <is>
+          <t>What Your</t>
+        </is>
+      </c>
+      <c r="F1382" t="inlineStr">
+        <is>
+          <t>info@providenceroofingandrepair.com</t>
+        </is>
+      </c>
+      <c r="G1382" t="inlineStr">
+        <is>
+          <t>(833) 435-4607</t>
+        </is>
+      </c>
+      <c r="H1382" t="inlineStr">
+        <is>
+          <t>Waldorf MD</t>
+        </is>
+      </c>
+      <c r="I1382" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1382" t="inlineStr">
+        <is>
+          <t>roof replacement Waldorf MD</t>
+        </is>
+      </c>
+      <c r="K1382" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1382" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="inlineStr">
+        <is>
+          <t>Swell Plumbing Co. | Trusted Plumber in Salem &amp; Willamette Valley</t>
+        </is>
+      </c>
+      <c r="B1383" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1383" t="inlineStr">
+        <is>
+          <t>swellplumbingco.com</t>
+        </is>
+      </c>
+      <c r="D1383" t="inlineStr">
+        <is>
+          <t>https://swellplumbingco.com/</t>
+        </is>
+      </c>
+      <c r="E1383" t="inlineStr">
+        <is>
+          <t>Google Swell</t>
+        </is>
+      </c>
+      <c r="F1383" t="inlineStr">
+        <is>
+          <t>swellconstructionllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1383" t="inlineStr">
+        <is>
+          <t>503-884-4072</t>
+        </is>
+      </c>
+      <c r="H1383" t="inlineStr">
+        <is>
+          <t>Salem OR</t>
+        </is>
+      </c>
+      <c r="I1383" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1383" t="inlineStr">
+        <is>
+          <t>plumber Salem OR</t>
+        </is>
+      </c>
+      <c r="K1383" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1383" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="inlineStr">
+        <is>
+          <t>Metropolitan Exteriors</t>
+        </is>
+      </c>
+      <c r="B1384" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1384" t="inlineStr">
+        <is>
+          <t>metropolitanexteriorsdmv.com</t>
+        </is>
+      </c>
+      <c r="D1384" t="inlineStr">
+        <is>
+          <t>https://metropolitanexteriorsdmv.com/pages/roofing-contractor-waldorf-md</t>
+        </is>
+      </c>
+      <c r="E1384" t="inlineStr">
+        <is>
+          <t>Exterior Innovations</t>
+        </is>
+      </c>
+      <c r="F1384" t="inlineStr">
+        <is>
+          <t>metroext@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1384" t="inlineStr">
+        <is>
+          <t>301-870-4500</t>
+        </is>
+      </c>
+      <c r="H1384" t="inlineStr">
+        <is>
+          <t>Waldorf MD</t>
+        </is>
+      </c>
+      <c r="I1384" t="n">
+        <v>88</v>
+      </c>
+      <c r="J1384" t="inlineStr">
+        <is>
+          <t>roof replacement Waldorf MD</t>
+        </is>
+      </c>
+      <c r="K1384" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1384" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:22 UTC (cycle 161)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1384"/>
+  <dimension ref="A1:L1385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -81494,6 +81494,66 @@
         </is>
       </c>
     </row>
+    <row r="1385">
+      <c r="A1385" t="inlineStr">
+        <is>
+          <t>Steward's Plumbing</t>
+        </is>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1385" t="inlineStr">
+        <is>
+          <t>stewardsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1385" t="inlineStr">
+        <is>
+          <t>https://www.stewardsplumbing.com/service-areas/rio-rancho/water-heaters/</t>
+        </is>
+      </c>
+      <c r="E1385" t="inlineStr">
+        <is>
+          <t>Rio Rancho</t>
+        </is>
+      </c>
+      <c r="F1385" t="inlineStr">
+        <is>
+          <t>info@stewardsplumbing.com</t>
+        </is>
+      </c>
+      <c r="G1385" t="inlineStr">
+        <is>
+          <t>505-906-6777</t>
+        </is>
+      </c>
+      <c r="H1385" t="inlineStr">
+        <is>
+          <t>Rio Rancho NM</t>
+        </is>
+      </c>
+      <c r="I1385" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1385" t="inlineStr">
+        <is>
+          <t>water heater repair Rio Rancho NM</t>
+        </is>
+      </c>
+      <c r="K1385" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1385" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:23 UTC (cycle 162)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1385"/>
+  <dimension ref="A1:L1393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -81554,6 +81554,474 @@
         </is>
       </c>
     </row>
+    <row r="1386">
+      <c r="A1386" t="inlineStr">
+        <is>
+          <t>Chaparosa Roofing</t>
+        </is>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>chaparosaroofing.com</t>
+        </is>
+      </c>
+      <c r="D1386" t="inlineStr">
+        <is>
+          <t>https://chaparosaroofing.com/service-areas/corona/residential/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E1386" t="inlineStr">
+        <is>
+          <t>High De</t>
+        </is>
+      </c>
+      <c r="F1386" t="inlineStr">
+        <is>
+          <t>info@chaparosaroofing.com</t>
+        </is>
+      </c>
+      <c r="G1386" t="inlineStr">
+        <is>
+          <t>(760) 240-0088</t>
+        </is>
+      </c>
+      <c r="H1386" t="inlineStr">
+        <is>
+          <t>Corona CA</t>
+        </is>
+      </c>
+      <c r="I1386" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1386" t="inlineStr">
+        <is>
+          <t>roof replacement Corona CA</t>
+        </is>
+      </c>
+      <c r="K1386" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1386" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="inlineStr">
+        <is>
+          <t>Red Peaks Roofing Inc | West Valley City, UT Metal Roofing &amp; Repairs</t>
+        </is>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1387" t="inlineStr">
+        <is>
+          <t>redpeaksroofing.com</t>
+        </is>
+      </c>
+      <c r="D1387" t="inlineStr">
+        <is>
+          <t>https://redpeaksroofing.com/service-areas/west-valley-city-ut-usa</t>
+        </is>
+      </c>
+      <c r="E1387" t="inlineStr">
+        <is>
+          <t>Red Peaks</t>
+        </is>
+      </c>
+      <c r="F1387" t="inlineStr">
+        <is>
+          <t>tig@redpeaksroofing.com</t>
+        </is>
+      </c>
+      <c r="G1387" t="inlineStr">
+        <is>
+          <t>(385)-482-9707</t>
+        </is>
+      </c>
+      <c r="H1387" t="inlineStr">
+        <is>
+          <t>West Valley City UT</t>
+        </is>
+      </c>
+      <c r="I1387" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1387" t="inlineStr">
+        <is>
+          <t>metal roofing contractor West Valley City UT</t>
+        </is>
+      </c>
+      <c r="K1387" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1387" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="inlineStr">
+        <is>
+          <t>Metal Roofing in West Valley City, UT | SPM Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1388" t="inlineStr">
+        <is>
+          <t>spmroofing.com</t>
+        </is>
+      </c>
+      <c r="D1388" t="inlineStr">
+        <is>
+          <t>https://spmroofing.com/geo/metal-roofing-west-valley-city-ut</t>
+        </is>
+      </c>
+      <c r="E1388" t="inlineStr"/>
+      <c r="F1388" t="inlineStr">
+        <is>
+          <t>spm.roofs@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1388" t="inlineStr">
+        <is>
+          <t>801-428-9475</t>
+        </is>
+      </c>
+      <c r="H1388" t="inlineStr">
+        <is>
+          <t>West Valley City UT</t>
+        </is>
+      </c>
+      <c r="I1388" t="n">
+        <v>94</v>
+      </c>
+      <c r="J1388" t="inlineStr">
+        <is>
+          <t>metal roofing contractor West Valley City UT</t>
+        </is>
+      </c>
+      <c r="K1388" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1388" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="inlineStr">
+        <is>
+          <t>Mega A/C Cooling &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1389" t="inlineStr">
+        <is>
+          <t>megaaircoolingandheat.com</t>
+        </is>
+      </c>
+      <c r="D1389" t="inlineStr">
+        <is>
+          <t>https://megaaircoolingandheat.com/furnace-repair-sugarland-tx/</t>
+        </is>
+      </c>
+      <c r="E1389" t="inlineStr">
+        <is>
+          <t>Common Furnace</t>
+        </is>
+      </c>
+      <c r="F1389" t="inlineStr">
+        <is>
+          <t>megaair2003@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1389" t="inlineStr">
+        <is>
+          <t>832-868-5196</t>
+        </is>
+      </c>
+      <c r="H1389" t="inlineStr">
+        <is>
+          <t>Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="I1389" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1389" t="inlineStr">
+        <is>
+          <t>furnace repair Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="K1389" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1389" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="inlineStr">
+        <is>
+          <t>Storm Guard</t>
+        </is>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1390" t="inlineStr">
+        <is>
+          <t>stormguardrc.com</t>
+        </is>
+      </c>
+      <c r="D1390" t="inlineStr">
+        <is>
+          <t>https://www.stormguardrc.com/tn/nashville/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E1390" t="inlineStr"/>
+      <c r="F1390" t="inlineStr">
+        <is>
+          <t>franchise@stormguardrc.com</t>
+        </is>
+      </c>
+      <c r="G1390" t="inlineStr">
+        <is>
+          <t>(615) 988-9420</t>
+        </is>
+      </c>
+      <c r="H1390" t="inlineStr">
+        <is>
+          <t>Nashville TN</t>
+        </is>
+      </c>
+      <c r="I1390" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1390" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Nashville TN</t>
+        </is>
+      </c>
+      <c r="K1390" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1390" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="inlineStr">
+        <is>
+          <t>Plumbing Solutions of Idaho</t>
+        </is>
+      </c>
+      <c r="B1391" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1391" t="inlineStr">
+        <is>
+          <t>plumbingsolutionsofidaho.com</t>
+        </is>
+      </c>
+      <c r="D1391" t="inlineStr">
+        <is>
+          <t>https://plumbingsolutionsofidaho.com/water-heaters/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E1391" t="inlineStr"/>
+      <c r="F1391" t="inlineStr">
+        <is>
+          <t>dispatch@plumbingsolutionsofidaho.com</t>
+        </is>
+      </c>
+      <c r="G1391" t="inlineStr">
+        <is>
+          <t>(208) 219-5708</t>
+        </is>
+      </c>
+      <c r="H1391" t="inlineStr">
+        <is>
+          <t>Boise ID</t>
+        </is>
+      </c>
+      <c r="I1391" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1391" t="inlineStr">
+        <is>
+          <t>water heater repair Boise ID</t>
+        </is>
+      </c>
+      <c r="K1391" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1391" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="inlineStr">
+        <is>
+          <t>Go Pro Roofing | Salt Lake City Roofing Experts</t>
+        </is>
+      </c>
+      <c r="B1392" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1392" t="inlineStr">
+        <is>
+          <t>gprroofing.com</t>
+        </is>
+      </c>
+      <c r="D1392" t="inlineStr">
+        <is>
+          <t>https://gprroofing.com/metal-roofing-contractors-west-valley-city-ut/</t>
+        </is>
+      </c>
+      <c r="E1392" t="inlineStr">
+        <is>
+          <t>Official Roof</t>
+        </is>
+      </c>
+      <c r="F1392" t="inlineStr">
+        <is>
+          <t>jose@gprroofing.com</t>
+        </is>
+      </c>
+      <c r="G1392" t="inlineStr">
+        <is>
+          <t>801-232-5823</t>
+        </is>
+      </c>
+      <c r="H1392" t="inlineStr">
+        <is>
+          <t>West Valley City UT</t>
+        </is>
+      </c>
+      <c r="I1392" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1392" t="inlineStr">
+        <is>
+          <t>metal roofing contractor West Valley City UT</t>
+        </is>
+      </c>
+      <c r="K1392" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1392" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="inlineStr">
+        <is>
+          <t>Ross Air</t>
+        </is>
+      </c>
+      <c r="B1393" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1393" t="inlineStr">
+        <is>
+          <t>rossair.com</t>
+        </is>
+      </c>
+      <c r="D1393" t="inlineStr">
+        <is>
+          <t>https://rossair.com/furnace-repair-heating-services-sugar-land-tx/</t>
+        </is>
+      </c>
+      <c r="E1393" t="inlineStr">
+        <is>
+          <t>Sugar Land</t>
+        </is>
+      </c>
+      <c r="F1393" t="inlineStr">
+        <is>
+          <t>service@rossair.com</t>
+        </is>
+      </c>
+      <c r="G1393" t="inlineStr">
+        <is>
+          <t>281-223-1176</t>
+        </is>
+      </c>
+      <c r="H1393" t="inlineStr">
+        <is>
+          <t>Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="I1393" t="n">
+        <v>82</v>
+      </c>
+      <c r="J1393" t="inlineStr">
+        <is>
+          <t>furnace repair Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="K1393" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1393" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:25 UTC (cycle 163)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1393"/>
+  <dimension ref="A1:L1396"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -81695,7 +81695,6 @@
           <t>https://spmroofing.com/geo/metal-roofing-west-valley-city-ut</t>
         </is>
       </c>
-      <c r="E1388" t="inlineStr"/>
       <c r="F1388" t="inlineStr">
         <is>
           <t>spm.roofs@gmail.com</t>
@@ -81811,7 +81810,6 @@
           <t>https://www.stormguardrc.com/tn/nashville/metal-roofing/</t>
         </is>
       </c>
-      <c r="E1390" t="inlineStr"/>
       <c r="F1390" t="inlineStr">
         <is>
           <t>franchise@stormguardrc.com</t>
@@ -81867,7 +81865,6 @@
           <t>https://plumbingsolutionsofidaho.com/water-heaters/water-heater-repair/</t>
         </is>
       </c>
-      <c r="E1391" t="inlineStr"/>
       <c r="F1391" t="inlineStr">
         <is>
           <t>dispatch@plumbingsolutionsofidaho.com</t>
@@ -82017,6 +82014,178 @@
         </is>
       </c>
       <c r="L1393" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="inlineStr">
+        <is>
+          <t>Expert Roofing Services Sugar Land, TX</t>
+        </is>
+      </c>
+      <c r="B1394" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1394" t="inlineStr">
+        <is>
+          <t>roofdaddyroofing.com</t>
+        </is>
+      </c>
+      <c r="D1394" t="inlineStr">
+        <is>
+          <t>https://www.roofdaddyroofing.com/service-areas/roofing-company-sugar-land-tx</t>
+        </is>
+      </c>
+      <c r="E1394" t="inlineStr">
+        <is>
+          <t>Suite Exec</t>
+        </is>
+      </c>
+      <c r="F1394" t="inlineStr">
+        <is>
+          <t>info@txroofdaddy.com</t>
+        </is>
+      </c>
+      <c r="G1394" t="inlineStr">
+        <is>
+          <t>(281) 844-1047</t>
+        </is>
+      </c>
+      <c r="H1394" t="inlineStr">
+        <is>
+          <t>Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="I1394" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1394" t="inlineStr">
+        <is>
+          <t>roof repair company Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="K1394" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1394" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="inlineStr">
+        <is>
+          <t>Affordable Roofing and Waterproofing</t>
+        </is>
+      </c>
+      <c r="B1395" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1395" t="inlineStr">
+        <is>
+          <t>affordableroofingtx.com</t>
+        </is>
+      </c>
+      <c r="D1395" t="inlineStr">
+        <is>
+          <t>https://www.affordableroofingtx.com/service-areas/sugar-land</t>
+        </is>
+      </c>
+      <c r="E1395" t="inlineStr">
+        <is>
+          <t>Drone Inspections</t>
+        </is>
+      </c>
+      <c r="F1395" t="inlineStr">
+        <is>
+          <t>info.tx@affordableroofingtx.com</t>
+        </is>
+      </c>
+      <c r="G1395" t="inlineStr">
+        <is>
+          <t>(713) 909-0443</t>
+        </is>
+      </c>
+      <c r="H1395" t="inlineStr">
+        <is>
+          <t>Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="I1395" t="n">
+        <v>88</v>
+      </c>
+      <c r="J1395" t="inlineStr">
+        <is>
+          <t>roof repair company Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="K1395" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1395" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="inlineStr">
+        <is>
+          <t>$199 Roof Repair</t>
+        </is>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1396" t="inlineStr">
+        <is>
+          <t>199roofrepair.com</t>
+        </is>
+      </c>
+      <c r="D1396" t="inlineStr">
+        <is>
+          <t>https://199roofrepair.com/sugar-land-tx/</t>
+        </is>
+      </c>
+      <c r="E1396" t="inlineStr"/>
+      <c r="F1396" t="inlineStr">
+        <is>
+          <t>199roofrepairllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1396" t="inlineStr"/>
+      <c r="H1396" t="inlineStr">
+        <is>
+          <t>Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="I1396" t="n">
+        <v>76</v>
+      </c>
+      <c r="J1396" t="inlineStr">
+        <is>
+          <t>roof repair company Sugar Land TX</t>
+        </is>
+      </c>
+      <c r="K1396" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1396" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:26 UTC (cycle 164)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1396"/>
+  <dimension ref="A1:L1400"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -82160,13 +82160,11 @@
           <t>https://199roofrepair.com/sugar-land-tx/</t>
         </is>
       </c>
-      <c r="E1396" t="inlineStr"/>
       <c r="F1396" t="inlineStr">
         <is>
           <t>199roofrepairllc@gmail.com</t>
         </is>
       </c>
-      <c r="G1396" t="inlineStr"/>
       <c r="H1396" t="inlineStr">
         <is>
           <t>Sugar Land TX</t>
@@ -82186,6 +82184,242 @@
         </is>
       </c>
       <c r="L1396" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="inlineStr">
+        <is>
+          <t>Total Roofing</t>
+        </is>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1397" t="inlineStr">
+        <is>
+          <t>totalroofingstl.com</t>
+        </is>
+      </c>
+      <c r="D1397" t="inlineStr">
+        <is>
+          <t>https://www.totalroofingstl.com/residential-roofing/metal-roofs/</t>
+        </is>
+      </c>
+      <c r="E1397" t="inlineStr">
+        <is>
+          <t>Mike Augustine</t>
+        </is>
+      </c>
+      <c r="F1397" t="inlineStr">
+        <is>
+          <t>mike.a@totalroofingstl.com</t>
+        </is>
+      </c>
+      <c r="G1397" t="inlineStr">
+        <is>
+          <t>(618) 719-6767</t>
+        </is>
+      </c>
+      <c r="H1397" t="inlineStr">
+        <is>
+          <t>St Louis MO</t>
+        </is>
+      </c>
+      <c r="I1397" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1397" t="inlineStr">
+        <is>
+          <t>metal roofing contractor St Louis MO</t>
+        </is>
+      </c>
+      <c r="K1397" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1397" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="inlineStr">
+        <is>
+          <t>Roofing Company in St. Louis | Siding Company St. Louis</t>
+        </is>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1398" t="inlineStr">
+        <is>
+          <t>gallagherbrosconstruction.com</t>
+        </is>
+      </c>
+      <c r="D1398" t="inlineStr">
+        <is>
+          <t>https://gallagherbrosconstruction.com/metal-roofing-in-st-louis/</t>
+        </is>
+      </c>
+      <c r="E1398" t="inlineStr">
+        <is>
+          <t>South County</t>
+        </is>
+      </c>
+      <c r="F1398" t="inlineStr">
+        <is>
+          <t>info@gallagherbrosconstruction.com</t>
+        </is>
+      </c>
+      <c r="G1398" t="inlineStr">
+        <is>
+          <t>314.646.8015</t>
+        </is>
+      </c>
+      <c r="H1398" t="inlineStr">
+        <is>
+          <t>St Louis MO</t>
+        </is>
+      </c>
+      <c r="I1398" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1398" t="inlineStr">
+        <is>
+          <t>metal roofing contractor St Louis MO</t>
+        </is>
+      </c>
+      <c r="K1398" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1398" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="inlineStr">
+        <is>
+          <t>Meridian Roofing and Renovation</t>
+        </is>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1399" t="inlineStr">
+        <is>
+          <t>buildmeridian.com</t>
+        </is>
+      </c>
+      <c r="D1399" t="inlineStr">
+        <is>
+          <t>https://buildmeridian.com/services/metal-roofing-st-louis-mo/</t>
+        </is>
+      </c>
+      <c r="E1399" t="inlineStr">
+        <is>
+          <t>Satisfied Customers</t>
+        </is>
+      </c>
+      <c r="F1399" t="inlineStr">
+        <is>
+          <t>alex@buildmeridian.com</t>
+        </is>
+      </c>
+      <c r="G1399" t="inlineStr">
+        <is>
+          <t>314-952-4158</t>
+        </is>
+      </c>
+      <c r="H1399" t="inlineStr">
+        <is>
+          <t>St Louis MO</t>
+        </is>
+      </c>
+      <c r="I1399" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1399" t="inlineStr">
+        <is>
+          <t>metal roofing contractor St Louis MO</t>
+        </is>
+      </c>
+      <c r="K1399" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1399" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="inlineStr">
+        <is>
+          <t>Premier Metal Roofing - St. Louis</t>
+        </is>
+      </c>
+      <c r="B1400" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1400" t="inlineStr">
+        <is>
+          <t>metalroofingstlouismo.com</t>
+        </is>
+      </c>
+      <c r="D1400" t="inlineStr">
+        <is>
+          <t>https://metalroofingstlouismo.com/</t>
+        </is>
+      </c>
+      <c r="E1400" t="inlineStr"/>
+      <c r="F1400" t="inlineStr">
+        <is>
+          <t>info@metalroofingstlouismo.com</t>
+        </is>
+      </c>
+      <c r="G1400" t="inlineStr">
+        <is>
+          <t>(314) 350-4076</t>
+        </is>
+      </c>
+      <c r="H1400" t="inlineStr">
+        <is>
+          <t>St Louis MO</t>
+        </is>
+      </c>
+      <c r="I1400" t="n">
+        <v>96</v>
+      </c>
+      <c r="J1400" t="inlineStr">
+        <is>
+          <t>metal roofing contractor St Louis MO</t>
+        </is>
+      </c>
+      <c r="K1400" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1400" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:28 UTC (cycle 165)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1400"/>
+  <dimension ref="A1:L1405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -82390,7 +82390,6 @@
           <t>https://metalroofingstlouismo.com/</t>
         </is>
       </c>
-      <c r="E1400" t="inlineStr"/>
       <c r="F1400" t="inlineStr">
         <is>
           <t>info@metalroofingstlouismo.com</t>
@@ -82420,6 +82419,298 @@
         </is>
       </c>
       <c r="L1400" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="inlineStr">
+        <is>
+          <t>Mount Vernon Roofer</t>
+        </is>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1401" t="inlineStr">
+        <is>
+          <t>mountvernonroofer.com</t>
+        </is>
+      </c>
+      <c r="D1401" t="inlineStr">
+        <is>
+          <t>https://mountvernonroofer.com/</t>
+        </is>
+      </c>
+      <c r="E1401" t="inlineStr">
+        <is>
+          <t>Mount Vernon</t>
+        </is>
+      </c>
+      <c r="F1401" t="inlineStr">
+        <is>
+          <t>info@mountvernonroofer.com</t>
+        </is>
+      </c>
+      <c r="G1401" t="inlineStr">
+        <is>
+          <t>(914) 491-1973</t>
+        </is>
+      </c>
+      <c r="H1401" t="inlineStr">
+        <is>
+          <t>Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="I1401" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1401" t="inlineStr">
+        <is>
+          <t>residential roofing company Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="K1401" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1401" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="inlineStr">
+        <is>
+          <t>Elite Roofing Company Long Island NY</t>
+        </is>
+      </c>
+      <c r="B1402" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1402" t="inlineStr">
+        <is>
+          <t>eliteroofingny.com</t>
+        </is>
+      </c>
+      <c r="D1402" t="inlineStr">
+        <is>
+          <t>https://www.eliteroofingny.com/roofing-company-mount-vernon/</t>
+        </is>
+      </c>
+      <c r="E1402" t="inlineStr"/>
+      <c r="F1402" t="inlineStr">
+        <is>
+          <t>info@eliteroofingny.com</t>
+        </is>
+      </c>
+      <c r="G1402" t="inlineStr">
+        <is>
+          <t>516-774-4477</t>
+        </is>
+      </c>
+      <c r="H1402" t="inlineStr">
+        <is>
+          <t>Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="I1402" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1402" t="inlineStr">
+        <is>
+          <t>residential roofing company Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="K1402" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1402" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" t="inlineStr">
+        <is>
+          <t>Chill Heating &amp; Cooling – HVAC Company in San Ramon, Walnut Creek and Fremont</t>
+        </is>
+      </c>
+      <c r="B1403" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1403" t="inlineStr">
+        <is>
+          <t>chill-services.com</t>
+        </is>
+      </c>
+      <c r="D1403" t="inlineStr">
+        <is>
+          <t>https://chill-services.com/service-area/fremont-hvac-services</t>
+        </is>
+      </c>
+      <c r="E1403" t="inlineStr">
+        <is>
+          <t>Chill Heating</t>
+        </is>
+      </c>
+      <c r="F1403" t="inlineStr">
+        <is>
+          <t>support@chill-services.com</t>
+        </is>
+      </c>
+      <c r="G1403" t="inlineStr">
+        <is>
+          <t>(925) 350-7558</t>
+        </is>
+      </c>
+      <c r="H1403" t="inlineStr">
+        <is>
+          <t>Fremont CA</t>
+        </is>
+      </c>
+      <c r="I1403" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1403" t="inlineStr">
+        <is>
+          <t>furnace repair Fremont CA</t>
+        </is>
+      </c>
+      <c r="K1403" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1403" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" t="inlineStr">
+        <is>
+          <t>On Time Roofing</t>
+        </is>
+      </c>
+      <c r="B1404" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1404" t="inlineStr">
+        <is>
+          <t>ontimeroofingny.com</t>
+        </is>
+      </c>
+      <c r="D1404" t="inlineStr">
+        <is>
+          <t>https://ontimeroofingny.com/roofing-mount-vernon-ny/</t>
+        </is>
+      </c>
+      <c r="E1404" t="inlineStr">
+        <is>
+          <t>Residential Roofing</t>
+        </is>
+      </c>
+      <c r="F1404" t="inlineStr">
+        <is>
+          <t>ontime533@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1404" t="inlineStr">
+        <is>
+          <t>914-924-4869</t>
+        </is>
+      </c>
+      <c r="H1404" t="inlineStr">
+        <is>
+          <t>Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="I1404" t="n">
+        <v>98</v>
+      </c>
+      <c r="J1404" t="inlineStr">
+        <is>
+          <t>residential roofing company Mount Vernon NY</t>
+        </is>
+      </c>
+      <c r="K1404" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1404" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" t="inlineStr">
+        <is>
+          <t>TFF HVAC</t>
+        </is>
+      </c>
+      <c r="B1405" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1405" t="inlineStr">
+        <is>
+          <t>tffhvac.com</t>
+        </is>
+      </c>
+      <c r="D1405" t="inlineStr">
+        <is>
+          <t>https://tffhvac.com/fremont-ca/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E1405" t="inlineStr"/>
+      <c r="F1405" t="inlineStr">
+        <is>
+          <t>info@tffhvac.com</t>
+        </is>
+      </c>
+      <c r="G1405" t="inlineStr">
+        <is>
+          <t>(408) 786-8120</t>
+        </is>
+      </c>
+      <c r="H1405" t="inlineStr">
+        <is>
+          <t>Fremont CA</t>
+        </is>
+      </c>
+      <c r="I1405" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1405" t="inlineStr">
+        <is>
+          <t>furnace repair Fremont CA</t>
+        </is>
+      </c>
+      <c r="K1405" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1405" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:31 UTC (cycle 167)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1405"/>
+  <dimension ref="A1:L1407"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -82505,7 +82505,6 @@
           <t>https://www.eliteroofingny.com/roofing-company-mount-vernon/</t>
         </is>
       </c>
-      <c r="E1402" t="inlineStr"/>
       <c r="F1402" t="inlineStr">
         <is>
           <t>info@eliteroofingny.com</t>
@@ -82681,7 +82680,6 @@
           <t>https://tffhvac.com/fremont-ca/furnace-repair/</t>
         </is>
       </c>
-      <c r="E1405" t="inlineStr"/>
       <c r="F1405" t="inlineStr">
         <is>
           <t>info@tffhvac.com</t>
@@ -82711,6 +82709,126 @@
         </is>
       </c>
       <c r="L1405" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" t="inlineStr">
+        <is>
+          <t>Action Plumbing, Heating, Air Conditioning and Electric, Inc</t>
+        </is>
+      </c>
+      <c r="B1406" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1406" t="inlineStr">
+        <is>
+          <t>iwantactionnow.com</t>
+        </is>
+      </c>
+      <c r="D1406" t="inlineStr">
+        <is>
+          <t>https://www.iwantactionnow.com/air-conditioning/installation</t>
+        </is>
+      </c>
+      <c r="E1406" t="inlineStr">
+        <is>
+          <t>Many Madison</t>
+        </is>
+      </c>
+      <c r="F1406" t="inlineStr">
+        <is>
+          <t>info@iwantactionnow.com</t>
+        </is>
+      </c>
+      <c r="G1406" t="inlineStr">
+        <is>
+          <t>(608)-837-3638</t>
+        </is>
+      </c>
+      <c r="H1406" t="inlineStr">
+        <is>
+          <t>Madison WI</t>
+        </is>
+      </c>
+      <c r="I1406" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1406" t="inlineStr">
+        <is>
+          <t>AC installation Madison WI</t>
+        </is>
+      </c>
+      <c r="K1406" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1406" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" t="inlineStr">
+        <is>
+          <t>Harker Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B1407" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1407" t="inlineStr">
+        <is>
+          <t>harkerheating.com</t>
+        </is>
+      </c>
+      <c r="D1407" t="inlineStr">
+        <is>
+          <t>https://www.harkerheating.com/ac-installation-madison-wi/</t>
+        </is>
+      </c>
+      <c r="E1407" t="inlineStr">
+        <is>
+          <t>Why Madison</t>
+        </is>
+      </c>
+      <c r="F1407" t="inlineStr">
+        <is>
+          <t>info@harkerheating.com</t>
+        </is>
+      </c>
+      <c r="G1407" t="inlineStr">
+        <is>
+          <t>(608) 255-6902</t>
+        </is>
+      </c>
+      <c r="H1407" t="inlineStr">
+        <is>
+          <t>Madison WI</t>
+        </is>
+      </c>
+      <c r="I1407" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1407" t="inlineStr">
+        <is>
+          <t>AC installation Madison WI</t>
+        </is>
+      </c>
+      <c r="K1407" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1407" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:32 UTC (cycle 168)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1407"/>
+  <dimension ref="A1:L1409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -82834,6 +82834,126 @@
         </is>
       </c>
     </row>
+    <row r="1408">
+      <c r="A1408" t="inlineStr">
+        <is>
+          <t>Orca Roofing &amp; Exteriors</t>
+        </is>
+      </c>
+      <c r="B1408" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1408" t="inlineStr">
+        <is>
+          <t>orcaroofing.com</t>
+        </is>
+      </c>
+      <c r="D1408" t="inlineStr">
+        <is>
+          <t>https://www.orcaroofing.com/location/bellevue/</t>
+        </is>
+      </c>
+      <c r="E1408" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F1408" t="inlineStr">
+        <is>
+          <t>info@orcaroofing.com</t>
+        </is>
+      </c>
+      <c r="G1408" t="inlineStr">
+        <is>
+          <t>(425) 549-9539</t>
+        </is>
+      </c>
+      <c r="H1408" t="inlineStr">
+        <is>
+          <t>Bellevue WA</t>
+        </is>
+      </c>
+      <c r="I1408" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1408" t="inlineStr">
+        <is>
+          <t>roofing contractor Bellevue WA</t>
+        </is>
+      </c>
+      <c r="K1408" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1408" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" t="inlineStr">
+        <is>
+          <t>Blitz Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B1409" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1409" t="inlineStr">
+        <is>
+          <t>blitzroofing.llc</t>
+        </is>
+      </c>
+      <c r="D1409" t="inlineStr">
+        <is>
+          <t>https://www.blitzroofing.llc/service-areas/bellevue</t>
+        </is>
+      </c>
+      <c r="E1409" t="inlineStr">
+        <is>
+          <t>Inspection About</t>
+        </is>
+      </c>
+      <c r="F1409" t="inlineStr">
+        <is>
+          <t>contact@blitzroofing.llc</t>
+        </is>
+      </c>
+      <c r="G1409" t="inlineStr">
+        <is>
+          <t>(425) 900-4828</t>
+        </is>
+      </c>
+      <c r="H1409" t="inlineStr">
+        <is>
+          <t>Bellevue WA</t>
+        </is>
+      </c>
+      <c r="I1409" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1409" t="inlineStr">
+        <is>
+          <t>roofing contractor Bellevue WA</t>
+        </is>
+      </c>
+      <c r="K1409" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1409" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:34 UTC (cycle 169)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1409"/>
+  <dimension ref="A1:L1410"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -82954,6 +82954,62 @@
         </is>
       </c>
     </row>
+    <row r="1410">
+      <c r="A1410" t="inlineStr">
+        <is>
+          <t>Schebler HVAC</t>
+        </is>
+      </c>
+      <c r="B1410" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1410" t="inlineStr">
+        <is>
+          <t>scheblerhvac.com</t>
+        </is>
+      </c>
+      <c r="D1410" t="inlineStr">
+        <is>
+          <t>https://www.scheblerhvac.com/davenport-ia/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E1410" t="inlineStr"/>
+      <c r="F1410" t="inlineStr">
+        <is>
+          <t>reshvac@schebler.com</t>
+        </is>
+      </c>
+      <c r="G1410" t="inlineStr">
+        <is>
+          <t>563.359.8001</t>
+        </is>
+      </c>
+      <c r="H1410" t="inlineStr">
+        <is>
+          <t>Davenport IA</t>
+        </is>
+      </c>
+      <c r="I1410" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1410" t="inlineStr">
+        <is>
+          <t>furnace repair Davenport IA</t>
+        </is>
+      </c>
+      <c r="K1410" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1410" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:37 UTC (cycle 171)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1410"/>
+  <dimension ref="A1:L1415"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -82975,7 +82975,6 @@
           <t>https://www.scheblerhvac.com/davenport-ia/furnace-repair/</t>
         </is>
       </c>
-      <c r="E1410" t="inlineStr"/>
       <c r="F1410" t="inlineStr">
         <is>
           <t>reshvac@schebler.com</t>
@@ -83005,6 +83004,298 @@
         </is>
       </c>
       <c r="L1410" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" t="inlineStr">
+        <is>
+          <t>AC Repair Brooklyn Park, MN | Air Conditioner Repair</t>
+        </is>
+      </c>
+      <c r="B1411" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1411" t="inlineStr">
+        <is>
+          <t>staffordhomeservice.com</t>
+        </is>
+      </c>
+      <c r="D1411" t="inlineStr">
+        <is>
+          <t>https://www.staffordhomeservice.com/air-conditioning/ac-repair-brooklyn-park-mn</t>
+        </is>
+      </c>
+      <c r="E1411" t="inlineStr">
+        <is>
+          <t>Repair For</t>
+        </is>
+      </c>
+      <c r="F1411" t="inlineStr">
+        <is>
+          <t>sales@staffordhomeservice.com</t>
+        </is>
+      </c>
+      <c r="G1411" t="inlineStr">
+        <is>
+          <t>(952) 927-7194</t>
+        </is>
+      </c>
+      <c r="H1411" t="inlineStr">
+        <is>
+          <t>Brooklyn Park MN</t>
+        </is>
+      </c>
+      <c r="I1411" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1411" t="inlineStr">
+        <is>
+          <t>air conditioning repair Brooklyn Park MN</t>
+        </is>
+      </c>
+      <c r="K1411" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1411" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" t="inlineStr">
+        <is>
+          <t>billyGO Air Conditioning &amp; Plumbing</t>
+        </is>
+      </c>
+      <c r="B1412" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1412" t="inlineStr">
+        <is>
+          <t>billygo.com</t>
+        </is>
+      </c>
+      <c r="D1412" t="inlineStr">
+        <is>
+          <t>https://www.billygo.com/drain-services/drain-cleaning-service/</t>
+        </is>
+      </c>
+      <c r="E1412" t="inlineStr">
+        <is>
+          <t>Team Billy</t>
+        </is>
+      </c>
+      <c r="F1412" t="inlineStr">
+        <is>
+          <t>support@billygo.com</t>
+        </is>
+      </c>
+      <c r="G1412" t="inlineStr">
+        <is>
+          <t>(833) 787-7188</t>
+        </is>
+      </c>
+      <c r="H1412" t="inlineStr">
+        <is>
+          <t>Dallas TX</t>
+        </is>
+      </c>
+      <c r="I1412" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1412" t="inlineStr">
+        <is>
+          <t>drain cleaning service Dallas TX</t>
+        </is>
+      </c>
+      <c r="K1412" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1412" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" t="inlineStr">
+        <is>
+          <t>Coastal Heating</t>
+        </is>
+      </c>
+      <c r="B1413" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1413" t="inlineStr">
+        <is>
+          <t>coastalahr.com</t>
+        </is>
+      </c>
+      <c r="D1413" t="inlineStr">
+        <is>
+          <t>https://coastalahr.com/</t>
+        </is>
+      </c>
+      <c r="E1413" t="inlineStr"/>
+      <c r="F1413" t="inlineStr">
+        <is>
+          <t>customerservice@coastalahr.com</t>
+        </is>
+      </c>
+      <c r="G1413" t="inlineStr">
+        <is>
+          <t>617-770-0636</t>
+        </is>
+      </c>
+      <c r="H1413" t="inlineStr">
+        <is>
+          <t>Quincy MA</t>
+        </is>
+      </c>
+      <c r="I1413" t="n">
+        <v>98</v>
+      </c>
+      <c r="J1413" t="inlineStr">
+        <is>
+          <t>AC installation Quincy MA</t>
+        </is>
+      </c>
+      <c r="K1413" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1413" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" t="inlineStr">
+        <is>
+          <t>Drain Cleaning Dallas TX</t>
+        </is>
+      </c>
+      <c r="B1414" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1414" t="inlineStr">
+        <is>
+          <t>draincleaningdallastx.net</t>
+        </is>
+      </c>
+      <c r="D1414" t="inlineStr">
+        <is>
+          <t>https://draincleaningdallastx.net/</t>
+        </is>
+      </c>
+      <c r="E1414" t="inlineStr">
+        <is>
+          <t>Retail Spaces</t>
+        </is>
+      </c>
+      <c r="F1414" t="inlineStr">
+        <is>
+          <t>hire@draincleaningdallastx.net</t>
+        </is>
+      </c>
+      <c r="G1414" t="inlineStr">
+        <is>
+          <t>(214) 771-9407</t>
+        </is>
+      </c>
+      <c r="H1414" t="inlineStr">
+        <is>
+          <t>Dallas TX</t>
+        </is>
+      </c>
+      <c r="I1414" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1414" t="inlineStr">
+        <is>
+          <t>drain cleaning service Dallas TX</t>
+        </is>
+      </c>
+      <c r="K1414" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1414" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" t="inlineStr">
+        <is>
+          <t>Home Comfort Solutions LLC</t>
+        </is>
+      </c>
+      <c r="B1415" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1415" t="inlineStr">
+        <is>
+          <t>homecomfortsolutionsma.com</t>
+        </is>
+      </c>
+      <c r="D1415" t="inlineStr">
+        <is>
+          <t>https://www.homecomfortsolutionsma.com/cooling-services-ma</t>
+        </is>
+      </c>
+      <c r="E1415" t="inlineStr">
+        <is>
+          <t>Home Comfort</t>
+        </is>
+      </c>
+      <c r="F1415" t="inlineStr">
+        <is>
+          <t>office@homecomfortsolutionsma.com</t>
+        </is>
+      </c>
+      <c r="G1415" t="inlineStr"/>
+      <c r="H1415" t="inlineStr">
+        <is>
+          <t>Quincy MA</t>
+        </is>
+      </c>
+      <c r="I1415" t="n">
+        <v>86</v>
+      </c>
+      <c r="J1415" t="inlineStr">
+        <is>
+          <t>AC installation Quincy MA</t>
+        </is>
+      </c>
+      <c r="K1415" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1415" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:38 UTC (cycle 172)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1415"/>
+  <dimension ref="A1:L1421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -83150,7 +83150,6 @@
           <t>https://coastalahr.com/</t>
         </is>
       </c>
-      <c r="E1413" t="inlineStr"/>
       <c r="F1413" t="inlineStr">
         <is>
           <t>customerservice@coastalahr.com</t>
@@ -83276,7 +83275,6 @@
           <t>office@homecomfortsolutionsma.com</t>
         </is>
       </c>
-      <c r="G1415" t="inlineStr"/>
       <c r="H1415" t="inlineStr">
         <is>
           <t>Quincy MA</t>
@@ -83296,6 +83294,366 @@
         </is>
       </c>
       <c r="L1415" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" t="inlineStr">
+        <is>
+          <t>Platinum preferred Roofing Contractor | Bufalo Contracting | Rockford &amp; Belvider</t>
+        </is>
+      </c>
+      <c r="B1416" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1416" t="inlineStr">
+        <is>
+          <t>bufalocontracting.com</t>
+        </is>
+      </c>
+      <c r="D1416" t="inlineStr">
+        <is>
+          <t>https://www.bufalocontracting.com/</t>
+        </is>
+      </c>
+      <c r="E1416" t="inlineStr">
+        <is>
+          <t>Bufalo Contracting</t>
+        </is>
+      </c>
+      <c r="F1416" t="inlineStr">
+        <is>
+          <t>sbufalo@bufalocontracting.com</t>
+        </is>
+      </c>
+      <c r="G1416" t="inlineStr">
+        <is>
+          <t>(779) 368-0256</t>
+        </is>
+      </c>
+      <c r="H1416" t="inlineStr">
+        <is>
+          <t>Rockford IL</t>
+        </is>
+      </c>
+      <c r="I1416" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1416" t="inlineStr">
+        <is>
+          <t>roofing contractor Rockford IL</t>
+        </is>
+      </c>
+      <c r="K1416" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1416" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" t="inlineStr">
+        <is>
+          <t>Premium Roofing Solutions</t>
+        </is>
+      </c>
+      <c r="B1417" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1417" t="inlineStr">
+        <is>
+          <t>premiumroofsllc.com</t>
+        </is>
+      </c>
+      <c r="D1417" t="inlineStr">
+        <is>
+          <t>https://premiumroofsllc.com/service-area/rockford-il/</t>
+        </is>
+      </c>
+      <c r="E1417" t="inlineStr">
+        <is>
+          <t>Homeowner Satisfaction</t>
+        </is>
+      </c>
+      <c r="F1417" t="inlineStr">
+        <is>
+          <t>sales@premiumroofsllc.com</t>
+        </is>
+      </c>
+      <c r="G1417" t="inlineStr">
+        <is>
+          <t>(844) 997-6633</t>
+        </is>
+      </c>
+      <c r="H1417" t="inlineStr">
+        <is>
+          <t>Rockford IL</t>
+        </is>
+      </c>
+      <c r="I1417" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1417" t="inlineStr">
+        <is>
+          <t>roofing contractor Rockford IL</t>
+        </is>
+      </c>
+      <c r="K1417" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1417" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" t="inlineStr">
+        <is>
+          <t>Mission Roofing And Restoration, LLC</t>
+        </is>
+      </c>
+      <c r="B1418" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1418" t="inlineStr">
+        <is>
+          <t>missionroofingnm.com</t>
+        </is>
+      </c>
+      <c r="D1418" t="inlineStr">
+        <is>
+          <t>https://www.missionroofingnm.com/roof-replacement-las-cruces-nm</t>
+        </is>
+      </c>
+      <c r="E1418" t="inlineStr">
+        <is>
+          <t>Competitive Pricing</t>
+        </is>
+      </c>
+      <c r="F1418" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G1418" t="inlineStr">
+        <is>
+          <t>(575) 650-9280</t>
+        </is>
+      </c>
+      <c r="H1418" t="inlineStr">
+        <is>
+          <t>Las Cruces NM</t>
+        </is>
+      </c>
+      <c r="I1418" t="n">
+        <v>96</v>
+      </c>
+      <c r="J1418" t="inlineStr">
+        <is>
+          <t>roof replacement Las Cruces NM</t>
+        </is>
+      </c>
+      <c r="K1418" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1418" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1419">
+      <c r="A1419" t="inlineStr">
+        <is>
+          <t>Las Cruces Ridge</t>
+        </is>
+      </c>
+      <c r="B1419" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1419" t="inlineStr">
+        <is>
+          <t>roofinglascruse.com</t>
+        </is>
+      </c>
+      <c r="D1419" t="inlineStr">
+        <is>
+          <t>https://roofinglascruse.com/roof-replacement-las-cruces/</t>
+        </is>
+      </c>
+      <c r="E1419" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F1419" t="inlineStr">
+        <is>
+          <t>support@roofinglascruse.com</t>
+        </is>
+      </c>
+      <c r="G1419" t="inlineStr">
+        <is>
+          <t>(575) 237 8088</t>
+        </is>
+      </c>
+      <c r="H1419" t="inlineStr">
+        <is>
+          <t>Las Cruces NM</t>
+        </is>
+      </c>
+      <c r="I1419" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1419" t="inlineStr">
+        <is>
+          <t>roof replacement Las Cruces NM</t>
+        </is>
+      </c>
+      <c r="K1419" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1419" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" t="inlineStr">
+        <is>
+          <t>Lutz Plumbing, Inc. | Kansas City's Local Plumber</t>
+        </is>
+      </c>
+      <c r="B1420" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1420" t="inlineStr">
+        <is>
+          <t>lutzplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1420" t="inlineStr">
+        <is>
+          <t>https://lutzplumbing.com/independence-mo/</t>
+        </is>
+      </c>
+      <c r="E1420" t="inlineStr">
+        <is>
+          <t>Why Independence</t>
+        </is>
+      </c>
+      <c r="F1420" t="inlineStr">
+        <is>
+          <t>website@lutzplumbing.com</t>
+        </is>
+      </c>
+      <c r="G1420" t="inlineStr">
+        <is>
+          <t>(913) 631-2667</t>
+        </is>
+      </c>
+      <c r="H1420" t="inlineStr">
+        <is>
+          <t>Independence MO</t>
+        </is>
+      </c>
+      <c r="I1420" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1420" t="inlineStr">
+        <is>
+          <t>plumbing company Independence MO</t>
+        </is>
+      </c>
+      <c r="K1420" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1420" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" t="inlineStr">
+        <is>
+          <t>Politz Enterprises</t>
+        </is>
+      </c>
+      <c r="B1421" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1421" t="inlineStr">
+        <is>
+          <t>politzenterprises.com</t>
+        </is>
+      </c>
+      <c r="D1421" t="inlineStr">
+        <is>
+          <t>https://politzenterprises.com/metal-roofing-installation-frederick-md/</t>
+        </is>
+      </c>
+      <c r="E1421" t="inlineStr">
+        <is>
+          <t>Politz Meet</t>
+        </is>
+      </c>
+      <c r="F1421" t="inlineStr">
+        <is>
+          <t>robertpolitz@politzenterprises.com</t>
+        </is>
+      </c>
+      <c r="G1421" t="inlineStr">
+        <is>
+          <t>301-620-2023</t>
+        </is>
+      </c>
+      <c r="H1421" t="inlineStr">
+        <is>
+          <t>Frederick MD</t>
+        </is>
+      </c>
+      <c r="I1421" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1421" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Frederick MD</t>
+        </is>
+      </c>
+      <c r="K1421" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1421" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:40 UTC (cycle 173)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1421"/>
+  <dimension ref="A1:L1423"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -83659,6 +83659,122 @@
         </is>
       </c>
     </row>
+    <row r="1422">
+      <c r="A1422" t="inlineStr">
+        <is>
+          <t>Cornel's Plumbing</t>
+        </is>
+      </c>
+      <c r="B1422" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1422" t="inlineStr">
+        <is>
+          <t>cornelsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1422" t="inlineStr">
+        <is>
+          <t>https://cornelsplumbing.com/plumbing-services/beaverton-plumbers/</t>
+        </is>
+      </c>
+      <c r="E1422" t="inlineStr"/>
+      <c r="F1422" t="inlineStr">
+        <is>
+          <t>contact@cornelsplumbing.com</t>
+        </is>
+      </c>
+      <c r="G1422" t="inlineStr">
+        <is>
+          <t>503-558-2045</t>
+        </is>
+      </c>
+      <c r="H1422" t="inlineStr">
+        <is>
+          <t>Beaverton OR</t>
+        </is>
+      </c>
+      <c r="I1422" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1422" t="inlineStr">
+        <is>
+          <t>plumbing company Beaverton OR</t>
+        </is>
+      </c>
+      <c r="K1422" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1422" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1423">
+      <c r="A1423" t="inlineStr">
+        <is>
+          <t>Residential &amp; Commercial Plumbing Beaverton Plumbing</t>
+        </is>
+      </c>
+      <c r="B1423" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1423" t="inlineStr">
+        <is>
+          <t>beavertonplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1423" t="inlineStr">
+        <is>
+          <t>https://www.beavertonplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E1423" t="inlineStr">
+        <is>
+          <t>Improvements In</t>
+        </is>
+      </c>
+      <c r="F1423" t="inlineStr">
+        <is>
+          <t>joel@beavertonplumbing.com</t>
+        </is>
+      </c>
+      <c r="G1423" t="inlineStr">
+        <is>
+          <t>503-643-7619</t>
+        </is>
+      </c>
+      <c r="H1423" t="inlineStr">
+        <is>
+          <t>Beaverton OR</t>
+        </is>
+      </c>
+      <c r="I1423" t="n">
+        <v>80</v>
+      </c>
+      <c r="J1423" t="inlineStr">
+        <is>
+          <t>plumbing company Beaverton OR</t>
+        </is>
+      </c>
+      <c r="K1423" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1423" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:41 UTC (cycle 174)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1423"/>
+  <dimension ref="A1:L1428"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -83680,7 +83680,6 @@
           <t>https://cornelsplumbing.com/plumbing-services/beaverton-plumbers/</t>
         </is>
       </c>
-      <c r="E1422" t="inlineStr"/>
       <c r="F1422" t="inlineStr">
         <is>
           <t>contact@cornelsplumbing.com</t>
@@ -83770,6 +83769,298 @@
         </is>
       </c>
       <c r="L1423" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1424">
+      <c r="A1424" t="inlineStr">
+        <is>
+          <t>Home Roofing Solutions</t>
+        </is>
+      </c>
+      <c r="B1424" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1424" t="inlineStr">
+        <is>
+          <t>homeroofingsolutions.com</t>
+        </is>
+      </c>
+      <c r="D1424" t="inlineStr">
+        <is>
+          <t>https://homeroofingsolutions.com/areas-served/lewiston/</t>
+        </is>
+      </c>
+      <c r="E1424" t="inlineStr">
+        <is>
+          <t>Request Free</t>
+        </is>
+      </c>
+      <c r="F1424" t="inlineStr">
+        <is>
+          <t>info@homeroofingsolutions.com</t>
+        </is>
+      </c>
+      <c r="G1424" t="inlineStr">
+        <is>
+          <t>(207) 489-2904</t>
+        </is>
+      </c>
+      <c r="H1424" t="inlineStr">
+        <is>
+          <t>Lewiston ME</t>
+        </is>
+      </c>
+      <c r="I1424" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1424" t="inlineStr">
+        <is>
+          <t>roofer Lewiston ME</t>
+        </is>
+      </c>
+      <c r="K1424" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1424" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1425">
+      <c r="A1425" t="inlineStr">
+        <is>
+          <t>Overson Roofing</t>
+        </is>
+      </c>
+      <c r="B1425" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1425" t="inlineStr">
+        <is>
+          <t>oversonroofing.com</t>
+        </is>
+      </c>
+      <c r="D1425" t="inlineStr">
+        <is>
+          <t>https://oversonroofing.com/residential-roofers/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E1425" t="inlineStr">
+        <is>
+          <t>Which One</t>
+        </is>
+      </c>
+      <c r="F1425" t="inlineStr">
+        <is>
+          <t>info@oversonroofing.com</t>
+        </is>
+      </c>
+      <c r="G1425" t="inlineStr">
+        <is>
+          <t>(480) 470-6654</t>
+        </is>
+      </c>
+      <c r="H1425" t="inlineStr">
+        <is>
+          <t>Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="I1425" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1425" t="inlineStr">
+        <is>
+          <t>roof replacement Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="K1425" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1425" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1426">
+      <c r="A1426" t="inlineStr">
+        <is>
+          <t>Roof Repair Phoenix | Roofing Contractors AZ | Scott Roofing Company is a reputa</t>
+        </is>
+      </c>
+      <c r="B1426" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1426" t="inlineStr">
+        <is>
+          <t>scottroofingco.com</t>
+        </is>
+      </c>
+      <c r="D1426" t="inlineStr">
+        <is>
+          <t>https://scottroofingco.com/</t>
+        </is>
+      </c>
+      <c r="E1426" t="inlineStr">
+        <is>
+          <t>Jesse Scott</t>
+        </is>
+      </c>
+      <c r="F1426" t="inlineStr">
+        <is>
+          <t>kmcatee@scottroofingco.com</t>
+        </is>
+      </c>
+      <c r="G1426" t="inlineStr">
+        <is>
+          <t>(602) 442-7663</t>
+        </is>
+      </c>
+      <c r="H1426" t="inlineStr">
+        <is>
+          <t>Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="I1426" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1426" t="inlineStr">
+        <is>
+          <t>roof replacement Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="K1426" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1426" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1427">
+      <c r="A1427" t="inlineStr">
+        <is>
+          <t>Arizona Roofing and Restoration - Arizona's Top Roofing Company</t>
+        </is>
+      </c>
+      <c r="B1427" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1427" t="inlineStr">
+        <is>
+          <t>azroofpros.com</t>
+        </is>
+      </c>
+      <c r="D1427" t="inlineStr">
+        <is>
+          <t>https://azroofpros.com/roof-replacement-phoenix-az/</t>
+        </is>
+      </c>
+      <c r="E1427" t="inlineStr"/>
+      <c r="F1427" t="inlineStr">
+        <is>
+          <t>emailinfo@azroofpros.com</t>
+        </is>
+      </c>
+      <c r="G1427" t="inlineStr">
+        <is>
+          <t>602-931-9464</t>
+        </is>
+      </c>
+      <c r="H1427" t="inlineStr">
+        <is>
+          <t>Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="I1427" t="n">
+        <v>88</v>
+      </c>
+      <c r="J1427" t="inlineStr">
+        <is>
+          <t>roof replacement Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="K1427" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1427" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1428">
+      <c r="A1428" t="inlineStr">
+        <is>
+          <t>Phoenix Roofing &amp; Repair</t>
+        </is>
+      </c>
+      <c r="B1428" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1428" t="inlineStr">
+        <is>
+          <t>phoenixroofingandrepair.com</t>
+        </is>
+      </c>
+      <c r="D1428" t="inlineStr">
+        <is>
+          <t>https://phoenixroofingandrepair.com/</t>
+        </is>
+      </c>
+      <c r="E1428" t="inlineStr">
+        <is>
+          <t>Phoenix Roofing</t>
+        </is>
+      </c>
+      <c r="F1428" t="inlineStr">
+        <is>
+          <t>info@bestazroofers.com</t>
+        </is>
+      </c>
+      <c r="G1428" t="inlineStr"/>
+      <c r="H1428" t="inlineStr">
+        <is>
+          <t>Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="I1428" t="n">
+        <v>66</v>
+      </c>
+      <c r="J1428" t="inlineStr">
+        <is>
+          <t>roof replacement Phoenix AZ</t>
+        </is>
+      </c>
+      <c r="K1428" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1428" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:43 UTC (cycle 175)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1428"/>
+  <dimension ref="A1:L1431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -83975,7 +83975,6 @@
           <t>https://azroofpros.com/roof-replacement-phoenix-az/</t>
         </is>
       </c>
-      <c r="E1427" t="inlineStr"/>
       <c r="F1427" t="inlineStr">
         <is>
           <t>emailinfo@azroofpros.com</t>
@@ -84041,7 +84040,6 @@
           <t>info@bestazroofers.com</t>
         </is>
       </c>
-      <c r="G1428" t="inlineStr"/>
       <c r="H1428" t="inlineStr">
         <is>
           <t>Phoenix AZ</t>
@@ -84061,6 +84059,186 @@
         </is>
       </c>
       <c r="L1428" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1429">
+      <c r="A1429" t="inlineStr">
+        <is>
+          <t>F.H. Furr Plumbing, Heating, Air Conditioning &amp; Electrical</t>
+        </is>
+      </c>
+      <c r="B1429" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1429" t="inlineStr">
+        <is>
+          <t>fhfurr.com</t>
+        </is>
+      </c>
+      <c r="D1429" t="inlineStr">
+        <is>
+          <t>https://www.fhfurr.com/richmond/heating-services/furnace-services/</t>
+        </is>
+      </c>
+      <c r="E1429" t="inlineStr">
+        <is>
+          <t>Furr Difference</t>
+        </is>
+      </c>
+      <c r="F1429" t="inlineStr">
+        <is>
+          <t>customerservice@fhfurr.com</t>
+        </is>
+      </c>
+      <c r="G1429" t="inlineStr">
+        <is>
+          <t>(833) 858-7249</t>
+        </is>
+      </c>
+      <c r="H1429" t="inlineStr">
+        <is>
+          <t>Richmond VA</t>
+        </is>
+      </c>
+      <c r="I1429" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1429" t="inlineStr">
+        <is>
+          <t>furnace repair Richmond VA</t>
+        </is>
+      </c>
+      <c r="K1429" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1429" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1430">
+      <c r="A1430" t="inlineStr">
+        <is>
+          <t>Turtle Roofing®</t>
+        </is>
+      </c>
+      <c r="B1430" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1430" t="inlineStr">
+        <is>
+          <t>turtleroofing.com</t>
+        </is>
+      </c>
+      <c r="D1430" t="inlineStr">
+        <is>
+          <t>https://turtleroofing.com/omaha-ne/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E1430" t="inlineStr">
+        <is>
+          <t>Shell Protection</t>
+        </is>
+      </c>
+      <c r="F1430" t="inlineStr">
+        <is>
+          <t>info@turtleroofing.com</t>
+        </is>
+      </c>
+      <c r="G1430" t="inlineStr">
+        <is>
+          <t>(402) 430-1554</t>
+        </is>
+      </c>
+      <c r="H1430" t="inlineStr">
+        <is>
+          <t>Omaha NE</t>
+        </is>
+      </c>
+      <c r="I1430" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1430" t="inlineStr">
+        <is>
+          <t>roof replacement Omaha NE</t>
+        </is>
+      </c>
+      <c r="K1430" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1430" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1431">
+      <c r="A1431" t="inlineStr">
+        <is>
+          <t>Husker Roofing Omaha | Roofing Contractors Omaha, NE</t>
+        </is>
+      </c>
+      <c r="B1431" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1431" t="inlineStr">
+        <is>
+          <t>huskerroofing.com</t>
+        </is>
+      </c>
+      <c r="D1431" t="inlineStr">
+        <is>
+          <t>https://huskerroofing.com/roof-repair-omaha/</t>
+        </is>
+      </c>
+      <c r="E1431" t="inlineStr">
+        <is>
+          <t>Why Omaha</t>
+        </is>
+      </c>
+      <c r="F1431" t="inlineStr">
+        <is>
+          <t>contact@huskerroofing.com</t>
+        </is>
+      </c>
+      <c r="G1431" t="inlineStr">
+        <is>
+          <t>4025530200</t>
+        </is>
+      </c>
+      <c r="H1431" t="inlineStr">
+        <is>
+          <t>Omaha NE</t>
+        </is>
+      </c>
+      <c r="I1431" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1431" t="inlineStr">
+        <is>
+          <t>roof replacement Omaha NE</t>
+        </is>
+      </c>
+      <c r="K1431" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1431" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:44 UTC (cycle 176)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1431"/>
+  <dimension ref="A1:L1432"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -84244,6 +84244,66 @@
         </is>
       </c>
     </row>
+    <row r="1432">
+      <c r="A1432" t="inlineStr">
+        <is>
+          <t>Integrity Duct &amp; HVAC Services</t>
+        </is>
+      </c>
+      <c r="B1432" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1432" t="inlineStr">
+        <is>
+          <t>integrityductandhvacservices.com</t>
+        </is>
+      </c>
+      <c r="D1432" t="inlineStr">
+        <is>
+          <t>https://integrityductandhvacservices.com/ac-repair-alexandria-va/</t>
+        </is>
+      </c>
+      <c r="E1432" t="inlineStr">
+        <is>
+          <t>Integrity Duct</t>
+        </is>
+      </c>
+      <c r="F1432" t="inlineStr">
+        <is>
+          <t>hvacvalue4@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1432" t="inlineStr">
+        <is>
+          <t>(571) 351-7391</t>
+        </is>
+      </c>
+      <c r="H1432" t="inlineStr">
+        <is>
+          <t>Alexandria VA</t>
+        </is>
+      </c>
+      <c r="I1432" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1432" t="inlineStr">
+        <is>
+          <t>air conditioning repair Alexandria VA</t>
+        </is>
+      </c>
+      <c r="K1432" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1432" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:46 UTC (cycle 177)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1432"/>
+  <dimension ref="A1:L1439"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -84304,6 +84304,418 @@
         </is>
       </c>
     </row>
+    <row r="1433">
+      <c r="A1433" t="inlineStr">
+        <is>
+          <t>Las Vegas Water Experts</t>
+        </is>
+      </c>
+      <c r="B1433" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1433" t="inlineStr">
+        <is>
+          <t>lasvegaswaterexperts.com</t>
+        </is>
+      </c>
+      <c r="D1433" t="inlineStr">
+        <is>
+          <t>https://lasvegaswaterexperts.com/plumbing-drain-rooter-cleaning-north-las-vegas-nv/</t>
+        </is>
+      </c>
+      <c r="E1433" t="inlineStr"/>
+      <c r="F1433" t="inlineStr">
+        <is>
+          <t>lasvegaswaterexperts@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1433" t="inlineStr">
+        <is>
+          <t>702-577-5505</t>
+        </is>
+      </c>
+      <c r="H1433" t="inlineStr">
+        <is>
+          <t>North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I1433" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1433" t="inlineStr">
+        <is>
+          <t>drain cleaning service North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K1433" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1433" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1434">
+      <c r="A1434" t="inlineStr">
+        <is>
+          <t>Maroon Plumbing</t>
+        </is>
+      </c>
+      <c r="B1434" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1434" t="inlineStr">
+        <is>
+          <t>maroonplumbers.com</t>
+        </is>
+      </c>
+      <c r="D1434" t="inlineStr">
+        <is>
+          <t>https://www.maroonplumbers.com/sewer-repair-services-in-college-station/</t>
+        </is>
+      </c>
+      <c r="E1434" t="inlineStr">
+        <is>
+          <t>Join Our</t>
+        </is>
+      </c>
+      <c r="F1434" t="inlineStr">
+        <is>
+          <t>info@www.maroonplumbers.com</t>
+        </is>
+      </c>
+      <c r="G1434" t="inlineStr">
+        <is>
+          <t>(979) 985-3500</t>
+        </is>
+      </c>
+      <c r="H1434" t="inlineStr">
+        <is>
+          <t>College Station TX</t>
+        </is>
+      </c>
+      <c r="I1434" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1434" t="inlineStr">
+        <is>
+          <t>sewer repair College Station TX</t>
+        </is>
+      </c>
+      <c r="K1434" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1434" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1435">
+      <c r="A1435" t="inlineStr">
+        <is>
+          <t>Charleston Roof Pros</t>
+        </is>
+      </c>
+      <c r="B1435" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1435" t="inlineStr">
+        <is>
+          <t>charlestonroofpros.com</t>
+        </is>
+      </c>
+      <c r="D1435" t="inlineStr">
+        <is>
+          <t>https://charlestonroofpros.com/residential-roofing/</t>
+        </is>
+      </c>
+      <c r="E1435" t="inlineStr">
+        <is>
+          <t>Estimate Why</t>
+        </is>
+      </c>
+      <c r="F1435" t="inlineStr">
+        <is>
+          <t>contact@charlestonroofpros.com</t>
+        </is>
+      </c>
+      <c r="G1435" t="inlineStr">
+        <is>
+          <t>(304) 576-8709</t>
+        </is>
+      </c>
+      <c r="H1435" t="inlineStr">
+        <is>
+          <t>Charleston WV</t>
+        </is>
+      </c>
+      <c r="I1435" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1435" t="inlineStr">
+        <is>
+          <t>residential roofing company Charleston WV</t>
+        </is>
+      </c>
+      <c r="K1435" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1435" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1436">
+      <c r="A1436" t="inlineStr">
+        <is>
+          <t>Barker's</t>
+        </is>
+      </c>
+      <c r="B1436" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1436" t="inlineStr">
+        <is>
+          <t>barkerservices.com</t>
+        </is>
+      </c>
+      <c r="D1436" t="inlineStr">
+        <is>
+          <t>https://barkerservices.com/plumbing/sewer-lines/</t>
+        </is>
+      </c>
+      <c r="E1436" t="inlineStr">
+        <is>
+          <t>Service Barker</t>
+        </is>
+      </c>
+      <c r="F1436" t="inlineStr">
+        <is>
+          <t>service@barkerservices.com</t>
+        </is>
+      </c>
+      <c r="G1436" t="inlineStr">
+        <is>
+          <t>(979) 398-5194</t>
+        </is>
+      </c>
+      <c r="H1436" t="inlineStr">
+        <is>
+          <t>College Station TX</t>
+        </is>
+      </c>
+      <c r="I1436" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1436" t="inlineStr">
+        <is>
+          <t>sewer repair College Station TX</t>
+        </is>
+      </c>
+      <c r="K1436" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1436" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1437">
+      <c r="A1437" t="inlineStr">
+        <is>
+          <t>Larson Air &amp; Plumbing</t>
+        </is>
+      </c>
+      <c r="B1437" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1437" t="inlineStr">
+        <is>
+          <t>larsonairlv.com</t>
+        </is>
+      </c>
+      <c r="D1437" t="inlineStr">
+        <is>
+          <t>https://larsonairlv.com/plumbing-plumber-repair-las-vegas/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E1437" t="inlineStr">
+        <is>
+          <t>Plumbing Experts</t>
+        </is>
+      </c>
+      <c r="F1437" t="inlineStr">
+        <is>
+          <t>service@larsonairlv.com</t>
+        </is>
+      </c>
+      <c r="G1437" t="inlineStr">
+        <is>
+          <t>702-940-0733</t>
+        </is>
+      </c>
+      <c r="H1437" t="inlineStr">
+        <is>
+          <t>North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I1437" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1437" t="inlineStr">
+        <is>
+          <t>drain cleaning service North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K1437" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1437" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1438">
+      <c r="A1438" t="inlineStr">
+        <is>
+          <t>Truline General Contracting</t>
+        </is>
+      </c>
+      <c r="B1438" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1438" t="inlineStr">
+        <is>
+          <t>truline.org</t>
+        </is>
+      </c>
+      <c r="D1438" t="inlineStr">
+        <is>
+          <t>https://www.truline.org/locations/west-virginia/charleston/</t>
+        </is>
+      </c>
+      <c r="E1438" t="inlineStr">
+        <is>
+          <t>Kanawha Cou</t>
+        </is>
+      </c>
+      <c r="F1438" t="inlineStr">
+        <is>
+          <t>office@truline.org</t>
+        </is>
+      </c>
+      <c r="G1438" t="inlineStr">
+        <is>
+          <t>304-894-4642</t>
+        </is>
+      </c>
+      <c r="H1438" t="inlineStr">
+        <is>
+          <t>Charleston WV</t>
+        </is>
+      </c>
+      <c r="I1438" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1438" t="inlineStr">
+        <is>
+          <t>residential roofing company Charleston WV</t>
+        </is>
+      </c>
+      <c r="K1438" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1438" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1439">
+      <c r="A1439" t="inlineStr">
+        <is>
+          <t>Drain cleaning in North Las Vegas</t>
+        </is>
+      </c>
+      <c r="B1439" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1439" t="inlineStr">
+        <is>
+          <t>lasvegasplumbingspecialists.com</t>
+        </is>
+      </c>
+      <c r="D1439" t="inlineStr">
+        <is>
+          <t>https://lasvegasplumbingspecialists.com/locations/north-las-vegas-nv/drain-cleaning</t>
+        </is>
+      </c>
+      <c r="E1439" t="inlineStr"/>
+      <c r="F1439" t="inlineStr">
+        <is>
+          <t>info@lasvegasplumbingspecialists.com</t>
+        </is>
+      </c>
+      <c r="G1439" t="inlineStr">
+        <is>
+          <t>(725) 677-1071</t>
+        </is>
+      </c>
+      <c r="H1439" t="inlineStr">
+        <is>
+          <t>North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I1439" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1439" t="inlineStr">
+        <is>
+          <t>drain cleaning service North Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K1439" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1439" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:51 UTC (cycle 180)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1439"/>
+  <dimension ref="A1:L1441"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -84325,7 +84325,6 @@
           <t>https://lasvegaswaterexperts.com/plumbing-drain-rooter-cleaning-north-las-vegas-nv/</t>
         </is>
       </c>
-      <c r="E1433" t="inlineStr"/>
       <c r="F1433" t="inlineStr">
         <is>
           <t>lasvegaswaterexperts@gmail.com</t>
@@ -84681,7 +84680,6 @@
           <t>https://lasvegasplumbingspecialists.com/locations/north-las-vegas-nv/drain-cleaning</t>
         </is>
       </c>
-      <c r="E1439" t="inlineStr"/>
       <c r="F1439" t="inlineStr">
         <is>
           <t>info@lasvegasplumbingspecialists.com</t>
@@ -84711,6 +84709,122 @@
         </is>
       </c>
       <c r="L1439" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1440">
+      <c r="A1440" t="inlineStr">
+        <is>
+          <t>JR&amp;CO</t>
+        </is>
+      </c>
+      <c r="B1440" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1440" t="inlineStr">
+        <is>
+          <t>jrcousa.com</t>
+        </is>
+      </c>
+      <c r="D1440" t="inlineStr">
+        <is>
+          <t>https://jrcousa.com/cedar-rapids/</t>
+        </is>
+      </c>
+      <c r="E1440" t="inlineStr">
+        <is>
+          <t>New Ownership</t>
+        </is>
+      </c>
+      <c r="F1440" t="inlineStr">
+        <is>
+          <t>info@jrcousa.com</t>
+        </is>
+      </c>
+      <c r="G1440" t="inlineStr">
+        <is>
+          <t>(319) 360-3499</t>
+        </is>
+      </c>
+      <c r="H1440" t="inlineStr">
+        <is>
+          <t>Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="I1440" t="n">
+        <v>88</v>
+      </c>
+      <c r="J1440" t="inlineStr">
+        <is>
+          <t>roofer Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="K1440" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1440" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1441">
+      <c r="A1441" t="inlineStr">
+        <is>
+          <t>Darnell Construction</t>
+        </is>
+      </c>
+      <c r="B1441" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1441" t="inlineStr">
+        <is>
+          <t>darnellroofing.com</t>
+        </is>
+      </c>
+      <c r="D1441" t="inlineStr">
+        <is>
+          <t>https://darnellroofing.com/</t>
+        </is>
+      </c>
+      <c r="E1441" t="inlineStr"/>
+      <c r="F1441" t="inlineStr">
+        <is>
+          <t>darnellconstruction2004@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1441" t="inlineStr">
+        <is>
+          <t>319-378-4775</t>
+        </is>
+      </c>
+      <c r="H1441" t="inlineStr">
+        <is>
+          <t>Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="I1441" t="n">
+        <v>80</v>
+      </c>
+      <c r="J1441" t="inlineStr">
+        <is>
+          <t>roofer Cedar Rapids IA</t>
+        </is>
+      </c>
+      <c r="K1441" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1441" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:54 UTC (cycle 182)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1441"/>
+  <dimension ref="A1:L1442"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -84795,7 +84795,6 @@
           <t>https://darnellroofing.com/</t>
         </is>
       </c>
-      <c r="E1441" t="inlineStr"/>
       <c r="F1441" t="inlineStr">
         <is>
           <t>darnellconstruction2004@gmail.com</t>
@@ -84825,6 +84824,66 @@
         </is>
       </c>
       <c r="L1441" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1442">
+      <c r="A1442" t="inlineStr">
+        <is>
+          <t>Roof Repair Services in Salt Lake City, UT | Roof Doctor</t>
+        </is>
+      </c>
+      <c r="B1442" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1442" t="inlineStr">
+        <is>
+          <t>roofdoctorutah.com</t>
+        </is>
+      </c>
+      <c r="D1442" t="inlineStr">
+        <is>
+          <t>https://roofdoctorutah.com/service/roof-repairs/</t>
+        </is>
+      </c>
+      <c r="E1442" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F1442" t="inlineStr">
+        <is>
+          <t>info@roofdoctorutah.com</t>
+        </is>
+      </c>
+      <c r="G1442" t="inlineStr">
+        <is>
+          <t>(801) 512-3614</t>
+        </is>
+      </c>
+      <c r="H1442" t="inlineStr">
+        <is>
+          <t>Salt Lake City UT</t>
+        </is>
+      </c>
+      <c r="I1442" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1442" t="inlineStr">
+        <is>
+          <t>roof repair company Salt Lake City UT</t>
+        </is>
+      </c>
+      <c r="K1442" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1442" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:55 UTC (cycle 183)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1442"/>
+  <dimension ref="A1:L1445"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -84889,6 +84889,182 @@
         </is>
       </c>
     </row>
+    <row r="1443">
+      <c r="A1443" t="inlineStr">
+        <is>
+          <t>Golem Roofing</t>
+        </is>
+      </c>
+      <c r="B1443" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1443" t="inlineStr">
+        <is>
+          <t>golemroofing.com</t>
+        </is>
+      </c>
+      <c r="D1443" t="inlineStr">
+        <is>
+          <t>https://golemroofing.com/roofing-long-beach-ca/</t>
+        </is>
+      </c>
+      <c r="E1443" t="inlineStr">
+        <is>
+          <t>Long Beach</t>
+        </is>
+      </c>
+      <c r="F1443" t="inlineStr">
+        <is>
+          <t>info@golemroofing.com</t>
+        </is>
+      </c>
+      <c r="G1443" t="inlineStr">
+        <is>
+          <t>(562) 991-8165</t>
+        </is>
+      </c>
+      <c r="H1443" t="inlineStr">
+        <is>
+          <t>Long Beach CA</t>
+        </is>
+      </c>
+      <c r="I1443" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1443" t="inlineStr">
+        <is>
+          <t>roofing contractor Long Beach CA</t>
+        </is>
+      </c>
+      <c r="K1443" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1443" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" t="inlineStr">
+        <is>
+          <t>Green Bay Roofing</t>
+        </is>
+      </c>
+      <c r="B1444" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1444" t="inlineStr">
+        <is>
+          <t>gbroof.com</t>
+        </is>
+      </c>
+      <c r="D1444" t="inlineStr">
+        <is>
+          <t>https://gbroof.com/</t>
+        </is>
+      </c>
+      <c r="E1444" t="inlineStr"/>
+      <c r="F1444" t="inlineStr">
+        <is>
+          <t>adam@gbroof.com</t>
+        </is>
+      </c>
+      <c r="G1444" t="inlineStr">
+        <is>
+          <t>(920) 518-1879</t>
+        </is>
+      </c>
+      <c r="H1444" t="inlineStr">
+        <is>
+          <t>Green Bay WI</t>
+        </is>
+      </c>
+      <c r="I1444" t="n">
+        <v>94</v>
+      </c>
+      <c r="J1444" t="inlineStr">
+        <is>
+          <t>roofing contractor Green Bay WI</t>
+        </is>
+      </c>
+      <c r="K1444" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1444" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" t="inlineStr">
+        <is>
+          <t>Pierce Roofing</t>
+        </is>
+      </c>
+      <c r="B1445" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1445" t="inlineStr">
+        <is>
+          <t>greenbayroofers.com</t>
+        </is>
+      </c>
+      <c r="D1445" t="inlineStr">
+        <is>
+          <t>https://www.greenbayroofers.com/</t>
+        </is>
+      </c>
+      <c r="E1445" t="inlineStr">
+        <is>
+          <t>Pierce Roofing</t>
+        </is>
+      </c>
+      <c r="F1445" t="inlineStr">
+        <is>
+          <t>pierceroofing01@aol.com</t>
+        </is>
+      </c>
+      <c r="G1445" t="inlineStr">
+        <is>
+          <t>(920) 609-8304</t>
+        </is>
+      </c>
+      <c r="H1445" t="inlineStr">
+        <is>
+          <t>Green Bay WI</t>
+        </is>
+      </c>
+      <c r="I1445" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1445" t="inlineStr">
+        <is>
+          <t>roofing contractor Green Bay WI</t>
+        </is>
+      </c>
+      <c r="K1445" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1445" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:57 UTC (cycle 184)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1445"/>
+  <dimension ref="A1:L1450"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -84970,7 +84970,6 @@
           <t>https://gbroof.com/</t>
         </is>
       </c>
-      <c r="E1444" t="inlineStr"/>
       <c r="F1444" t="inlineStr">
         <is>
           <t>adam@gbroof.com</t>
@@ -85060,6 +85059,298 @@
         </is>
       </c>
       <c r="L1445" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" t="inlineStr">
+        <is>
+          <t>Northglenn Heating &amp; AC</t>
+        </is>
+      </c>
+      <c r="B1446" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1446" t="inlineStr">
+        <is>
+          <t>northglennheatingac.com</t>
+        </is>
+      </c>
+      <c r="D1446" t="inlineStr">
+        <is>
+          <t>https://www.northglennheatingac.com/locations/aurora/air-conditioning-repair-aurora/</t>
+        </is>
+      </c>
+      <c r="E1446" t="inlineStr"/>
+      <c r="F1446" t="inlineStr">
+        <is>
+          <t>service@northglennheatingac.com</t>
+        </is>
+      </c>
+      <c r="G1446" t="inlineStr">
+        <is>
+          <t>303-452-4146</t>
+        </is>
+      </c>
+      <c r="H1446" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I1446" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1446" t="inlineStr">
+        <is>
+          <t>air conditioning repair Aurora CO</t>
+        </is>
+      </c>
+      <c r="K1446" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1446" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" t="inlineStr">
+        <is>
+          <t>Elkhorn Heating, Air Conditioning, Plumbing &amp; Electrical</t>
+        </is>
+      </c>
+      <c r="B1447" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1447" t="inlineStr">
+        <is>
+          <t>myelkhorn.com</t>
+        </is>
+      </c>
+      <c r="D1447" t="inlineStr">
+        <is>
+          <t>https://myelkhorn.com/lakewood-heating-services/</t>
+        </is>
+      </c>
+      <c r="E1447" t="inlineStr"/>
+      <c r="F1447" t="inlineStr">
+        <is>
+          <t>info@myelkhorn.com</t>
+        </is>
+      </c>
+      <c r="G1447" t="inlineStr">
+        <is>
+          <t>720-615-0098</t>
+        </is>
+      </c>
+      <c r="H1447" t="inlineStr">
+        <is>
+          <t>Lakewood CO</t>
+        </is>
+      </c>
+      <c r="I1447" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1447" t="inlineStr">
+        <is>
+          <t>furnace repair Lakewood CO</t>
+        </is>
+      </c>
+      <c r="K1447" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1447" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" t="inlineStr">
+        <is>
+          <t>Absolute Plumbing, Electrical, Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B1448" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1448" t="inlineStr">
+        <is>
+          <t>absolutefix.com</t>
+        </is>
+      </c>
+      <c r="D1448" t="inlineStr">
+        <is>
+          <t>https://absolutefix.com/service-area/air-conditioning-repair/aurora-co/</t>
+        </is>
+      </c>
+      <c r="E1448" t="inlineStr">
+        <is>
+          <t>Why Aurora</t>
+        </is>
+      </c>
+      <c r="F1448" t="inlineStr">
+        <is>
+          <t>booking@absolutefix.com</t>
+        </is>
+      </c>
+      <c r="G1448" t="inlineStr">
+        <is>
+          <t>(720) 807-5715</t>
+        </is>
+      </c>
+      <c r="H1448" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I1448" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1448" t="inlineStr">
+        <is>
+          <t>air conditioning repair Aurora CO</t>
+        </is>
+      </c>
+      <c r="K1448" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1448" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" t="inlineStr">
+        <is>
+          <t>Drain Cleaning Services | Clog Removal | New Braunfels, TX</t>
+        </is>
+      </c>
+      <c r="B1449" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1449" t="inlineStr">
+        <is>
+          <t>culpepperplumbingservice.com</t>
+        </is>
+      </c>
+      <c r="D1449" t="inlineStr">
+        <is>
+          <t>https://www.culpepperplumbingservice.com/drain-cleaning-services</t>
+        </is>
+      </c>
+      <c r="E1449" t="inlineStr">
+        <is>
+          <t>Professional Drain</t>
+        </is>
+      </c>
+      <c r="F1449" t="inlineStr">
+        <is>
+          <t>culpepperplumbing@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G1449" t="inlineStr">
+        <is>
+          <t>(830) 214-6640</t>
+        </is>
+      </c>
+      <c r="H1449" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I1449" t="n">
+        <v>94</v>
+      </c>
+      <c r="J1449" t="inlineStr">
+        <is>
+          <t>drain cleaning service New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K1449" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1449" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" t="inlineStr">
+        <is>
+          <t>Bonita Lake Plumbers</t>
+        </is>
+      </c>
+      <c r="B1450" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1450" t="inlineStr">
+        <is>
+          <t>emergencyplumbinglakewoodco.com</t>
+        </is>
+      </c>
+      <c r="D1450" t="inlineStr">
+        <is>
+          <t>https://emergencyplumbinglakewoodco.com/services/furnace-repair-replacement/</t>
+        </is>
+      </c>
+      <c r="E1450" t="inlineStr">
+        <is>
+          <t>Detail Information</t>
+        </is>
+      </c>
+      <c r="F1450" t="inlineStr">
+        <is>
+          <t>bonitalakeplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1450" t="inlineStr">
+        <is>
+          <t>(720) 783-2999</t>
+        </is>
+      </c>
+      <c r="H1450" t="inlineStr">
+        <is>
+          <t>Lakewood CO</t>
+        </is>
+      </c>
+      <c r="I1450" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1450" t="inlineStr">
+        <is>
+          <t>furnace repair Lakewood CO</t>
+        </is>
+      </c>
+      <c r="K1450" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1450" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 22:58 UTC (cycle 185)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1450"/>
+  <dimension ref="A1:L1453"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -85085,7 +85085,6 @@
           <t>https://www.northglennheatingac.com/locations/aurora/air-conditioning-repair-aurora/</t>
         </is>
       </c>
-      <c r="E1446" t="inlineStr"/>
       <c r="F1446" t="inlineStr">
         <is>
           <t>service@northglennheatingac.com</t>
@@ -85141,7 +85140,6 @@
           <t>https://myelkhorn.com/lakewood-heating-services/</t>
         </is>
       </c>
-      <c r="E1447" t="inlineStr"/>
       <c r="F1447" t="inlineStr">
         <is>
           <t>info@myelkhorn.com</t>
@@ -85351,6 +85349,186 @@
         </is>
       </c>
       <c r="L1450" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" t="inlineStr">
+        <is>
+          <t>Atlanta Roofing Specialists</t>
+        </is>
+      </c>
+      <c r="B1451" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1451" t="inlineStr">
+        <is>
+          <t>atlantaroofingspecialists.com</t>
+        </is>
+      </c>
+      <c r="D1451" t="inlineStr">
+        <is>
+          <t>https://atlantaroofingspecialists.com/</t>
+        </is>
+      </c>
+      <c r="E1451" t="inlineStr">
+        <is>
+          <t>Metro Atlanta</t>
+        </is>
+      </c>
+      <c r="F1451" t="inlineStr">
+        <is>
+          <t>customerservice@myatlantaroof.com</t>
+        </is>
+      </c>
+      <c r="G1451" t="inlineStr">
+        <is>
+          <t>(770) 419-2222</t>
+        </is>
+      </c>
+      <c r="H1451" t="inlineStr">
+        <is>
+          <t>Atlanta GA</t>
+        </is>
+      </c>
+      <c r="I1451" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1451" t="inlineStr">
+        <is>
+          <t>roofing contractor Atlanta GA</t>
+        </is>
+      </c>
+      <c r="K1451" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1451" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1452">
+      <c r="A1452" t="inlineStr">
+        <is>
+          <t>Country Suburban Heating &amp; Air Conditioning, Inc.</t>
+        </is>
+      </c>
+      <c r="B1452" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1452" t="inlineStr">
+        <is>
+          <t>countrysuburbanhvac.com</t>
+        </is>
+      </c>
+      <c r="D1452" t="inlineStr">
+        <is>
+          <t>https://www.countrysuburbanhvac.com/utica-ny-heating-air-conditioning-contractor/</t>
+        </is>
+      </c>
+      <c r="E1452" t="inlineStr">
+        <is>
+          <t>General Philip</t>
+        </is>
+      </c>
+      <c r="F1452" t="inlineStr">
+        <is>
+          <t>hg.countrysuburban@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1452" t="inlineStr">
+        <is>
+          <t>315-735-5300</t>
+        </is>
+      </c>
+      <c r="H1452" t="inlineStr">
+        <is>
+          <t>Utica NY</t>
+        </is>
+      </c>
+      <c r="I1452" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1452" t="inlineStr">
+        <is>
+          <t>heating and cooling company Utica NY</t>
+        </is>
+      </c>
+      <c r="K1452" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1452" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" t="inlineStr">
+        <is>
+          <t>ONE STOP HEATING AND COOLING</t>
+        </is>
+      </c>
+      <c r="B1453" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1453" t="inlineStr">
+        <is>
+          <t>onestopheatingandcooling.co</t>
+        </is>
+      </c>
+      <c r="D1453" t="inlineStr">
+        <is>
+          <t>https://onestopheatingandcooling.co/</t>
+        </is>
+      </c>
+      <c r="E1453" t="inlineStr">
+        <is>
+          <t>All Makes</t>
+        </is>
+      </c>
+      <c r="F1453" t="inlineStr">
+        <is>
+          <t>mirzetkendic@hotmail.com</t>
+        </is>
+      </c>
+      <c r="G1453" t="inlineStr">
+        <is>
+          <t>(315) 749-5605</t>
+        </is>
+      </c>
+      <c r="H1453" t="inlineStr">
+        <is>
+          <t>Utica NY</t>
+        </is>
+      </c>
+      <c r="I1453" t="n">
+        <v>88</v>
+      </c>
+      <c r="J1453" t="inlineStr">
+        <is>
+          <t>heating and cooling company Utica NY</t>
+        </is>
+      </c>
+      <c r="K1453" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1453" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 23:00 UTC (cycle 186)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1453"/>
+  <dimension ref="A1:L1455"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -85534,6 +85534,118 @@
         </is>
       </c>
     </row>
+    <row r="1454">
+      <c r="A1454" t="inlineStr">
+        <is>
+          <t>Lincoln Drain</t>
+        </is>
+      </c>
+      <c r="B1454" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1454" t="inlineStr">
+        <is>
+          <t>lincolndrain.com</t>
+        </is>
+      </c>
+      <c r="D1454" t="inlineStr">
+        <is>
+          <t>https://www.lincolndrain.com/</t>
+        </is>
+      </c>
+      <c r="E1454" t="inlineStr"/>
+      <c r="F1454" t="inlineStr">
+        <is>
+          <t>contact@omahadrainservice.com</t>
+        </is>
+      </c>
+      <c r="G1454" t="inlineStr">
+        <is>
+          <t>(402) 237-2088</t>
+        </is>
+      </c>
+      <c r="H1454" t="inlineStr">
+        <is>
+          <t>Lincoln NE</t>
+        </is>
+      </c>
+      <c r="I1454" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1454" t="inlineStr">
+        <is>
+          <t>drain cleaning service Lincoln NE</t>
+        </is>
+      </c>
+      <c r="K1454" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1454" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" t="inlineStr">
+        <is>
+          <t>Jim &amp; Sons Plumbing &amp; Rooter | Plumbers in Riverside &amp; Inland Empire, CA</t>
+        </is>
+      </c>
+      <c r="B1455" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1455" t="inlineStr">
+        <is>
+          <t>jimandsonsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1455" t="inlineStr">
+        <is>
+          <t>https://jimandsonsplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E1455" t="inlineStr"/>
+      <c r="F1455" t="inlineStr">
+        <is>
+          <t>service@jimandsonsplumbing.com</t>
+        </is>
+      </c>
+      <c r="G1455" t="inlineStr">
+        <is>
+          <t>(951) 248-9134</t>
+        </is>
+      </c>
+      <c r="H1455" t="inlineStr">
+        <is>
+          <t>Riverside CA</t>
+        </is>
+      </c>
+      <c r="I1455" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1455" t="inlineStr">
+        <is>
+          <t>plumber Riverside CA</t>
+        </is>
+      </c>
+      <c r="K1455" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1455" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 23:01 UTC (cycle 187)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1455"/>
+  <dimension ref="A1:L1462"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -85555,7 +85555,6 @@
           <t>https://www.lincolndrain.com/</t>
         </is>
       </c>
-      <c r="E1454" t="inlineStr"/>
       <c r="F1454" t="inlineStr">
         <is>
           <t>contact@omahadrainservice.com</t>
@@ -85611,7 +85610,6 @@
           <t>https://jimandsonsplumbing.com/</t>
         </is>
       </c>
-      <c r="E1455" t="inlineStr"/>
       <c r="F1455" t="inlineStr">
         <is>
           <t>service@jimandsonsplumbing.com</t>
@@ -85641,6 +85639,422 @@
         </is>
       </c>
       <c r="L1455" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" t="inlineStr">
+        <is>
+          <t>Peach 3 Group NY</t>
+        </is>
+      </c>
+      <c r="B1456" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1456" t="inlineStr">
+        <is>
+          <t>peach3group.com</t>
+        </is>
+      </c>
+      <c r="D1456" t="inlineStr">
+        <is>
+          <t>https://peach3group.com/services/roofing-contractors-new-rochelle-ny/</t>
+        </is>
+      </c>
+      <c r="E1456" t="inlineStr">
+        <is>
+          <t>New Rochelle</t>
+        </is>
+      </c>
+      <c r="F1456" t="inlineStr">
+        <is>
+          <t>info@peach3group.com</t>
+        </is>
+      </c>
+      <c r="G1456" t="inlineStr">
+        <is>
+          <t>(914) 451-8300</t>
+        </is>
+      </c>
+      <c r="H1456" t="inlineStr">
+        <is>
+          <t>New Rochelle NY</t>
+        </is>
+      </c>
+      <c r="I1456" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1456" t="inlineStr">
+        <is>
+          <t>roof replacement New Rochelle NY</t>
+        </is>
+      </c>
+      <c r="K1456" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1456" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" t="inlineStr">
+        <is>
+          <t>Torrance Elite Roofing: Top Quality Commercial &amp; Residential Roofing Solutions i</t>
+        </is>
+      </c>
+      <c r="B1457" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1457" t="inlineStr">
+        <is>
+          <t>torranceeliteroofing.com</t>
+        </is>
+      </c>
+      <c r="D1457" t="inlineStr">
+        <is>
+          <t>https://www.torranceeliteroofing.com/roof-repair</t>
+        </is>
+      </c>
+      <c r="E1457" t="inlineStr">
+        <is>
+          <t>Solutions We</t>
+        </is>
+      </c>
+      <c r="F1457" t="inlineStr">
+        <is>
+          <t>info@torranceeliteroofing.com</t>
+        </is>
+      </c>
+      <c r="G1457" t="inlineStr">
+        <is>
+          <t>(310) 361-1321</t>
+        </is>
+      </c>
+      <c r="H1457" t="inlineStr">
+        <is>
+          <t>Torrance CA</t>
+        </is>
+      </c>
+      <c r="I1457" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1457" t="inlineStr">
+        <is>
+          <t>roof repair company Torrance CA</t>
+        </is>
+      </c>
+      <c r="K1457" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1457" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" t="inlineStr">
+        <is>
+          <t>Choose Essential</t>
+        </is>
+      </c>
+      <c r="B1458" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1458" t="inlineStr">
+        <is>
+          <t>chooseessential.com</t>
+        </is>
+      </c>
+      <c r="D1458" t="inlineStr">
+        <is>
+          <t>https://chooseessential.com/service-areas/torrance-ca/</t>
+        </is>
+      </c>
+      <c r="E1458" t="inlineStr"/>
+      <c r="F1458" t="inlineStr">
+        <is>
+          <t>support@chooseessential.com</t>
+        </is>
+      </c>
+      <c r="G1458" t="inlineStr">
+        <is>
+          <t>818-823-1158</t>
+        </is>
+      </c>
+      <c r="H1458" t="inlineStr">
+        <is>
+          <t>Torrance CA</t>
+        </is>
+      </c>
+      <c r="I1458" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1458" t="inlineStr">
+        <is>
+          <t>roof repair company Torrance CA</t>
+        </is>
+      </c>
+      <c r="K1458" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1458" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" t="inlineStr">
+        <is>
+          <t>Royal Roofing Company</t>
+        </is>
+      </c>
+      <c r="B1459" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1459" t="inlineStr">
+        <is>
+          <t>royalroofing.com</t>
+        </is>
+      </c>
+      <c r="D1459" t="inlineStr">
+        <is>
+          <t>https://royalroofing.com/roof-repair-torrance-ca/</t>
+        </is>
+      </c>
+      <c r="E1459" t="inlineStr">
+        <is>
+          <t>Owners Steve</t>
+        </is>
+      </c>
+      <c r="F1459" t="inlineStr">
+        <is>
+          <t>service@royalroofing.com</t>
+        </is>
+      </c>
+      <c r="G1459" t="inlineStr">
+        <is>
+          <t>562-928-1200</t>
+        </is>
+      </c>
+      <c r="H1459" t="inlineStr">
+        <is>
+          <t>Torrance CA</t>
+        </is>
+      </c>
+      <c r="I1459" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1459" t="inlineStr">
+        <is>
+          <t>roof repair company Torrance CA</t>
+        </is>
+      </c>
+      <c r="K1459" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1459" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" t="inlineStr">
+        <is>
+          <t>Torrance Roofing Masters</t>
+        </is>
+      </c>
+      <c r="B1460" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1460" t="inlineStr">
+        <is>
+          <t>torranceroofingmasters.com</t>
+        </is>
+      </c>
+      <c r="D1460" t="inlineStr">
+        <is>
+          <t>https://torranceroofingmasters.com/</t>
+        </is>
+      </c>
+      <c r="E1460" t="inlineStr">
+        <is>
+          <t>South Bay</t>
+        </is>
+      </c>
+      <c r="F1460" t="inlineStr">
+        <is>
+          <t>info@torranceroofingmasters.com</t>
+        </is>
+      </c>
+      <c r="G1460" t="inlineStr">
+        <is>
+          <t>(424) 492-2022</t>
+        </is>
+      </c>
+      <c r="H1460" t="inlineStr">
+        <is>
+          <t>Torrance CA</t>
+        </is>
+      </c>
+      <c r="I1460" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1460" t="inlineStr">
+        <is>
+          <t>roof repair company Torrance CA</t>
+        </is>
+      </c>
+      <c r="K1460" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1460" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" t="inlineStr">
+        <is>
+          <t>CMS Roofing | Roofing Contractors in Bowling Green &amp; Owensboro, KY</t>
+        </is>
+      </c>
+      <c r="B1461" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1461" t="inlineStr">
+        <is>
+          <t>cmsroofing.com</t>
+        </is>
+      </c>
+      <c r="D1461" t="inlineStr">
+        <is>
+          <t>https://www.cmsroofing.com/</t>
+        </is>
+      </c>
+      <c r="E1461" t="inlineStr">
+        <is>
+          <t>Why Property</t>
+        </is>
+      </c>
+      <c r="F1461" t="inlineStr">
+        <is>
+          <t>office@cmsroofing.com</t>
+        </is>
+      </c>
+      <c r="G1461" t="inlineStr">
+        <is>
+          <t>270-843-5405</t>
+        </is>
+      </c>
+      <c r="H1461" t="inlineStr">
+        <is>
+          <t>Bowling Green KY</t>
+        </is>
+      </c>
+      <c r="I1461" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1461" t="inlineStr">
+        <is>
+          <t>roofer Bowling Green KY</t>
+        </is>
+      </c>
+      <c r="K1461" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1461" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" t="inlineStr">
+        <is>
+          <t>Best West Roofing Los Angeles | Roofing, Repair &amp; Replacements</t>
+        </is>
+      </c>
+      <c r="B1462" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1462" t="inlineStr">
+        <is>
+          <t>thebestwestroofing.com</t>
+        </is>
+      </c>
+      <c r="D1462" t="inlineStr">
+        <is>
+          <t>https://thebestwestroofing.com/cities/torrance-roof-repair/</t>
+        </is>
+      </c>
+      <c r="E1462" t="inlineStr">
+        <is>
+          <t>Why Choose</t>
+        </is>
+      </c>
+      <c r="F1462" t="inlineStr">
+        <is>
+          <t>info@thebestwestroofing.com</t>
+        </is>
+      </c>
+      <c r="G1462" t="inlineStr">
+        <is>
+          <t>(323) 304-3580</t>
+        </is>
+      </c>
+      <c r="H1462" t="inlineStr">
+        <is>
+          <t>Torrance CA</t>
+        </is>
+      </c>
+      <c r="I1462" t="n">
+        <v>88</v>
+      </c>
+      <c r="J1462" t="inlineStr">
+        <is>
+          <t>roof repair company Torrance CA</t>
+        </is>
+      </c>
+      <c r="K1462" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1462" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 23:03 UTC (cycle 188)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1462"/>
+  <dimension ref="A1:L1465"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -85785,7 +85785,6 @@
           <t>https://chooseessential.com/service-areas/torrance-ca/</t>
         </is>
       </c>
-      <c r="E1458" t="inlineStr"/>
       <c r="F1458" t="inlineStr">
         <is>
           <t>support@chooseessential.com</t>
@@ -86055,6 +86054,186 @@
         </is>
       </c>
       <c r="L1462" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" t="inlineStr">
+        <is>
+          <t>Roofing Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="B1463" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1463" t="inlineStr">
+        <is>
+          <t>roofingsterlingheights.com</t>
+        </is>
+      </c>
+      <c r="D1463" t="inlineStr">
+        <is>
+          <t>https://www.roofingsterlingheights.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E1463" t="inlineStr">
+        <is>
+          <t>Style Most</t>
+        </is>
+      </c>
+      <c r="F1463" t="inlineStr">
+        <is>
+          <t>admin@roofingsterlingheights.com</t>
+        </is>
+      </c>
+      <c r="G1463" t="inlineStr">
+        <is>
+          <t>(586) 331-0594</t>
+        </is>
+      </c>
+      <c r="H1463" t="inlineStr">
+        <is>
+          <t>Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="I1463" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1463" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="K1463" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1463" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1464">
+      <c r="A1464" t="inlineStr">
+        <is>
+          <t>Metal Roofing Sterling Heights MI | The Roof Specialists</t>
+        </is>
+      </c>
+      <c r="B1464" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1464" t="inlineStr">
+        <is>
+          <t>theroofspecialistsmi.com</t>
+        </is>
+      </c>
+      <c r="D1464" t="inlineStr">
+        <is>
+          <t>https://theroofspecialistsmi.com/services/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E1464" t="inlineStr">
+        <is>
+          <t>Sterling Heights</t>
+        </is>
+      </c>
+      <c r="F1464" t="inlineStr">
+        <is>
+          <t>theroofspecialistmi@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1464" t="inlineStr">
+        <is>
+          <t>(586) 765-7663</t>
+        </is>
+      </c>
+      <c r="H1464" t="inlineStr">
+        <is>
+          <t>Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="I1464" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1464" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="K1464" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1464" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" t="inlineStr">
+        <is>
+          <t>Metal Roofing Sterling Heights, MI</t>
+        </is>
+      </c>
+      <c r="B1465" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1465" t="inlineStr">
+        <is>
+          <t>eliteroofingmi.com</t>
+        </is>
+      </c>
+      <c r="D1465" t="inlineStr">
+        <is>
+          <t>https://www.eliteroofingmi.com/cities/guides/sterling-heights/metal-roofing.html</t>
+        </is>
+      </c>
+      <c r="E1465" t="inlineStr">
+        <is>
+          <t>Sterling Heights</t>
+        </is>
+      </c>
+      <c r="F1465" t="inlineStr">
+        <is>
+          <t>info@eliteroofing.com</t>
+        </is>
+      </c>
+      <c r="G1465" t="inlineStr">
+        <is>
+          <t>(555) 123-4567</t>
+        </is>
+      </c>
+      <c r="H1465" t="inlineStr">
+        <is>
+          <t>Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="I1465" t="n">
+        <v>86</v>
+      </c>
+      <c r="J1465" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="K1465" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1465" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 23:04 UTC (cycle 189)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1465"/>
+  <dimension ref="A1:L1470"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -86239,6 +86239,290 @@
         </is>
       </c>
     </row>
+    <row r="1466">
+      <c r="A1466" t="inlineStr">
+        <is>
+          <t>Smurl HVAC</t>
+        </is>
+      </c>
+      <c r="B1466" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1466" t="inlineStr">
+        <is>
+          <t>smurlhvac.com</t>
+        </is>
+      </c>
+      <c r="D1466" t="inlineStr">
+        <is>
+          <t>https://www.smurlhvac.com/</t>
+        </is>
+      </c>
+      <c r="E1466" t="inlineStr"/>
+      <c r="F1466" t="inlineStr">
+        <is>
+          <t>smurlhvacinfo@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1466" t="inlineStr">
+        <is>
+          <t>(570) 344-2870</t>
+        </is>
+      </c>
+      <c r="H1466" t="inlineStr">
+        <is>
+          <t>Scranton PA</t>
+        </is>
+      </c>
+      <c r="I1466" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1466" t="inlineStr">
+        <is>
+          <t>HVAC contractor Scranton PA</t>
+        </is>
+      </c>
+      <c r="K1466" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1466" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" t="inlineStr">
+        <is>
+          <t>VaughnPlumbingHvac</t>
+        </is>
+      </c>
+      <c r="B1467" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1467" t="inlineStr">
+        <is>
+          <t>vaughnplumbinghvac.com</t>
+        </is>
+      </c>
+      <c r="D1467" t="inlineStr">
+        <is>
+          <t>https://vaughnplumbinghvac.com/heating-cooling-in-nashua-nh/</t>
+        </is>
+      </c>
+      <c r="E1467" t="inlineStr">
+        <is>
+          <t>Owner Meet</t>
+        </is>
+      </c>
+      <c r="F1467" t="inlineStr">
+        <is>
+          <t>admin@plexlogo.com</t>
+        </is>
+      </c>
+      <c r="G1467" t="inlineStr">
+        <is>
+          <t>978-866-6040</t>
+        </is>
+      </c>
+      <c r="H1467" t="inlineStr">
+        <is>
+          <t>Nashua NH</t>
+        </is>
+      </c>
+      <c r="I1467" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1467" t="inlineStr">
+        <is>
+          <t>furnace repair Nashua NH</t>
+        </is>
+      </c>
+      <c r="K1467" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1467" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" t="inlineStr">
+        <is>
+          <t>Mayhem Roofing</t>
+        </is>
+      </c>
+      <c r="B1468" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1468" t="inlineStr">
+        <is>
+          <t>mayhemroofing.com</t>
+        </is>
+      </c>
+      <c r="D1468" t="inlineStr">
+        <is>
+          <t>https://www.mayhemroofing.com/metal-roofs/</t>
+        </is>
+      </c>
+      <c r="E1468" t="inlineStr"/>
+      <c r="F1468" t="inlineStr">
+        <is>
+          <t>info@mayhemroofing.com</t>
+        </is>
+      </c>
+      <c r="G1468" t="inlineStr">
+        <is>
+          <t>(803) 233-8023</t>
+        </is>
+      </c>
+      <c r="H1468" t="inlineStr">
+        <is>
+          <t>Columbia SC</t>
+        </is>
+      </c>
+      <c r="I1468" t="n">
+        <v>98</v>
+      </c>
+      <c r="J1468" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Columbia SC</t>
+        </is>
+      </c>
+      <c r="K1468" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1468" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" t="inlineStr">
+        <is>
+          <t>Taylor Made Custom Coatings, LLC</t>
+        </is>
+      </c>
+      <c r="B1469" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1469" t="inlineStr">
+        <is>
+          <t>metalroofcolumbiasc.com</t>
+        </is>
+      </c>
+      <c r="D1469" t="inlineStr">
+        <is>
+          <t>https://www.metalroofcolumbiasc.com/</t>
+        </is>
+      </c>
+      <c r="E1469" t="inlineStr"/>
+      <c r="F1469" t="inlineStr">
+        <is>
+          <t>moreinfo@metalroofcolumbiasc.com</t>
+        </is>
+      </c>
+      <c r="G1469" t="inlineStr">
+        <is>
+          <t>(803) 234-5985</t>
+        </is>
+      </c>
+      <c r="H1469" t="inlineStr">
+        <is>
+          <t>Columbia SC</t>
+        </is>
+      </c>
+      <c r="I1469" t="n">
+        <v>96</v>
+      </c>
+      <c r="J1469" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Columbia SC</t>
+        </is>
+      </c>
+      <c r="K1469" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1469" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" t="inlineStr">
+        <is>
+          <t>AC Repair, Installation</t>
+        </is>
+      </c>
+      <c r="B1470" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1470" t="inlineStr">
+        <is>
+          <t>thegasconnectionhvac.com</t>
+        </is>
+      </c>
+      <c r="D1470" t="inlineStr">
+        <is>
+          <t>https://www.thegasconnectionhvac.com/</t>
+        </is>
+      </c>
+      <c r="E1470" t="inlineStr"/>
+      <c r="F1470" t="inlineStr">
+        <is>
+          <t>info@thegasconnectionnh.com</t>
+        </is>
+      </c>
+      <c r="G1470" t="inlineStr">
+        <is>
+          <t>(603) 889-1161</t>
+        </is>
+      </c>
+      <c r="H1470" t="inlineStr">
+        <is>
+          <t>Nashua NH</t>
+        </is>
+      </c>
+      <c r="I1470" t="n">
+        <v>78</v>
+      </c>
+      <c r="J1470" t="inlineStr">
+        <is>
+          <t>furnace repair Nashua NH</t>
+        </is>
+      </c>
+      <c r="K1470" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1470" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 23:08 UTC (cycle 192)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1470"/>
+  <dimension ref="A1:L1476"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -86260,7 +86260,6 @@
           <t>https://www.smurlhvac.com/</t>
         </is>
       </c>
-      <c r="E1466" t="inlineStr"/>
       <c r="F1466" t="inlineStr">
         <is>
           <t>smurlhvacinfo@gmail.com</t>
@@ -86376,7 +86375,6 @@
           <t>https://www.mayhemroofing.com/metal-roofs/</t>
         </is>
       </c>
-      <c r="E1468" t="inlineStr"/>
       <c r="F1468" t="inlineStr">
         <is>
           <t>info@mayhemroofing.com</t>
@@ -86432,7 +86430,6 @@
           <t>https://www.metalroofcolumbiasc.com/</t>
         </is>
       </c>
-      <c r="E1469" t="inlineStr"/>
       <c r="F1469" t="inlineStr">
         <is>
           <t>moreinfo@metalroofcolumbiasc.com</t>
@@ -86488,7 +86485,6 @@
           <t>https://www.thegasconnectionhvac.com/</t>
         </is>
       </c>
-      <c r="E1470" t="inlineStr"/>
       <c r="F1470" t="inlineStr">
         <is>
           <t>info@thegasconnectionnh.com</t>
@@ -86518,6 +86514,358 @@
         </is>
       </c>
       <c r="L1470" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" t="inlineStr">
+        <is>
+          <t>Roofing Company in St. George, UT | Red Rock Roofing</t>
+        </is>
+      </c>
+      <c r="B1471" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1471" t="inlineStr">
+        <is>
+          <t>stgeorgeroofingutah.com</t>
+        </is>
+      </c>
+      <c r="D1471" t="inlineStr">
+        <is>
+          <t>https://stgeorgeroofingutah.com/</t>
+        </is>
+      </c>
+      <c r="E1471" t="inlineStr">
+        <is>
+          <t>Washington County</t>
+        </is>
+      </c>
+      <c r="F1471" t="inlineStr">
+        <is>
+          <t>redrockroofingutah@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1471" t="inlineStr">
+        <is>
+          <t>435-222-7141</t>
+        </is>
+      </c>
+      <c r="H1471" t="inlineStr">
+        <is>
+          <t>St George UT</t>
+        </is>
+      </c>
+      <c r="I1471" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1471" t="inlineStr">
+        <is>
+          <t>roof replacement St George UT</t>
+        </is>
+      </c>
+      <c r="K1471" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1471" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1472">
+      <c r="A1472" t="inlineStr">
+        <is>
+          <t>HVAC | Fredericksburg, VA | 540-373-3004</t>
+        </is>
+      </c>
+      <c r="B1472" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1472" t="inlineStr">
+        <is>
+          <t>mainsheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D1472" t="inlineStr">
+        <is>
+          <t>https://www.mainsheatingandair.com/</t>
+        </is>
+      </c>
+      <c r="E1472" t="inlineStr">
+        <is>
+          <t>Team Reviews</t>
+        </is>
+      </c>
+      <c r="F1472" t="inlineStr">
+        <is>
+          <t>mainsheatingandaircond@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G1472" t="inlineStr">
+        <is>
+          <t>540-373-3004</t>
+        </is>
+      </c>
+      <c r="H1472" t="inlineStr">
+        <is>
+          <t>Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="I1472" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1472" t="inlineStr">
+        <is>
+          <t>AC installation Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="K1472" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1472" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" t="inlineStr">
+        <is>
+          <t>AC Installation | Fredericksburg, VA</t>
+        </is>
+      </c>
+      <c r="B1473" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1473" t="inlineStr">
+        <is>
+          <t>veteransdoitall.com</t>
+        </is>
+      </c>
+      <c r="D1473" t="inlineStr">
+        <is>
+          <t>https://www.veteransdoitall.com/ac-installation</t>
+        </is>
+      </c>
+      <c r="E1473" t="inlineStr"/>
+      <c r="F1473" t="inlineStr">
+        <is>
+          <t>info@veteransdoitall.com</t>
+        </is>
+      </c>
+      <c r="G1473" t="inlineStr">
+        <is>
+          <t>(540) 237-1606</t>
+        </is>
+      </c>
+      <c r="H1473" t="inlineStr">
+        <is>
+          <t>Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="I1473" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1473" t="inlineStr">
+        <is>
+          <t>AC installation Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="K1473" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1473" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1474">
+      <c r="A1474" t="inlineStr">
+        <is>
+          <t>All Climate Mechanical - Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B1474" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1474" t="inlineStr">
+        <is>
+          <t>allclimatehvac.com</t>
+        </is>
+      </c>
+      <c r="D1474" t="inlineStr">
+        <is>
+          <t>https://allclimatehvac.com/furnace-repair-bloomington-mn/</t>
+        </is>
+      </c>
+      <c r="E1474" t="inlineStr"/>
+      <c r="F1474" t="inlineStr">
+        <is>
+          <t>info@allclimatehvac.com</t>
+        </is>
+      </c>
+      <c r="G1474" t="inlineStr">
+        <is>
+          <t>763-548-8095</t>
+        </is>
+      </c>
+      <c r="H1474" t="inlineStr">
+        <is>
+          <t>Bloomington MN</t>
+        </is>
+      </c>
+      <c r="I1474" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1474" t="inlineStr">
+        <is>
+          <t>furnace repair Bloomington MN</t>
+        </is>
+      </c>
+      <c r="K1474" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1474" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1475">
+      <c r="A1475" t="inlineStr">
+        <is>
+          <t>Durham Roofing Company, Save Up to $1,000 Off a New Roof | Feazel</t>
+        </is>
+      </c>
+      <c r="B1475" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1475" t="inlineStr">
+        <is>
+          <t>feazelinc.com</t>
+        </is>
+      </c>
+      <c r="D1475" t="inlineStr">
+        <is>
+          <t>https://www.feazelinc.com/durham-nc/</t>
+        </is>
+      </c>
+      <c r="E1475" t="inlineStr">
+        <is>
+          <t>Continue Reading</t>
+        </is>
+      </c>
+      <c r="F1475" t="inlineStr">
+        <is>
+          <t>info@feazelinc.com</t>
+        </is>
+      </c>
+      <c r="G1475" t="inlineStr">
+        <is>
+          <t>(614) 350-3213</t>
+        </is>
+      </c>
+      <c r="H1475" t="inlineStr">
+        <is>
+          <t>Durham NC</t>
+        </is>
+      </c>
+      <c r="I1475" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1475" t="inlineStr">
+        <is>
+          <t>roof replacement Durham NC</t>
+        </is>
+      </c>
+      <c r="K1475" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1475" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1476">
+      <c r="A1476" t="inlineStr">
+        <is>
+          <t>Kasper Mechanical</t>
+        </is>
+      </c>
+      <c r="B1476" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1476" t="inlineStr">
+        <is>
+          <t>kaspermechanical.com</t>
+        </is>
+      </c>
+      <c r="D1476" t="inlineStr">
+        <is>
+          <t>https://www.kaspermechanical.com/air-conditioner-replacement/</t>
+        </is>
+      </c>
+      <c r="E1476" t="inlineStr">
+        <is>
+          <t>Bradley Edmonds</t>
+        </is>
+      </c>
+      <c r="F1476" t="inlineStr">
+        <is>
+          <t>info@www.kaspermechanical.com</t>
+        </is>
+      </c>
+      <c r="G1476" t="inlineStr">
+        <is>
+          <t>540-300-7917</t>
+        </is>
+      </c>
+      <c r="H1476" t="inlineStr">
+        <is>
+          <t>Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="I1476" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1476" t="inlineStr">
+        <is>
+          <t>AC installation Fredericksburg VA</t>
+        </is>
+      </c>
+      <c r="K1476" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1476" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 23:10 UTC (cycle 193)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1476"/>
+  <dimension ref="A1:L1479"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -86660,7 +86660,6 @@
           <t>https://www.veteransdoitall.com/ac-installation</t>
         </is>
       </c>
-      <c r="E1473" t="inlineStr"/>
       <c r="F1473" t="inlineStr">
         <is>
           <t>info@veteransdoitall.com</t>
@@ -86716,7 +86715,6 @@
           <t>https://allclimatehvac.com/furnace-repair-bloomington-mn/</t>
         </is>
       </c>
-      <c r="E1474" t="inlineStr"/>
       <c r="F1474" t="inlineStr">
         <is>
           <t>info@allclimatehvac.com</t>
@@ -86866,6 +86864,182 @@
         </is>
       </c>
       <c r="L1476" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1477">
+      <c r="A1477" t="inlineStr">
+        <is>
+          <t>Richmond, VA Roofing Contractor</t>
+        </is>
+      </c>
+      <c r="B1477" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1477" t="inlineStr">
+        <is>
+          <t>absoluteroof.co</t>
+        </is>
+      </c>
+      <c r="D1477" t="inlineStr">
+        <is>
+          <t>https://absoluteroof.co/locations/richmond-virginia</t>
+        </is>
+      </c>
+      <c r="E1477" t="inlineStr">
+        <is>
+          <t>Roofing Materials</t>
+        </is>
+      </c>
+      <c r="F1477" t="inlineStr">
+        <is>
+          <t>info@absoluteroof.co</t>
+        </is>
+      </c>
+      <c r="G1477" t="inlineStr">
+        <is>
+          <t>(844) 522-7658</t>
+        </is>
+      </c>
+      <c r="H1477" t="inlineStr">
+        <is>
+          <t>Richmond VA</t>
+        </is>
+      </c>
+      <c r="I1477" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1477" t="inlineStr">
+        <is>
+          <t>roof repair company Richmond VA</t>
+        </is>
+      </c>
+      <c r="K1477" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1477" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1478">
+      <c r="A1478" t="inlineStr">
+        <is>
+          <t>Emergency Plumber | Manchester, NH | Twins Plumbing and Heating Inc.</t>
+        </is>
+      </c>
+      <c r="B1478" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1478" t="inlineStr">
+        <is>
+          <t>twinsph.com</t>
+        </is>
+      </c>
+      <c r="D1478" t="inlineStr">
+        <is>
+          <t>https://www.twinsph.com/emergency-plumber</t>
+        </is>
+      </c>
+      <c r="E1478" t="inlineStr"/>
+      <c r="F1478" t="inlineStr">
+        <is>
+          <t>service@twinsph.com</t>
+        </is>
+      </c>
+      <c r="G1478" t="inlineStr">
+        <is>
+          <t>(603) 450-8946</t>
+        </is>
+      </c>
+      <c r="H1478" t="inlineStr">
+        <is>
+          <t>Manchester NH</t>
+        </is>
+      </c>
+      <c r="I1478" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1478" t="inlineStr">
+        <is>
+          <t>emergency plumber Manchester NH</t>
+        </is>
+      </c>
+      <c r="K1478" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1478" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1479">
+      <c r="A1479" t="inlineStr">
+        <is>
+          <t>Evergreen Roofing</t>
+        </is>
+      </c>
+      <c r="B1479" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1479" t="inlineStr">
+        <is>
+          <t>evergreenroofingva.com</t>
+        </is>
+      </c>
+      <c r="D1479" t="inlineStr">
+        <is>
+          <t>https://evergreenroofingva.com/locations/richmond/</t>
+        </is>
+      </c>
+      <c r="E1479" t="inlineStr">
+        <is>
+          <t>Send Request</t>
+        </is>
+      </c>
+      <c r="F1479" t="inlineStr">
+        <is>
+          <t>info@evergreenroofingva.com</t>
+        </is>
+      </c>
+      <c r="G1479" t="inlineStr">
+        <is>
+          <t>(804) 238-7837</t>
+        </is>
+      </c>
+      <c r="H1479" t="inlineStr">
+        <is>
+          <t>Richmond VA</t>
+        </is>
+      </c>
+      <c r="I1479" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1479" t="inlineStr">
+        <is>
+          <t>roof repair company Richmond VA</t>
+        </is>
+      </c>
+      <c r="K1479" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1479" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 23:11 UTC (cycle 194)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1479"/>
+  <dimension ref="A1:L1484"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -86950,7 +86950,6 @@
           <t>https://www.twinsph.com/emergency-plumber</t>
         </is>
       </c>
-      <c r="E1478" t="inlineStr"/>
       <c r="F1478" t="inlineStr">
         <is>
           <t>service@twinsph.com</t>
@@ -87040,6 +87039,302 @@
         </is>
       </c>
       <c r="L1479" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1480">
+      <c r="A1480" t="inlineStr">
+        <is>
+          <t>Northpoint Roofing</t>
+        </is>
+      </c>
+      <c r="B1480" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1480" t="inlineStr">
+        <is>
+          <t>northpointroofing.com</t>
+        </is>
+      </c>
+      <c r="D1480" t="inlineStr">
+        <is>
+          <t>https://www.northpointroofing.com/service-areas/nashua-nh/residential-roofing/</t>
+        </is>
+      </c>
+      <c r="E1480" t="inlineStr">
+        <is>
+          <t>New Hampshire</t>
+        </is>
+      </c>
+      <c r="F1480" t="inlineStr">
+        <is>
+          <t>customerservice@northpointroofing.com</t>
+        </is>
+      </c>
+      <c r="G1480" t="inlineStr">
+        <is>
+          <t>603-497-9500</t>
+        </is>
+      </c>
+      <c r="H1480" t="inlineStr">
+        <is>
+          <t>Nashua NH</t>
+        </is>
+      </c>
+      <c r="I1480" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1480" t="inlineStr">
+        <is>
+          <t>residential roofing company Nashua NH</t>
+        </is>
+      </c>
+      <c r="K1480" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1480" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1481">
+      <c r="A1481" t="inlineStr">
+        <is>
+          <t>Cabezon Roofing</t>
+        </is>
+      </c>
+      <c r="B1481" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1481" t="inlineStr">
+        <is>
+          <t>cabezonroofing.com</t>
+        </is>
+      </c>
+      <c r="D1481" t="inlineStr">
+        <is>
+          <t>https://cabezonroofing.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E1481" t="inlineStr">
+        <is>
+          <t>Keep Readi</t>
+        </is>
+      </c>
+      <c r="F1481" t="inlineStr">
+        <is>
+          <t>randy@cabezonroofing.com</t>
+        </is>
+      </c>
+      <c r="G1481" t="inlineStr">
+        <is>
+          <t>(505)-221-4628</t>
+        </is>
+      </c>
+      <c r="H1481" t="inlineStr">
+        <is>
+          <t>Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="I1481" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1481" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="K1481" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1481" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1482">
+      <c r="A1482" t="inlineStr">
+        <is>
+          <t>Metal Roofing Company in Albuquerque, NM | Sunshine Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B1482" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1482" t="inlineStr">
+        <is>
+          <t>sunshine-roofingllc.com</t>
+        </is>
+      </c>
+      <c r="D1482" t="inlineStr">
+        <is>
+          <t>https://sunshine-roofingllc.com/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E1482" t="inlineStr">
+        <is>
+          <t>Years Of</t>
+        </is>
+      </c>
+      <c r="F1482" t="inlineStr">
+        <is>
+          <t>info@sunshine-roofingllc.com</t>
+        </is>
+      </c>
+      <c r="G1482" t="inlineStr">
+        <is>
+          <t>(505) 572-0287</t>
+        </is>
+      </c>
+      <c r="H1482" t="inlineStr">
+        <is>
+          <t>Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="I1482" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1482" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="K1482" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1482" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1483">
+      <c r="A1483" t="inlineStr">
+        <is>
+          <t>Plumbers in Fargo, ND | NorthStar Plumbing &amp; Drain Cleaning</t>
+        </is>
+      </c>
+      <c r="B1483" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1483" t="inlineStr">
+        <is>
+          <t>northstarplumbingnd.com</t>
+        </is>
+      </c>
+      <c r="D1483" t="inlineStr">
+        <is>
+          <t>https://www.northstarplumbingnd.com/</t>
+        </is>
+      </c>
+      <c r="E1483" t="inlineStr"/>
+      <c r="F1483" t="inlineStr">
+        <is>
+          <t>northstarplumbingnd@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1483" t="inlineStr">
+        <is>
+          <t>(701) 367-9592</t>
+        </is>
+      </c>
+      <c r="H1483" t="inlineStr">
+        <is>
+          <t>Fargo ND</t>
+        </is>
+      </c>
+      <c r="I1483" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1483" t="inlineStr">
+        <is>
+          <t>plumber Fargo ND</t>
+        </is>
+      </c>
+      <c r="K1483" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1483" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1484">
+      <c r="A1484" t="inlineStr">
+        <is>
+          <t>Rock Construction</t>
+        </is>
+      </c>
+      <c r="B1484" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1484" t="inlineStr">
+        <is>
+          <t>rockconstructionnm.com</t>
+        </is>
+      </c>
+      <c r="D1484" t="inlineStr">
+        <is>
+          <t>https://rockconstructionnm.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E1484" t="inlineStr">
+        <is>
+          <t>Advanced Protective</t>
+        </is>
+      </c>
+      <c r="F1484" t="inlineStr">
+        <is>
+          <t>tj@rockconstructionnm.com</t>
+        </is>
+      </c>
+      <c r="G1484" t="inlineStr">
+        <is>
+          <t>(505) 220-8553</t>
+        </is>
+      </c>
+      <c r="H1484" t="inlineStr">
+        <is>
+          <t>Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="I1484" t="n">
+        <v>84</v>
+      </c>
+      <c r="J1484" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="K1484" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1484" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 23:14 UTC (cycle 196)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1484"/>
+  <dimension ref="A1:L1487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -87245,7 +87245,6 @@
           <t>https://www.northstarplumbingnd.com/</t>
         </is>
       </c>
-      <c r="E1483" t="inlineStr"/>
       <c r="F1483" t="inlineStr">
         <is>
           <t>northstarplumbingnd@gmail.com</t>
@@ -87335,6 +87334,186 @@
         </is>
       </c>
       <c r="L1484" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1485">
+      <c r="A1485" t="inlineStr">
+        <is>
+          <t>Best HVAC Company in Boston, MA - Trusted Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B1485" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1485" t="inlineStr">
+        <is>
+          <t>bostonairsolutions.com</t>
+        </is>
+      </c>
+      <c r="D1485" t="inlineStr">
+        <is>
+          <t>https://www.bostonairsolutions.com/</t>
+        </is>
+      </c>
+      <c r="E1485" t="inlineStr">
+        <is>
+          <t>Homeowner We</t>
+        </is>
+      </c>
+      <c r="F1485" t="inlineStr">
+        <is>
+          <t>info@bostonairsolutions.com</t>
+        </is>
+      </c>
+      <c r="G1485" t="inlineStr">
+        <is>
+          <t>(617) 752-0854</t>
+        </is>
+      </c>
+      <c r="H1485" t="inlineStr">
+        <is>
+          <t>Boston MA</t>
+        </is>
+      </c>
+      <c r="I1485" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1485" t="inlineStr">
+        <is>
+          <t>heating and cooling company Boston MA</t>
+        </is>
+      </c>
+      <c r="K1485" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1485" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1486">
+      <c r="A1486" t="inlineStr">
+        <is>
+          <t>Boston HVAC Contractors: Heating &amp; Air Conditioning Inc.</t>
+        </is>
+      </c>
+      <c r="B1486" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1486" t="inlineStr">
+        <is>
+          <t>bostonhvac.net</t>
+        </is>
+      </c>
+      <c r="D1486" t="inlineStr">
+        <is>
+          <t>https://www.bostonhvac.net/</t>
+        </is>
+      </c>
+      <c r="E1486" t="inlineStr">
+        <is>
+          <t>Air Conditioning</t>
+        </is>
+      </c>
+      <c r="F1486" t="inlineStr">
+        <is>
+          <t>info@bostonhvaccontractors.com</t>
+        </is>
+      </c>
+      <c r="G1486" t="inlineStr">
+        <is>
+          <t>(617) 634-0731</t>
+        </is>
+      </c>
+      <c r="H1486" t="inlineStr">
+        <is>
+          <t>Boston MA</t>
+        </is>
+      </c>
+      <c r="I1486" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1486" t="inlineStr">
+        <is>
+          <t>heating and cooling company Boston MA</t>
+        </is>
+      </c>
+      <c r="K1486" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1486" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1487">
+      <c r="A1487" t="inlineStr">
+        <is>
+          <t>Boston Heating &amp; Air Conditioning | Trusted HVAC Services</t>
+        </is>
+      </c>
+      <c r="B1487" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1487" t="inlineStr">
+        <is>
+          <t>b-hvac.com</t>
+        </is>
+      </c>
+      <c r="D1487" t="inlineStr">
+        <is>
+          <t>https://www.b-hvac.com/</t>
+        </is>
+      </c>
+      <c r="E1487" t="inlineStr">
+        <is>
+          <t>Day Service</t>
+        </is>
+      </c>
+      <c r="F1487" t="inlineStr">
+        <is>
+          <t>info@b-hvac.com</t>
+        </is>
+      </c>
+      <c r="G1487" t="inlineStr">
+        <is>
+          <t>(617) 315-3698</t>
+        </is>
+      </c>
+      <c r="H1487" t="inlineStr">
+        <is>
+          <t>Boston MA</t>
+        </is>
+      </c>
+      <c r="I1487" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1487" t="inlineStr">
+        <is>
+          <t>heating and cooling company Boston MA</t>
+        </is>
+      </c>
+      <c r="K1487" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1487" t="inlineStr">
         <is>
           <t>2026-09-06</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-06 23:19 UTC (cycle 199)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1487"/>
+  <dimension ref="A1:L1490"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -87519,6 +87519,186 @@
         </is>
       </c>
     </row>
+    <row r="1488">
+      <c r="A1488" t="inlineStr">
+        <is>
+          <t>Emergency Plumber St Charles MO | Warrior Sewer and Drain</t>
+        </is>
+      </c>
+      <c r="B1488" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1488" t="inlineStr">
+        <is>
+          <t>warriordrain.com</t>
+        </is>
+      </c>
+      <c r="D1488" t="inlineStr">
+        <is>
+          <t>https://warriordrain.com/emergency-plumber-st-charles-mo</t>
+        </is>
+      </c>
+      <c r="E1488" t="inlineStr">
+        <is>
+          <t>St Charles</t>
+        </is>
+      </c>
+      <c r="F1488" t="inlineStr">
+        <is>
+          <t>myally@warriordrain.com</t>
+        </is>
+      </c>
+      <c r="G1488" t="inlineStr">
+        <is>
+          <t>636 498-2686</t>
+        </is>
+      </c>
+      <c r="H1488" t="inlineStr">
+        <is>
+          <t>St Charles MO</t>
+        </is>
+      </c>
+      <c r="I1488" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1488" t="inlineStr">
+        <is>
+          <t>emergency plumber St Charles MO</t>
+        </is>
+      </c>
+      <c r="K1488" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1488" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1489">
+      <c r="A1489" t="inlineStr">
+        <is>
+          <t>Berry Good Heating and Air</t>
+        </is>
+      </c>
+      <c r="B1489" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1489" t="inlineStr">
+        <is>
+          <t>berrygoodheatingandair.com</t>
+        </is>
+      </c>
+      <c r="D1489" t="inlineStr">
+        <is>
+          <t>https://berrygoodheatingandair.com/ac-repair-atlanta/</t>
+        </is>
+      </c>
+      <c r="E1489" t="inlineStr">
+        <is>
+          <t>Berry Good</t>
+        </is>
+      </c>
+      <c r="F1489" t="inlineStr">
+        <is>
+          <t>customerservice@berrygoodheatingandair.com</t>
+        </is>
+      </c>
+      <c r="G1489" t="inlineStr">
+        <is>
+          <t>770-990-6809</t>
+        </is>
+      </c>
+      <c r="H1489" t="inlineStr">
+        <is>
+          <t>Atlanta GA</t>
+        </is>
+      </c>
+      <c r="I1489" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1489" t="inlineStr">
+        <is>
+          <t>air conditioning repair Atlanta GA</t>
+        </is>
+      </c>
+      <c r="K1489" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1489" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1490">
+      <c r="A1490" t="inlineStr">
+        <is>
+          <t>Empire HVAC</t>
+        </is>
+      </c>
+      <c r="B1490" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1490" t="inlineStr">
+        <is>
+          <t>empirehvac.com</t>
+        </is>
+      </c>
+      <c r="D1490" t="inlineStr">
+        <is>
+          <t>https://empirehvac.com/hvac-services-atlanta-ga/air-conditioning-services/ac-repair-maintenance/</t>
+        </is>
+      </c>
+      <c r="E1490" t="inlineStr">
+        <is>
+          <t>Conditioning Our</t>
+        </is>
+      </c>
+      <c r="F1490" t="inlineStr">
+        <is>
+          <t>forms@empirehvac.com</t>
+        </is>
+      </c>
+      <c r="G1490" t="inlineStr">
+        <is>
+          <t>404-294-0900</t>
+        </is>
+      </c>
+      <c r="H1490" t="inlineStr">
+        <is>
+          <t>Atlanta GA</t>
+        </is>
+      </c>
+      <c r="I1490" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1490" t="inlineStr">
+        <is>
+          <t>air conditioning repair Atlanta GA</t>
+        </is>
+      </c>
+      <c r="K1490" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1490" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-06 23:20 UTC (cycle 200)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1490"/>
+  <dimension ref="A1:L1493"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -87699,6 +87699,186 @@
         </is>
       </c>
     </row>
+    <row r="1491">
+      <c r="A1491" t="inlineStr">
+        <is>
+          <t>Contractor Starter Theme</t>
+        </is>
+      </c>
+      <c r="B1491" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1491" t="inlineStr">
+        <is>
+          <t>greatstateroof.com</t>
+        </is>
+      </c>
+      <c r="D1491" t="inlineStr">
+        <is>
+          <t>https://greatstateroof.com/roofing/rock-hill-sc/</t>
+        </is>
+      </c>
+      <c r="E1491" t="inlineStr">
+        <is>
+          <t>Keep Reading</t>
+        </is>
+      </c>
+      <c r="F1491" t="inlineStr">
+        <is>
+          <t>office@greatstateroof.com</t>
+        </is>
+      </c>
+      <c r="G1491" t="inlineStr">
+        <is>
+          <t>704-389-9985</t>
+        </is>
+      </c>
+      <c r="H1491" t="inlineStr">
+        <is>
+          <t>Rock Hill SC</t>
+        </is>
+      </c>
+      <c r="I1491" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1491" t="inlineStr">
+        <is>
+          <t>residential roofing company Rock Hill SC</t>
+        </is>
+      </c>
+      <c r="K1491" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1491" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1492">
+      <c r="A1492" t="inlineStr">
+        <is>
+          <t>Eastern Oak Roofing</t>
+        </is>
+      </c>
+      <c r="B1492" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1492" t="inlineStr">
+        <is>
+          <t>easternoakroofing.com</t>
+        </is>
+      </c>
+      <c r="D1492" t="inlineStr">
+        <is>
+          <t>https://easternoakroofing.com/rock-hill/</t>
+        </is>
+      </c>
+      <c r="E1492" t="inlineStr">
+        <is>
+          <t>Rock Hill</t>
+        </is>
+      </c>
+      <c r="F1492" t="inlineStr">
+        <is>
+          <t>easternoakroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1492" t="inlineStr">
+        <is>
+          <t>704-669-8218</t>
+        </is>
+      </c>
+      <c r="H1492" t="inlineStr">
+        <is>
+          <t>Rock Hill SC</t>
+        </is>
+      </c>
+      <c r="I1492" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1492" t="inlineStr">
+        <is>
+          <t>residential roofing company Rock Hill SC</t>
+        </is>
+      </c>
+      <c r="K1492" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1492" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="1493">
+      <c r="A1493" t="inlineStr">
+        <is>
+          <t>Rock Hill Roofing</t>
+        </is>
+      </c>
+      <c r="B1493" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1493" t="inlineStr">
+        <is>
+          <t>rockhillroofing.net</t>
+        </is>
+      </c>
+      <c r="D1493" t="inlineStr">
+        <is>
+          <t>https://rockhillroofing.net/residential-roofing.html</t>
+        </is>
+      </c>
+      <c r="E1493" t="inlineStr">
+        <is>
+          <t>Common Roofing</t>
+        </is>
+      </c>
+      <c r="F1493" t="inlineStr">
+        <is>
+          <t>info@rockhillroofing.net</t>
+        </is>
+      </c>
+      <c r="G1493" t="inlineStr">
+        <is>
+          <t>(803) 590-1409</t>
+        </is>
+      </c>
+      <c r="H1493" t="inlineStr">
+        <is>
+          <t>Rock Hill SC</t>
+        </is>
+      </c>
+      <c r="I1493" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1493" t="inlineStr">
+        <is>
+          <t>residential roofing company Rock Hill SC</t>
+        </is>
+      </c>
+      <c r="K1493" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1493" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 03:23 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1493"/>
+  <dimension ref="A1:P1493"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -439,6 +439,10 @@
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="9" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="34" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,6 +506,26 @@
           <t>Date Found</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Audit PDF</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Audit Status</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Emailed At</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Email Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -562,6 +586,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>audits/audit_savannahroofingexperts.com.pdf</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -617,6 +651,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>audits/audit_honoluluplumbingpro.com.pdf</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -677,6 +721,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>audits/audit_kortedoesitall.com.pdf</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -737,6 +791,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>failed: RuntimeError: PDF text never mentions fortwayneplumbingpro.com or 'Fort Wayne Plumbing Pro' - it may be a generic or wrong-company report</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -792,6 +851,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>audits/audit_mastersheatcool.com.pdf</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -850,6 +919,16 @@
       <c r="L7" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>audits/audit_theheatpumpstore.com.pdf</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 03:33 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -791,9 +791,14 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>audits/audit_fortwayneplumbingpro.com.pdf</t>
+        </is>
+      </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>failed: RuntimeError: PDF text never mentions fortwayneplumbingpro.com or 'Fort Wayne Plumbing Pro' - it may be a generic or wrong-company report</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -991,6 +996,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>audits/audit_aceroofingga.com.pdf</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1051,6 +1066,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>audits/audit_precisionroofingusa.com.pdf</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1111,6 +1136,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>failed: RuntimeError: PDF text never mentions coastalroofga.com or 'Metal Roofing in Savannah, GA | Commercial &amp; Residential | CRG' - it may be a generic or wrong-company report</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1171,6 +1201,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>audits/audit_stevesplumbinghawaii.com.pdf</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1224,6 +1264,16 @@
       <c r="L12" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>audits/audit_crowleyplumbingandheatinginc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 03:43 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -1136,9 +1136,14 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>audits/audit_coastalroofga.com.pdf</t>
+        </is>
+      </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>failed: RuntimeError: PDF text never mentions coastalroofga.com or 'Metal Roofing in Savannah, GA | Commercial &amp; Residential | CRG' - it may be a generic or wrong-company report</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -1336,6 +1341,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>audits/audit_talyaroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1391,6 +1406,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>audits/audit_endurancewh.com.pdf</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1451,6 +1476,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>audits/audit_rightwaymechanicalco.com.pdf</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1511,6 +1546,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>audits/audit_lakewoodheatpumps.com.pdf</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1564,6 +1609,16 @@
       <c r="L17" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>audits/audit_ba-hvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 03:53 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -1681,6 +1681,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>audits/audit_gvexteriors.com.pdf</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1741,6 +1751,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>audits/audit_instantroofer.com.pdf</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1801,6 +1821,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>audits/audit_southavenacrepair.com.pdf</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1861,6 +1891,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>audits/audit_trentonroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1921,6 +1961,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>audits/audit_homeimprovementewing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1974,6 +2024,16 @@
       <c r="L23" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>audits/audit_mckeeroofingpa.com.pdf</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 04:03 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -2091,6 +2091,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>audits/audit_champaignil.gov.pdf</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2146,6 +2156,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>audits/audit_montvilleroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2206,6 +2226,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>audits/audit_surpriseplumbers.co.pdf</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2266,6 +2296,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>audits/audit_idahofallsheatingandcooling.com.pdf</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2326,6 +2366,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>audits/audit_rsandrews.com.pdf</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2379,6 +2429,16 @@
       <c r="L29" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>audits/audit_magicmensd.com.pdf</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 04:13 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -2501,6 +2501,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>audits/audit_miracleplumbingaz.com.pdf</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2561,6 +2571,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>audits/audit_bigfootheating.com.pdf</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2621,6 +2641,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>audits/audit_theplumberguy.com.pdf</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2676,6 +2706,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>audits/audit_azevedoplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2736,6 +2776,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>audits/audit_bskcsoilandseptic.com.pdf</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2794,6 +2844,16 @@
       <c r="L35" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>audits/audit_sprinterheating.com.pdf</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 04:23 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -2916,6 +2916,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>audits/audit_ryanroofinglawrence.com.pdf</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2976,6 +2986,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>audits/audit_morgilloroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3036,6 +3056,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>audits/audit_acmesewerdraincleaning.com.pdf</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3096,6 +3126,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>audits/audit_gmrmetalroofsny.com.pdf</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3156,6 +3196,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>audits/audit_978plumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3214,6 +3264,16 @@
       <c r="L41" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>audits/audit_rivercitypros.com.pdf</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 04:33 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -3331,6 +3331,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>audits/audit_justcalldc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3386,6 +3396,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>audits/audit_metalroofsyracuse.com.pdf</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3441,6 +3461,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>audits/audit_metalroofmemphis.com.pdf</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3501,6 +3531,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>audits/audit_proline-roofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -3561,6 +3601,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>audits/audit_erscontractor.com.pdf</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3619,6 +3669,16 @@
       <c r="L47" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>audits/audit_deanroofs.com.pdf</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 04:43 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -3741,6 +3741,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>audits/audit_allproplumbers.com.pdf</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3801,6 +3811,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>audits/audit_happyroof.com.pdf</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3861,6 +3881,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>audits/audit_roofersbrooklynny.com.pdf</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3916,6 +3946,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>audits/audit_tommysplumbing.net.pdf</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3976,6 +4016,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>audits/audit_rightnowheatcool.com.pdf</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4034,6 +4084,16 @@
       <c r="L53" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>audits/audit_luckyairandplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 04:53 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -4151,6 +4151,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>audits/audit_rivercityheatingandair.net.pdf</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4211,6 +4221,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>audits/audit_heat-pump-installation-elizabeth.aeshvacnj.com.pdf</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4266,6 +4286,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>audits/audit_triplecrownplumbingco.com.pdf</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4326,6 +4356,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>audits/audit_autumnairbirmingham.com.pdf</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4386,6 +4426,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>audits/audit_heavenlythroneplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -4444,6 +4494,16 @@
       <c r="L59" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>audits/audit_dimaticcontrol.com.pdf</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 05:03 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -4566,6 +4566,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>audits/audit_mountaintimeplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -4626,6 +4636,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>audits/audit_azroofingsystems.com.pdf</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -4681,6 +4701,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>audits/audit_metalroofinglosangeles.net.pdf</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -4741,6 +4771,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>audits/audit_redroofing.org.pdf</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -4801,6 +4841,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>audits/audit_adssheetmetal.com.pdf</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -4854,6 +4904,16 @@
       <c r="L65" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>audits/audit_economywiring.com.pdf</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 05:13 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -4976,6 +4976,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>audits/audit_lyonsroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5036,6 +5046,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>audits/audit_cornerstoneroofingrestoration.com.pdf</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5096,6 +5116,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>audits/audit_preciseplumbingmo.com.pdf</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5156,6 +5186,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>audits/audit_springfieldmoplumber.com.pdf</t>
+        </is>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5216,6 +5256,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>audits/audit_alphahvacelectric.com.pdf</t>
+        </is>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5269,6 +5319,16 @@
       <c r="L71" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>audits/audit_batesroofingllc.net.pdf</t>
+        </is>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 05:23 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -5391,6 +5391,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>audits/audit_longbeachroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -5451,6 +5461,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>audits/audit_chandlerplumberdrain.com.pdf</t>
+        </is>
+      </c>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5511,6 +5531,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>audits/audit_schulteroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5571,6 +5601,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>audits/audit_pipeproslasvegas.com.pdf</t>
+        </is>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -5631,6 +5671,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>audits/audit_loaconstruction.com.pdf</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -5684,6 +5734,16 @@
       <c r="L77" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>audits/audit_superiorhvacct.com.pdf</t>
+        </is>
+      </c>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 05:33 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -5801,6 +5801,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>audits/audit_dtheatingandcooling.com.pdf</t>
+        </is>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -5861,6 +5871,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>audits/audit_ironroofco.com.pdf</t>
+        </is>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5916,6 +5936,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>audits/audit_alltimeairconditioning.com.pdf</t>
+        </is>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5976,6 +6006,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>audits/audit_vanguardcoolingheating.com.pdf</t>
+        </is>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6036,6 +6076,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>audits/audit_gmthomeservices.com.pdf</t>
+        </is>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6094,6 +6144,16 @@
       <c r="L83" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>audits/audit_stormmastersct.com.pdf</t>
+        </is>
+      </c>
+      <c r="N83" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 05:43 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -6216,6 +6216,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>audits/audit_heatinggeek.com.pdf</t>
+        </is>
+      </c>
+      <c r="N84" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6276,6 +6286,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>audits/audit_floridabreezehvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6331,6 +6351,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>audits/audit_cassidyac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N86" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -6391,6 +6421,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>audits/audit_roofingwaterburyct.com.pdf</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6451,6 +6491,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>audits/audit_amproofingllc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6509,6 +6559,16 @@
       <c r="L89" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>audits/audit_westairheating.com.pdf</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 05:53 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -6631,6 +6631,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>audits/audit_trustproofroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -6691,6 +6701,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>audits/audit_ppmplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6751,6 +6771,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>audits/audit_911plumbingandhvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -6811,6 +6841,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>audits/audit_burkhardtheating.com.pdf</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -6871,6 +6911,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>failed: RuntimeError: PDF text never mentions socalplumbingpro.com or 'Plumbing Services in Ontario, CA' - it may be a generic or wrong-company report</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -6929,6 +6974,16 @@
       <c r="L95" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>audits/audit_expresscooling.org.pdf</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 06:03 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -6911,9 +6911,14 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>audits/audit_socalplumbingpro.com.pdf</t>
+        </is>
+      </c>
       <c r="N94" t="inlineStr">
         <is>
-          <t>failed: RuntimeError: PDF text never mentions socalplumbingpro.com or 'Plumbing Services in Ontario, CA' - it may be a generic or wrong-company report</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -7046,6 +7051,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>audits/audit_bluebuiltroofs.com.pdf</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7106,6 +7121,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>audits/audit_ditterinc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7161,6 +7186,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>audits/audit_callcommunityair.com.pdf</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -7221,6 +7256,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>audits/audit_masterroofmtpleasant.com.pdf</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -7279,6 +7324,16 @@
       <c r="L100" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>audits/audit_zimheatingandcooling.com.pdf</t>
+        </is>
+      </c>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 06:13 UTC (cycle 18)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -7391,6 +7391,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>audits/audit_thirdcoast-hvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7451,6 +7461,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M102" t="inlineStr">
+        <is>
+          <t>audits/audit_westernrooter.com.pdf</t>
+        </is>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -7511,6 +7531,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M103" t="inlineStr">
+        <is>
+          <t>audits/audit_hometownroofingsc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -7566,6 +7596,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M104" t="inlineStr">
+        <is>
+          <t>audits/audit_elizabethhvacllc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N104" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -7626,6 +7666,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>audits/audit_getyourairfix.com.pdf</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7684,6 +7734,16 @@
       <c r="L106" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>audits/audit_comfortprosatx.com.pdf</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 06:24 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -7806,6 +7806,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>audits/audit_aaroofingservice.com.pdf</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -7866,6 +7876,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>audits/audit_eliteroofpro.com.pdf</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -7926,6 +7946,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>audits/audit_prohvacroundrock.com.pdf</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -7986,6 +8016,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M110" t="inlineStr">
+        <is>
+          <t>audits/audit_roofingcompaniesphoenix.com.pdf</t>
+        </is>
+      </c>
+      <c r="N110" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -8041,6 +8081,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M111" t="inlineStr">
+        <is>
+          <t>audits/audit_mrcroofinghawaii.com.pdf</t>
+        </is>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -8099,6 +8149,16 @@
       <c r="L112" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M112" t="inlineStr">
+        <is>
+          <t>audits/audit_twincityroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N112" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 06:33 UTC (cycle 20)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -8216,6 +8216,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M113" t="inlineStr">
+        <is>
+          <t>audits/audit_protechroofinghawaii.com.pdf</t>
+        </is>
+      </c>
+      <c r="N113" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -8276,6 +8286,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M114" t="inlineStr">
+        <is>
+          <t>audits/audit_custombiltmetals.com.pdf</t>
+        </is>
+      </c>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -8331,6 +8351,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M115" t="inlineStr">
+        <is>
+          <t>audits/audit_concordnhhvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -8391,6 +8421,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M116" t="inlineStr">
+        <is>
+          <t>audits/audit_pinnacleroofingtn.com.pdf</t>
+        </is>
+      </c>
+      <c r="N116" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -8451,6 +8491,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M117" t="inlineStr">
+        <is>
+          <t>audits/audit_sterlingroofingmt.com.pdf</t>
+        </is>
+      </c>
+      <c r="N117" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -8504,6 +8554,16 @@
       <c r="L118" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>audits/audit_landlcontractors.com.pdf</t>
+        </is>
+      </c>
+      <c r="N118" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 06:43 UTC (cycle 21)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -8626,6 +8626,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M119" t="inlineStr">
+        <is>
+          <t>audits/audit_usaroofingmurfreesboro.com.pdf</t>
+        </is>
+      </c>
+      <c r="N119" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -8686,6 +8696,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>audits/audit_kirknessroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N120" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -8746,6 +8766,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M121" t="inlineStr">
+        <is>
+          <t>audits/audit_bestchoiceroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N121" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -8806,6 +8836,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>audits/audit_totalexteriorsllc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N122" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -8866,6 +8906,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M123" t="inlineStr">
+        <is>
+          <t>audits/audit_shalom2u.com.pdf</t>
+        </is>
+      </c>
+      <c r="N123" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -8924,6 +8974,16 @@
       <c r="L124" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M124" t="inlineStr">
+        <is>
+          <t>audits/audit_hoffmanexteriorsct.com.pdf</t>
+        </is>
+      </c>
+      <c r="N124" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 06:53 UTC (cycle 22)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -9046,6 +9046,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M125" t="inlineStr">
+        <is>
+          <t>audits/audit_dentairconditioning.com.pdf</t>
+        </is>
+      </c>
+      <c r="N125" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -9101,6 +9111,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="N126" t="inlineStr">
+        <is>
+          <t>failed: RuntimeError: PDF text never mentions reedsreasonablehvac.com or 'Reed’s Reasonable Heating and Cooling' - it may be a generic or wrong-company report</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -9161,6 +9176,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M127" t="inlineStr">
+        <is>
+          <t>audits/audit_sunrisehvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N127" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -9216,6 +9241,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M128" t="inlineStr">
+        <is>
+          <t>audits/audit_airpromaster.com.pdf</t>
+        </is>
+      </c>
+      <c r="N128" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -9276,6 +9311,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M129" t="inlineStr">
+        <is>
+          <t>audits/audit_airconditioningchamp.com.pdf</t>
+        </is>
+      </c>
+      <c r="N129" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -9329,6 +9374,16 @@
       <c r="L130" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>audits/audit_constantairbalancing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 07:03 UTC (cycle 23)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -9111,9 +9111,14 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M126" t="inlineStr">
+        <is>
+          <t>audits/audit_reedsreasonablehvac.com.pdf</t>
+        </is>
+      </c>
       <c r="N126" t="inlineStr">
         <is>
-          <t>failed: RuntimeError: PDF text never mentions reedsreasonablehvac.com or 'Reed’s Reasonable Heating and Cooling' - it may be a generic or wrong-company report</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -9446,6 +9451,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>audits/audit_evergreenheatcooling.com.pdf</t>
+        </is>
+      </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -9506,6 +9521,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>audits/audit_primeexteriors.com.pdf</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -9566,6 +9591,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>audits/audit_lambcogc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -9621,6 +9656,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>audits/audit_masterroofcontracting.com.pdf</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -9679,6 +9724,16 @@
       <c r="L135" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>audits/audit_richardsonroofingoh.com.pdf</t>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 07:14 UTC (cycle 24)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -9791,6 +9791,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>audits/audit_advancehaws.com.pdf</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -9851,6 +9861,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>audits/audit_comoexteriors.com.pdf</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -9911,6 +9931,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>audits/audit_mtkmechanical.com.pdf</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -9966,6 +9996,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>audits/audit_jkmechanical.com.pdf</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -10026,6 +10066,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>audits/audit_schroerandsonsmetalroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -10084,6 +10134,16 @@
       <c r="L141" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>audits/audit_brocktonhvacpro.com.pdf</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 07:24 UTC (cycle 25)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -10201,6 +10201,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>audits/audit_mcallisterenergy.com.pdf</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -10261,6 +10271,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>audits/audit_knowlesmechanical.com.pdf</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -10316,6 +10336,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>audits/audit_alltownheatingandac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -10376,6 +10406,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>audits/audit_lumenhvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -10431,6 +10471,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>audits/audit_prestigeaire.com.pdf</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -10489,6 +10539,16 @@
       <c r="L147" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>audits/audit_aghvactn.com.pdf</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 07:34 UTC (cycle 26)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -10611,6 +10611,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>audits/audit_bumbleroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -10671,6 +10681,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>audits/audit_thebestroofguys.com.pdf</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -10731,6 +10751,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>audits/audit_fmfroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -10791,6 +10821,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>audits/audit_bluetrusstx.com.pdf</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -10851,6 +10891,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>audits/audit_woodlandsroofingcontractor.com.pdf</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -10904,6 +10954,16 @@
       <c r="L153" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>audits/audit_probuildhomeservices.com.pdf</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 07:44 UTC (cycle 27)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -11026,6 +11026,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>audits/audit_autryplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -11081,6 +11091,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>audits/audit_championcomfortexperts.com.pdf</t>
+        </is>
+      </c>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -11141,6 +11161,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>audits/audit_blueplanetplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -11201,6 +11231,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>audits/audit_pureairatlanta.com.pdf</t>
+        </is>
+      </c>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -11261,6 +11301,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>audits/audit_schwartzheatingandcooling.com.pdf</t>
+        </is>
+      </c>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -11319,6 +11369,16 @@
       <c r="L159" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>audits/audit_keyheatingandcoolingky.com.pdf</t>
+        </is>
+      </c>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 07:54 UTC (cycle 28)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -11441,6 +11441,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>audits/audit_briskaircool.com.pdf</t>
+        </is>
+      </c>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -11501,6 +11511,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>audits/audit_gonzalesplumbingaz.com.pdf</t>
+        </is>
+      </c>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -11556,6 +11576,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>audits/audit_hvacosta.com.pdf</t>
+        </is>
+      </c>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -11616,6 +11646,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>audits/audit_arizonadraincleaning.com.pdf</t>
+        </is>
+      </c>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -11676,6 +11716,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>audits/audit_redlineroofingtx.com.pdf</t>
+        </is>
+      </c>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -11734,6 +11784,16 @@
       <c r="L165" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>audits/audit_airoserviceusa.com.pdf</t>
+        </is>
+      </c>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 08:04 UTC (cycle 29)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -11851,6 +11851,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>audits/audit_westarkplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N166" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -11911,6 +11921,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>audits/audit_mastonstulsa.com.pdf</t>
+        </is>
+      </c>
+      <c r="N167" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -11966,6 +11986,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>audits/audit_firstcallcarrolltonplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N168" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -12026,6 +12056,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>audits/audit_carrolltonplumbingservice.com.pdf</t>
+        </is>
+      </c>
+      <c r="N169" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -12086,6 +12126,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>audits/audit_918pros.com.pdf</t>
+        </is>
+      </c>
+      <c r="N170" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -12139,6 +12189,16 @@
       <c r="L171" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>audits/audit_alldrainsemergencyplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N171" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 08:14 UTC (cycle 30)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -12256,6 +12256,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M172" t="inlineStr">
+        <is>
+          <t>audits/audit_spotonplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N172" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -12316,6 +12326,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M173" t="inlineStr">
+        <is>
+          <t>audits/audit_gordyroofingtylertx.com.pdf</t>
+        </is>
+      </c>
+      <c r="N173" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -12376,6 +12396,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M174" t="inlineStr">
+        <is>
+          <t>audits/audit_plumbingservicescarrollton.com.pdf</t>
+        </is>
+      </c>
+      <c r="N174" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -12436,6 +12466,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M175" t="inlineStr">
+        <is>
+          <t>audits/audit_austinairconditioning.com.pdf</t>
+        </is>
+      </c>
+      <c r="N175" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -12496,6 +12536,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M176" t="inlineStr">
+        <is>
+          <t>audits/audit_riverroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N176" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -12554,6 +12604,16 @@
       <c r="L177" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr">
+        <is>
+          <t>audits/audit_worldairhvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N177" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 09:04 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -12671,6 +12671,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M178" t="inlineStr">
+        <is>
+          <t>audits/audit_famouscoolair.com.pdf</t>
+        </is>
+      </c>
+      <c r="N178" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -12726,6 +12736,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M179" t="inlineStr">
+        <is>
+          <t>audits/audit_bigskyheatingcooling.com.pdf</t>
+        </is>
+      </c>
+      <c r="N179" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -12786,6 +12806,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M180" t="inlineStr">
+        <is>
+          <t>audits/audit_actheatingandcooling.com.pdf</t>
+        </is>
+      </c>
+      <c r="N180" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -12846,6 +12876,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M181" t="inlineStr">
+        <is>
+          <t>audits/audit_priorityoneheating.com.pdf</t>
+        </is>
+      </c>
+      <c r="N181" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -12901,6 +12941,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M182" t="inlineStr">
+        <is>
+          <t>audits/audit_ehomecomfort.com.pdf</t>
+        </is>
+      </c>
+      <c r="N182" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -12959,6 +13009,16 @@
       <c r="L183" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr">
+        <is>
+          <t>audits/audit_airmaxacrepair.com.pdf</t>
+        </is>
+      </c>
+      <c r="N183" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 09:14 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -13076,6 +13076,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="N184" t="inlineStr">
+        <is>
+          <t>failed: RuntimeError: PDF text never mentions yourmstrplumber.com or 'Evans Plumbing LLC' - it may be a generic or wrong-company report</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -13136,6 +13141,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M185" t="inlineStr">
+        <is>
+          <t>audits/audit_jcohvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N185" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -13191,6 +13206,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M186" t="inlineStr">
+        <is>
+          <t>audits/audit_suttonheat.com.pdf</t>
+        </is>
+      </c>
+      <c r="N186" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -13251,6 +13276,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M187" t="inlineStr">
+        <is>
+          <t>audits/audit_mikebachmanplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N187" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -13311,6 +13346,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M188" t="inlineStr">
+        <is>
+          <t>audits/audit_all-starhvacknoxville.com.pdf</t>
+        </is>
+      </c>
+      <c r="N188" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -13369,6 +13414,16 @@
       <c r="L189" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr">
+        <is>
+          <t>audits/audit_victoryheatandair.com.pdf</t>
+        </is>
+      </c>
+      <c r="N189" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 09:24 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -13481,6 +13481,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M190" t="inlineStr">
+        <is>
+          <t>audits/audit_ozarkmountainair.com.pdf</t>
+        </is>
+      </c>
+      <c r="N190" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -13536,6 +13546,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>audits/audit_renoplumbingdoctor.com.pdf</t>
+        </is>
+      </c>
+      <c r="N191" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -13596,6 +13616,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>audits/audit_justcallheritage.com.pdf</t>
+        </is>
+      </c>
+      <c r="N192" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -13656,6 +13686,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>audits/audit_911exteriors.com.pdf</t>
+        </is>
+      </c>
+      <c r="N193" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -13714,6 +13754,16 @@
       <c r="L194" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>audits/audit_callballthatsall.com.pdf</t>
+        </is>
+      </c>
+      <c r="N194" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 09:34 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -13826,6 +13826,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>audits/audit_johnsonplumbingnv.com.pdf</t>
+        </is>
+      </c>
+      <c r="N195" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -13881,6 +13891,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>audits/audit_jennerandsons.com.pdf</t>
+        </is>
+      </c>
+      <c r="N196" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -13941,6 +13961,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>audits/audit_redemptioncrs.com.pdf</t>
+        </is>
+      </c>
+      <c r="N197" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -14001,6 +14031,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>audits/audit_12stonesroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N198" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -14059,6 +14099,16 @@
       <c r="L199" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>audits/audit_brodyallenexteriors.com.pdf</t>
+        </is>
+      </c>
+      <c r="N199" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 09:44 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -14166,6 +14166,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>audits/audit_innovativecontrolhvacr.com.pdf</t>
+        </is>
+      </c>
+      <c r="N200" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -14226,6 +14236,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>audits/audit_njplumberdirectory.com.pdf</t>
+        </is>
+      </c>
+      <c r="N201" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -14286,6 +14306,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>audits/audit_aurorailhvacservice.com.pdf</t>
+        </is>
+      </c>
+      <c r="N202" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -14346,6 +14376,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>audits/audit_clcroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N203" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -14404,6 +14444,16 @@
       <c r="L204" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>audits/audit_scroofingtx.com.pdf</t>
+        </is>
+      </c>
+      <c r="N204" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 09:54 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -14511,6 +14511,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>audits/audit_mckinneyroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N205" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -14566,6 +14576,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>audits/audit_rightwaynm.com.pdf</t>
+        </is>
+      </c>
+      <c r="N206" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -14626,6 +14646,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>audits/audit_premiumroofingnm.com.pdf</t>
+        </is>
+      </c>
+      <c r="N207" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -14686,6 +14716,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>audits/audit_roofsolutionsandconstruction.com.pdf</t>
+        </is>
+      </c>
+      <c r="N208" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -14744,6 +14784,16 @@
       <c r="L209" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>audits/audit_jrgnm.com.pdf</t>
+        </is>
+      </c>
+      <c r="N209" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 10:04 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -14856,6 +14856,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>audits/audit_teamenoch.com.pdf</t>
+        </is>
+      </c>
+      <c r="N210" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -14916,6 +14926,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>audits/audit_cenvarroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N211" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -14976,6 +14996,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>audits/audit_hbgplumbers.com.pdf</t>
+        </is>
+      </c>
+      <c r="N212" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -15036,6 +15066,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>audits/audit_aboveroofingwv.com.pdf</t>
+        </is>
+      </c>
+      <c r="N213" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -15094,6 +15134,16 @@
       <c r="L214" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>audits/audit_plumbworksinc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N214" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 10:14 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -15201,6 +15201,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>audits/audit_myrtlebeachplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N215" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -15256,6 +15266,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>audits/audit_masterplumbingsc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N216" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -15316,6 +15336,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>audits/audit_beachplumbingsc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N217" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -15366,6 +15396,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>audits/audit_saltlineplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N218" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -15424,6 +15464,16 @@
       <c r="L219" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M219" t="inlineStr">
+        <is>
+          <t>audits/audit_fishersplumbingpros.com.pdf</t>
+        </is>
+      </c>
+      <c r="N219" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 10:24 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -15536,6 +15536,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M220" t="inlineStr">
+        <is>
+          <t>audits/audit_newhausroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N220" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -15596,6 +15606,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M221" t="inlineStr">
+        <is>
+          <t>audits/audit_roofingcontractorriversideca.com.pdf</t>
+        </is>
+      </c>
+      <c r="N221" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -15651,6 +15671,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M222" t="inlineStr">
+        <is>
+          <t>audits/audit_meridiancool.com.pdf</t>
+        </is>
+      </c>
+      <c r="N222" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -15711,6 +15741,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M223" t="inlineStr">
+        <is>
+          <t>audits/audit_westernhvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N223" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -15764,6 +15804,16 @@
       <c r="L224" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M224" t="inlineStr">
+        <is>
+          <t>audits/audit_emergencyplumberfishers.com.pdf</t>
+        </is>
+      </c>
+      <c r="N224" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 10:34 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -15876,6 +15876,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t>audits/audit_veridynehvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N225" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -15936,6 +15946,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t>audits/audit_caliroofingsolutions.com.pdf</t>
+        </is>
+      </c>
+      <c r="N226" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -15996,6 +16016,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t>audits/audit_sunshineheatingandcoolingservices.com.pdf</t>
+        </is>
+      </c>
+      <c r="N227" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -16056,6 +16086,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t>audits/audit_activeplumbinginc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N228" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -16114,6 +16154,16 @@
       <c r="L229" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t>audits/audit_burishbuilderswest.com.pdf</t>
+        </is>
+      </c>
+      <c r="N229" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 10:44 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -16226,6 +16226,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t>audits/audit_callhortonthatswho.com.pdf</t>
+        </is>
+      </c>
+      <c r="N230" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -16286,6 +16296,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t>audits/audit_kingdomplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N231" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -16346,6 +16366,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t>audits/audit_tillmansheatingandair.com.pdf</t>
+        </is>
+      </c>
+      <c r="N232" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -16401,6 +16431,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t>audits/audit_beavertonheatpump.com.pdf</t>
+        </is>
+      </c>
+      <c r="N233" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -16459,6 +16499,16 @@
       <c r="L234" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t>audits/audit_centralairpdx.com.pdf</t>
+        </is>
+      </c>
+      <c r="N234" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 10:54 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -16566,6 +16566,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M235" t="inlineStr">
+        <is>
+          <t>audits/audit_mightyph.com.pdf</t>
+        </is>
+      </c>
+      <c r="N235" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -16621,6 +16631,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M236" t="inlineStr">
+        <is>
+          <t>audits/audit_simplymechanicalco.com.pdf</t>
+        </is>
+      </c>
+      <c r="N236" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -16681,6 +16701,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M237" t="inlineStr">
+        <is>
+          <t>audits/audit_callaviator.com.pdf</t>
+        </is>
+      </c>
+      <c r="N237" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -16741,6 +16771,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M238" t="inlineStr">
+        <is>
+          <t>audits/audit_plumberlakewoodco.com.pdf</t>
+        </is>
+      </c>
+      <c r="N238" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -16799,6 +16839,16 @@
       <c r="L239" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M239" t="inlineStr">
+        <is>
+          <t>audits/audit_vangenderenheating.com.pdf</t>
+        </is>
+      </c>
+      <c r="N239" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 11:04 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -16911,6 +16911,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M240" t="inlineStr">
+        <is>
+          <t>audits/audit_jumphvaccolorado.com.pdf</t>
+        </is>
+      </c>
+      <c r="N240" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -16971,6 +16981,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M241" t="inlineStr">
+        <is>
+          <t>audits/audit_oregonclimatetech.com.pdf</t>
+        </is>
+      </c>
+      <c r="N241" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -17031,6 +17051,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M242" t="inlineStr">
+        <is>
+          <t>audits/audit_stewartsplumbinginc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N242" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -17091,6 +17121,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M243" t="inlineStr">
+        <is>
+          <t>audits/audit_jtechconst.com.pdf</t>
+        </is>
+      </c>
+      <c r="N243" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -17149,6 +17189,16 @@
       <c r="L244" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M244" t="inlineStr">
+        <is>
+          <t>audits/audit_nebraskapetesbuilders.com.pdf</t>
+        </is>
+      </c>
+      <c r="N244" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 11:14 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -17261,6 +17261,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M245" t="inlineStr">
+        <is>
+          <t>audits/audit_rafaroof.com.pdf</t>
+        </is>
+      </c>
+      <c r="N245" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -17321,6 +17331,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M246" t="inlineStr">
+        <is>
+          <t>audits/audit_normanroofingco.com.pdf</t>
+        </is>
+      </c>
+      <c r="N246" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -17381,6 +17401,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M247" t="inlineStr">
+        <is>
+          <t>audits/audit_elmcityroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N247" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -17441,6 +17471,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M248" t="inlineStr">
+        <is>
+          <t>audits/audit_bigleagueroofingllc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N248" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -17499,6 +17539,16 @@
       <c r="L249" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M249" t="inlineStr">
+        <is>
+          <t>audits/audit_normanroofingpro.com.pdf</t>
+        </is>
+      </c>
+      <c r="N249" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 11:24 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -17606,6 +17606,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M250" t="inlineStr">
+        <is>
+          <t>audits/audit_allentownpaacrepair.com.pdf</t>
+        </is>
+      </c>
+      <c r="N250" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -17666,6 +17676,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M251" t="inlineStr">
+        <is>
+          <t>audits/audit_diamondstateplumbing.net.pdf</t>
+        </is>
+      </c>
+      <c r="N251" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -17726,6 +17746,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M252" t="inlineStr">
+        <is>
+          <t>audits/audit_amgplumbingark.com.pdf</t>
+        </is>
+      </c>
+      <c r="N252" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -17781,6 +17811,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M253" t="inlineStr">
+        <is>
+          <t>audits/audit_arpipemaster.com.pdf</t>
+        </is>
+      </c>
+      <c r="N253" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -17839,6 +17879,16 @@
       <c r="L254" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M254" t="inlineStr">
+        <is>
+          <t>audits/audit_peninsularoof.net.pdf</t>
+        </is>
+      </c>
+      <c r="N254" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 11:34 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -17951,6 +17951,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M255" t="inlineStr">
+        <is>
+          <t>audits/audit_westjordanhvacpros.com.pdf</t>
+        </is>
+      </c>
+      <c r="N255" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -18011,6 +18021,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M256" t="inlineStr">
+        <is>
+          <t>audits/audit_bestroofingva.com.pdf</t>
+        </is>
+      </c>
+      <c r="N256" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -18071,6 +18091,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>audits/audit_keystoneheatingandair.com.pdf</t>
+        </is>
+      </c>
+      <c r="N257" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -18131,6 +18161,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>audits/audit_utah-heatingcooling.com.pdf</t>
+        </is>
+      </c>
+      <c r="N258" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -18189,6 +18229,16 @@
       <c r="L259" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>audits/audit_lucasheatingcooling.com.pdf</t>
+        </is>
+      </c>
+      <c r="N259" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 11:44 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -18301,6 +18301,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>audits/audit_larsenhvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N260" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -18361,6 +18371,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>audits/audit_protechroof.net.pdf</t>
+        </is>
+      </c>
+      <c r="N261" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -18421,6 +18441,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>audits/audit_roofassistant.com.pdf</t>
+        </is>
+      </c>
+      <c r="N262" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -18476,6 +18506,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>audits/audit_restorationroofingco.com.pdf</t>
+        </is>
+      </c>
+      <c r="N263" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -18534,6 +18574,16 @@
       <c r="L264" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M264" t="inlineStr">
+        <is>
+          <t>audits/audit_sedonaplumbingandheating.com.pdf</t>
+        </is>
+      </c>
+      <c r="N264" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 11:54 UTC (cycle 18)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -18646,6 +18646,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M265" t="inlineStr">
+        <is>
+          <t>audits/audit_callyellowdog.com.pdf</t>
+        </is>
+      </c>
+      <c r="N265" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -18706,6 +18716,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M266" t="inlineStr">
+        <is>
+          <t>audits/audit_njroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N266" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -18766,6 +18786,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M267" t="inlineStr">
+        <is>
+          <t>audits/audit_sumzeroenergysystems.com.pdf</t>
+        </is>
+      </c>
+      <c r="N267" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -18826,6 +18856,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>audits/audit_trinitytotalhome.com.pdf</t>
+        </is>
+      </c>
+      <c r="N268" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -18884,6 +18924,16 @@
       <c r="L269" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M269" t="inlineStr">
+        <is>
+          <t>audits/audit_knoxvilleroofingandsiding.com.pdf</t>
+        </is>
+      </c>
+      <c r="N269" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 12:04 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -18996,6 +18996,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M270" t="inlineStr">
+        <is>
+          <t>audits/audit_alltimateroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N270" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -19051,6 +19061,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M271" t="inlineStr">
+        <is>
+          <t>audits/audit_hightidecontracting.com.pdf</t>
+        </is>
+      </c>
+      <c r="N271" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -19111,6 +19131,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M272" t="inlineStr">
+        <is>
+          <t>audits/audit_onehourcomfort.com.pdf</t>
+        </is>
+      </c>
+      <c r="N272" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -19171,6 +19201,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M273" t="inlineStr">
+        <is>
+          <t>audits/audit_barnettroofingknoxville.com.pdf</t>
+        </is>
+      </c>
+      <c r="N273" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -19229,6 +19269,16 @@
       <c r="L274" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M274" t="inlineStr">
+        <is>
+          <t>audits/audit_bentonroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N274" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 12:14 UTC (cycle 20)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -13076,9 +13076,14 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M184" t="inlineStr">
+        <is>
+          <t>audits/audit_yourmstrplumber.com.pdf</t>
+        </is>
+      </c>
       <c r="N184" t="inlineStr">
         <is>
-          <t>failed: RuntimeError: PDF text never mentions yourmstrplumber.com or 'Evans Plumbing LLC' - it may be a generic or wrong-company report</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -19336,6 +19341,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M275" t="inlineStr">
+        <is>
+          <t>audits/audit_lancasterroofingcompany.com.pdf</t>
+        </is>
+      </c>
+      <c r="N275" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -19391,6 +19406,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M276" t="inlineStr">
+        <is>
+          <t>audits/audit_middlecreekroof.com.pdf</t>
+        </is>
+      </c>
+      <c r="N276" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -19451,6 +19476,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M277" t="inlineStr">
+        <is>
+          <t>audits/audit_capeharthc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N277" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -19511,6 +19546,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="N278" t="inlineStr">
+        <is>
+          <t>failed: RuntimeError: PDF text never mentions prothermalhvac.com or 'ProThermal Heating and Cooling' - it may be a generic or wrong-company report</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -19564,6 +19604,16 @@
       <c r="L279" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M279" t="inlineStr">
+        <is>
+          <t>audits/audit_waterworkplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N279" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 12:24 UTC (cycle 21)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -19546,9 +19546,14 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M278" t="inlineStr">
+        <is>
+          <t>audits/audit_prothermalhvac.com.pdf</t>
+        </is>
+      </c>
       <c r="N278" t="inlineStr">
         <is>
-          <t>failed: RuntimeError: PDF text never mentions prothermalhvac.com or 'ProThermal Heating and Cooling' - it may be a generic or wrong-company report</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -19676,6 +19681,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M280" t="inlineStr">
+        <is>
+          <t>audits/audit_areaplumbingandsewer.com.pdf</t>
+        </is>
+      </c>
+      <c r="N280" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -19736,6 +19751,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>audits/audit_rvheat.com.pdf</t>
+        </is>
+      </c>
+      <c r="N281" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -19796,6 +19821,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M282" t="inlineStr">
+        <is>
+          <t>audits/audit_541hvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N282" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -19851,6 +19886,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M283" t="inlineStr">
+        <is>
+          <t>audits/audit_myadvancedair.com.pdf</t>
+        </is>
+      </c>
+      <c r="N283" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -19909,6 +19954,16 @@
       <c r="L284" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M284" t="inlineStr">
+        <is>
+          <t>audits/audit_mountainwestac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N284" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 12:34 UTC (cycle 22)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -20026,6 +20026,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M285" t="inlineStr">
+        <is>
+          <t>audits/audit_hawthornephc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N285" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -20086,6 +20096,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M286" t="inlineStr">
+        <is>
+          <t>audits/audit_foxfamilyhvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N286" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -20146,6 +20166,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M287" t="inlineStr">
+        <is>
+          <t>audits/audit_tier1roofingsolutions.com.pdf</t>
+        </is>
+      </c>
+      <c r="N287" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -20201,6 +20231,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>audits/audit_bishopshvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N288" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -20256,6 +20296,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>audits/audit_airworkssolutions.com.pdf</t>
+        </is>
+      </c>
+      <c r="N289" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -20314,6 +20364,16 @@
       <c r="L290" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>audits/audit_hvacpulse.com.pdf</t>
+        </is>
+      </c>
+      <c r="N290" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 12:44 UTC (cycle 23)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -20436,6 +20436,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M291" t="inlineStr">
+        <is>
+          <t>audits/audit_rivercityheatingcooling.com.pdf</t>
+        </is>
+      </c>
+      <c r="N291" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -20496,6 +20506,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M292" t="inlineStr">
+        <is>
+          <t>audits/audit_max-roofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N292" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -20556,6 +20576,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M293" t="inlineStr">
+        <is>
+          <t>audits/audit_falconroofs.com.pdf</t>
+        </is>
+      </c>
+      <c r="N293" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -20611,6 +20641,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M294" t="inlineStr">
+        <is>
+          <t>audits/audit_davidsqualitycontracting.com.pdf</t>
+        </is>
+      </c>
+      <c r="N294" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -20671,6 +20711,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M295" t="inlineStr">
+        <is>
+          <t>audits/audit_nextdoor.build.pdf</t>
+        </is>
+      </c>
+      <c r="N295" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -20729,6 +20779,16 @@
       <c r="L296" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M296" t="inlineStr">
+        <is>
+          <t>audits/audit_airtechofkaty.com.pdf</t>
+        </is>
+      </c>
+      <c r="N296" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 12:54 UTC (cycle 24)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -20851,6 +20851,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M297" t="inlineStr">
+        <is>
+          <t>audits/audit_afterhoursplumbingllc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N297" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -20906,6 +20916,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M298" t="inlineStr">
+        <is>
+          <t>audits/audit_plumberproservice.com.pdf</t>
+        </is>
+      </c>
+      <c r="N298" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -20966,6 +20986,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M299" t="inlineStr">
+        <is>
+          <t>audits/audit_mackeyservicestx.com.pdf</t>
+        </is>
+      </c>
+      <c r="N299" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -21026,6 +21056,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M300" t="inlineStr">
+        <is>
+          <t>audits/audit_24sevenac.net.pdf</t>
+        </is>
+      </c>
+      <c r="N300" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -21086,6 +21126,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M301" t="inlineStr">
+        <is>
+          <t>audits/audit_summers-plumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N301" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -21144,6 +21194,16 @@
       <c r="L302" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M302" t="inlineStr">
+        <is>
+          <t>audits/audit_amarillosfinestplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N302" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 13:05 UTC (cycle 25)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -21267,6 +21267,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M303" t="inlineStr">
+        <is>
+          <t>audits/audit_katyair.com.pdf</t>
+        </is>
+      </c>
+      <c r="N303" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -21322,6 +21332,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M304" t="inlineStr">
+        <is>
+          <t>audits/audit_clogbustersllc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N304" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -21377,6 +21397,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M305" t="inlineStr">
+        <is>
+          <t>audits/audit_thorpeac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N305" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -21437,6 +21467,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M306" t="inlineStr">
+        <is>
+          <t>audits/audit_smartheatingandairconditioning.com.pdf</t>
+        </is>
+      </c>
+      <c r="N306" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -21497,6 +21537,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M307" t="inlineStr">
+        <is>
+          <t>audits/audit_heat-pump-installation-appleton.janesvilleairductcleaning.com.pdf</t>
+        </is>
+      </c>
+      <c r="N307" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
@@ -21555,6 +21605,16 @@
       <c r="L308" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M308" t="inlineStr">
+        <is>
+          <t>audits/audit_harryclarkac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N308" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 13:14 UTC (cycle 26)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -21677,6 +21677,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M309" t="inlineStr">
+        <is>
+          <t>audits/audit_suncoastplumbingsc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N309" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
@@ -21737,6 +21747,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M310" t="inlineStr">
+        <is>
+          <t>audits/audit_escondidoqualityroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N310" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
@@ -21797,6 +21817,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M311" t="inlineStr">
+        <is>
+          <t>audits/audit_rooferconroe.com.pdf</t>
+        </is>
+      </c>
+      <c r="N311" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
@@ -21852,6 +21882,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M312" t="inlineStr">
+        <is>
+          <t>audits/audit_christianroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N312" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -21912,6 +21952,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M313" t="inlineStr">
+        <is>
+          <t>audits/audit_myroofimprovement.com.pdf</t>
+        </is>
+      </c>
+      <c r="N313" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
@@ -21970,6 +22020,16 @@
       <c r="L314" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M314" t="inlineStr">
+        <is>
+          <t>audits/audit_escondidoroofingpros.com.pdf</t>
+        </is>
+      </c>
+      <c r="N314" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 13:24 UTC (cycle 27)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -22092,6 +22092,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M315" t="inlineStr">
+        <is>
+          <t>audits/audit_conroeroofpro.com.pdf</t>
+        </is>
+      </c>
+      <c r="N315" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
@@ -22152,6 +22162,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M316" t="inlineStr">
+        <is>
+          <t>audits/audit_rapid-city.wegnerroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N316" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -22212,6 +22232,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M317" t="inlineStr">
+        <is>
+          <t>audits/audit_californiaplumbingsd.com.pdf</t>
+        </is>
+      </c>
+      <c r="N317" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -22272,6 +22302,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M318" t="inlineStr">
+        <is>
+          <t>audits/audit_coreplumbingsd.com.pdf</t>
+        </is>
+      </c>
+      <c r="N318" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -22332,6 +22372,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M319" t="inlineStr">
+        <is>
+          <t>audits/audit_sandiegoemergencyplumber.org.pdf</t>
+        </is>
+      </c>
+      <c r="N319" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -22390,6 +22440,16 @@
       <c r="L320" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M320" t="inlineStr">
+        <is>
+          <t>audits/audit_repipehero.com.pdf</t>
+        </is>
+      </c>
+      <c r="N320" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 13:34 UTC (cycle 28)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -22512,6 +22512,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M321" t="inlineStr">
+        <is>
+          <t>audits/audit_duracraftroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N321" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -22567,6 +22577,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M322" t="inlineStr">
+        <is>
+          <t>audits/audit_waglersteel.com.pdf</t>
+        </is>
+      </c>
+      <c r="N322" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -22627,6 +22647,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M323" t="inlineStr">
+        <is>
+          <t>audits/audit_ridgevalleyexteriors.com.pdf</t>
+        </is>
+      </c>
+      <c r="N323" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -22687,6 +22717,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M324" t="inlineStr">
+        <is>
+          <t>audits/audit_raleighncmetalroofing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N324" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -22742,6 +22782,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M325" t="inlineStr">
+        <is>
+          <t>audits/audit_bigbearrfg.com.pdf</t>
+        </is>
+      </c>
+      <c r="N325" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -22795,6 +22845,16 @@
       <c r="L326" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M326" t="inlineStr">
+        <is>
+          <t>audits/audit_thermochillmech.com.pdf</t>
+        </is>
+      </c>
+      <c r="N326" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 13:44 UTC (cycle 29)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -22912,6 +22912,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M327" t="inlineStr">
+        <is>
+          <t>audits/audit_jerrykelly.com.pdf</t>
+        </is>
+      </c>
+      <c r="N327" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -22972,6 +22982,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M328" t="inlineStr">
+        <is>
+          <t>audits/audit_staycool-hvac.com.pdf</t>
+        </is>
+      </c>
+      <c r="N328" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
@@ -23027,6 +23047,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M329" t="inlineStr">
+        <is>
+          <t>audits/audit_southshorecomfort.com.pdf</t>
+        </is>
+      </c>
+      <c r="N329" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -23087,6 +23117,11 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="N330" t="inlineStr">
+        <is>
+          <t>failed: RuntimeError: PDF text never mentions wentzvilleair.com or 'Wentzville Air &amp; Refrigeration' - it may be a generic or wrong-company report</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -23142,6 +23177,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M331" t="inlineStr">
+        <is>
+          <t>audits/audit_firstcallheating.com.pdf</t>
+        </is>
+      </c>
+      <c r="N331" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -23195,6 +23240,16 @@
       <c r="L332" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M332" t="inlineStr">
+        <is>
+          <t>audits/audit_callrkhc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N332" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 13:54 UTC (cycle 30)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -23307,6 +23307,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M333" t="inlineStr">
+        <is>
+          <t>audits/audit_foremanheating.com.pdf</t>
+        </is>
+      </c>
+      <c r="N333" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -23367,6 +23377,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M334" t="inlineStr">
+        <is>
+          <t>audits/audit_brasstacksplumbing.com.pdf</t>
+        </is>
+      </c>
+      <c r="N334" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -23427,6 +23447,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M335" t="inlineStr">
+        <is>
+          <t>audits/audit_andersonacservice.com.pdf</t>
+        </is>
+      </c>
+      <c r="N335" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -23482,6 +23512,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M336" t="inlineStr">
+        <is>
+          <t>audits/audit_beaconbiloxi.com.pdf</t>
+        </is>
+      </c>
+      <c r="N336" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
@@ -23535,6 +23575,16 @@
       <c r="L337" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M337" t="inlineStr">
+        <is>
+          <t>audits/audit_westmechanical.net.pdf</t>
+        </is>
+      </c>
+      <c r="N337" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Audit + outreach: 2026-09-07 17:29 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -23642,6 +23642,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M338" t="inlineStr">
+        <is>
+          <t>audits/audit_azmonsterair.com.pdf</t>
+        </is>
+      </c>
+      <c r="N338" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -23702,6 +23712,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M339" t="inlineStr">
+        <is>
+          <t>audits/audit_fasttrackheatingandcooling.com.pdf</t>
+        </is>
+      </c>
+      <c r="N339" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
@@ -23762,6 +23782,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M340" t="inlineStr">
+        <is>
+          <t>audits/audit_thomsenroofinginc.com.pdf</t>
+        </is>
+      </c>
+      <c r="N340" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
@@ -23817,6 +23847,16 @@
           <t>2026-09-06</t>
         </is>
       </c>
+      <c r="M341" t="inlineStr">
+        <is>
+          <t>audits/audit_boulderroof.com.pdf</t>
+        </is>
+      </c>
+      <c r="N341" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
@@ -23875,6 +23915,16 @@
       <c r="L342" t="inlineStr">
         <is>
           <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="M342" t="inlineStr">
+        <is>
+          <t>audits/audit_meteorhomeremodeling.com.pdf</t>
+        </is>
+      </c>
+      <c r="N342" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Leads: 2026-09-07 17:36 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_master.xlsx
+++ b/output/leads_master.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1493"/>
+  <dimension ref="A1:P1501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -91308,6 +91308,482 @@
         </is>
       </c>
     </row>
+    <row r="1494">
+      <c r="A1494" t="inlineStr">
+        <is>
+          <t>Water Heater Repair in Bellingham WA | Lavergne's Plumbing</t>
+        </is>
+      </c>
+      <c r="B1494" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1494" t="inlineStr">
+        <is>
+          <t>lavergneplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1494" t="inlineStr">
+        <is>
+          <t>https://www.lavergneplumbing.com/water-heater-repair/</t>
+        </is>
+      </c>
+      <c r="E1494" t="inlineStr"/>
+      <c r="F1494" t="inlineStr">
+        <is>
+          <t>info@lavergneplumbing.com</t>
+        </is>
+      </c>
+      <c r="G1494" t="inlineStr">
+        <is>
+          <t>360-685-8098</t>
+        </is>
+      </c>
+      <c r="H1494" t="inlineStr">
+        <is>
+          <t>Bellingham WA</t>
+        </is>
+      </c>
+      <c r="I1494" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1494" t="inlineStr">
+        <is>
+          <t>water heater repair Bellingham WA</t>
+        </is>
+      </c>
+      <c r="K1494" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1494" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="1495">
+      <c r="A1495" t="inlineStr">
+        <is>
+          <t>North County Premier Roofing -</t>
+        </is>
+      </c>
+      <c r="B1495" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1495" t="inlineStr">
+        <is>
+          <t>premierroofinc.com</t>
+        </is>
+      </c>
+      <c r="D1495" t="inlineStr">
+        <is>
+          <t>https://premierroofinc.com/roofing-company-chula-vista-ca/</t>
+        </is>
+      </c>
+      <c r="E1495" t="inlineStr">
+        <is>
+          <t>Jonathan Ortega</t>
+        </is>
+      </c>
+      <c r="F1495" t="inlineStr">
+        <is>
+          <t>jonathan@premierroofinc.com</t>
+        </is>
+      </c>
+      <c r="G1495" t="inlineStr">
+        <is>
+          <t>(760) 899-5525</t>
+        </is>
+      </c>
+      <c r="H1495" t="inlineStr">
+        <is>
+          <t>Chula Vista CA</t>
+        </is>
+      </c>
+      <c r="I1495" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1495" t="inlineStr">
+        <is>
+          <t>roof repair company Chula Vista CA</t>
+        </is>
+      </c>
+      <c r="K1495" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1495" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="1496">
+      <c r="A1496" t="inlineStr">
+        <is>
+          <t>Schomer's Plumbing, Heating and AC</t>
+        </is>
+      </c>
+      <c r="B1496" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1496" t="inlineStr">
+        <is>
+          <t>schomersplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1496" t="inlineStr">
+        <is>
+          <t>https://www.schomersplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E1496" t="inlineStr">
+        <is>
+          <t>Brett Miller</t>
+        </is>
+      </c>
+      <c r="F1496" t="inlineStr">
+        <is>
+          <t>alex@findeight.com</t>
+        </is>
+      </c>
+      <c r="G1496" t="inlineStr">
+        <is>
+          <t>(765) 447-4014</t>
+        </is>
+      </c>
+      <c r="H1496" t="inlineStr">
+        <is>
+          <t>Lafayette IN</t>
+        </is>
+      </c>
+      <c r="I1496" t="n">
+        <v>100</v>
+      </c>
+      <c r="J1496" t="inlineStr">
+        <is>
+          <t>plumbing company Lafayette IN</t>
+        </is>
+      </c>
+      <c r="K1496" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1496" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="1497">
+      <c r="A1497" t="inlineStr">
+        <is>
+          <t>619 Roofing</t>
+        </is>
+      </c>
+      <c r="B1497" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1497" t="inlineStr">
+        <is>
+          <t>619roofing.com</t>
+        </is>
+      </c>
+      <c r="D1497" t="inlineStr">
+        <is>
+          <t>https://619roofing.com/san-diego-ca/repair-contractors/chula-vista/</t>
+        </is>
+      </c>
+      <c r="E1497" t="inlineStr">
+        <is>
+          <t>Orange County</t>
+        </is>
+      </c>
+      <c r="F1497" t="inlineStr">
+        <is>
+          <t>info@619roofing.com</t>
+        </is>
+      </c>
+      <c r="G1497" t="inlineStr">
+        <is>
+          <t>(619) 609-0214</t>
+        </is>
+      </c>
+      <c r="H1497" t="inlineStr">
+        <is>
+          <t>Chula Vista CA</t>
+        </is>
+      </c>
+      <c r="I1497" t="n">
+        <v>98</v>
+      </c>
+      <c r="J1497" t="inlineStr">
+        <is>
+          <t>roof repair company Chula Vista CA</t>
+        </is>
+      </c>
+      <c r="K1497" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1497" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="1498">
+      <c r="A1498" t="inlineStr">
+        <is>
+          <t>Roof Repair | Tuscaloosa, AL</t>
+        </is>
+      </c>
+      <c r="B1498" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C1498" t="inlineStr">
+        <is>
+          <t>crimsonroofingllctuscaloosa.com</t>
+        </is>
+      </c>
+      <c r="D1498" t="inlineStr">
+        <is>
+          <t>https://www.crimsonroofingllctuscaloosa.com/roof-repair</t>
+        </is>
+      </c>
+      <c r="E1498" t="inlineStr">
+        <is>
+          <t>Free Roof</t>
+        </is>
+      </c>
+      <c r="F1498" t="inlineStr">
+        <is>
+          <t>kamryn.crimsonr@gmail.com</t>
+        </is>
+      </c>
+      <c r="G1498" t="inlineStr">
+        <is>
+          <t>334-303-6875</t>
+        </is>
+      </c>
+      <c r="H1498" t="inlineStr">
+        <is>
+          <t>Tuscaloosa AL</t>
+        </is>
+      </c>
+      <c r="I1498" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1498" t="inlineStr">
+        <is>
+          <t>roof repair company Tuscaloosa AL</t>
+        </is>
+      </c>
+      <c r="K1498" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1498" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="1499">
+      <c r="A1499" t="inlineStr">
+        <is>
+          <t>CPI Plumbing &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B1499" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C1499" t="inlineStr">
+        <is>
+          <t>cpiplumbing.com</t>
+        </is>
+      </c>
+      <c r="D1499" t="inlineStr">
+        <is>
+          <t>https://www.cpiplumbing.com/bellingham/water-heaters/</t>
+        </is>
+      </c>
+      <c r="E1499" t="inlineStr">
+        <is>
+          <t>Serving Washington</t>
+        </is>
+      </c>
+      <c r="F1499" t="inlineStr">
+        <is>
+          <t>customerservice@cpiplumbing.com</t>
+        </is>
+      </c>
+      <c r="G1499" t="inlineStr">
+        <is>
+          <t>360-822-9306</t>
+        </is>
+      </c>
+      <c r="H1499" t="inlineStr">
+        <is>
+          <t>Bellingham WA</t>
+        </is>
+      </c>
+      <c r="I1499" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1499" t="inlineStr">
+        <is>
+          <t>water heater repair Bellingham WA</t>
+        </is>
+      </c>
+      <c r="K1499" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1499" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="1500">
+      <c r="A1500" t="inlineStr">
+        <is>
+          <t>24h Plumbing Pros</t>
+        </is>
+      </c>
+      <c r="B1500" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1500" t="inlineStr">
+        <is>
+          <t>24hplumbingpros.com</t>
+        </is>
+      </c>
+      <c r="D1500" t="inlineStr">
+        <is>
+          <t>https://www.24hplumbingpros.com/locations/emergency-plumber-champaign/</t>
+        </is>
+      </c>
+      <c r="E1500" t="inlineStr">
+        <is>
+          <t>Plumbing Pros</t>
+        </is>
+      </c>
+      <c r="F1500" t="inlineStr">
+        <is>
+          <t>hello@24hplumbingpros.com</t>
+        </is>
+      </c>
+      <c r="G1500" t="inlineStr">
+        <is>
+          <t>877-959-6069</t>
+        </is>
+      </c>
+      <c r="H1500" t="inlineStr">
+        <is>
+          <t>Champaign IL</t>
+        </is>
+      </c>
+      <c r="I1500" t="n">
+        <v>90</v>
+      </c>
+      <c r="J1500" t="inlineStr">
+        <is>
+          <t>emergency plumber Champaign IL</t>
+        </is>
+      </c>
+      <c r="K1500" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1500" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="1501">
+      <c r="A1501" t="inlineStr">
+        <is>
+          <t>Water Heater Repair &amp; Installation in Bellingham, WA: Hot Water When You Need It</t>
+        </is>
+      </c>
+      <c r="B1501" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C1501" t="inlineStr">
+        <is>
+          <t>fantastic-plumbing.com</t>
+        </is>
+      </c>
+      <c r="D1501" t="inlineStr">
+        <is>
+          <t>https://fantastic-plumbing.com/water-heater-repair-installation-bellingham-wa/</t>
+        </is>
+      </c>
+      <c r="E1501" t="inlineStr">
+        <is>
+          <t>Upgrades Many</t>
+        </is>
+      </c>
+      <c r="F1501" t="inlineStr">
+        <is>
+          <t>info@fantastic-plumbing.com</t>
+        </is>
+      </c>
+      <c r="G1501" t="inlineStr">
+        <is>
+          <t>(888) 918-9104</t>
+        </is>
+      </c>
+      <c r="H1501" t="inlineStr">
+        <is>
+          <t>Bellingham WA</t>
+        </is>
+      </c>
+      <c r="I1501" t="n">
+        <v>80</v>
+      </c>
+      <c r="J1501" t="inlineStr">
+        <is>
+          <t>water heater repair Bellingham WA</t>
+        </is>
+      </c>
+      <c r="K1501" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L1501" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>